<commit_message>
Added html report for each brand scores
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="AB3" s="7" t="n">
-        <v>168</v>
+        <v>27</v>
       </c>
       <c r="AC3" s="7" t="inlineStr">
         <is>
@@ -1461,7 +1461,7 @@
       </c>
       <c r="AD3" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="AB4" s="4" t="n">
-        <v>51</v>
+        <v>168</v>
       </c>
       <c r="AC4" s="4" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="AD4" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="AB5" s="7" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="AC5" s="7" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="AD5" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="AB6" s="4" t="n">
-        <v>157</v>
+        <v>47</v>
       </c>
       <c r="AC6" s="4" t="inlineStr">
         <is>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="AD6" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="AB7" s="7" t="n">
-        <v>2</v>
+        <v>157</v>
       </c>
       <c r="AC7" s="7" t="inlineStr">
         <is>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="AD7" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
       <c r="AB8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC8" s="4" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="AD8" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="AB9" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC9" s="7" t="inlineStr">
         <is>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="AD9" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -2037,16 +2037,16 @@
         </is>
       </c>
       <c r="AB10" s="4" t="n">
-        <v>428</v>
+        <v>1</v>
       </c>
       <c r="AC10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="AD10" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="AB11" s="7" t="n">
-        <v>166</v>
+        <v>428</v>
       </c>
       <c r="AC11" s="7" t="inlineStr">
         <is>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="AD11" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="AB12" s="4" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="AC12" s="4" t="inlineStr">
         <is>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="AD12" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="AB13" s="7" t="n">
-        <v>35</v>
+        <v>166</v>
       </c>
       <c r="AC13" s="7" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="AD13" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="AB14" s="4" t="n">
-        <v>144</v>
+        <v>54</v>
       </c>
       <c r="AC14" s="4" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="AD14" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="AB15" s="7" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="AC15" s="7" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="AD15" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
         </is>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>4</v>
+        <v>144</v>
       </c>
       <c r="AC16" s="4" t="inlineStr">
         <is>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="AD16" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="AB17" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AC17" s="7" t="inlineStr">
         <is>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="AD17" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -2669,16 +2669,16 @@
         </is>
       </c>
       <c r="AB18" s="4" t="n">
-        <v>478</v>
+        <v>4</v>
       </c>
       <c r="AC18" s="4" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="AD18" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -2748,16 +2748,16 @@
         </is>
       </c>
       <c r="AB19" s="7" t="n">
-        <v>183</v>
+        <v>6</v>
       </c>
       <c r="AC19" s="7" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="AD19" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="AB20" s="4" t="n">
-        <v>51</v>
+        <v>478</v>
       </c>
       <c r="AC20" s="4" t="inlineStr">
         <is>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="AD20" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="AB21" s="7" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="AC21" s="7" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="AD21" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="AB22" s="4" t="n">
-        <v>1</v>
+        <v>183</v>
       </c>
       <c r="AC22" s="4" t="inlineStr">
         <is>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="AD22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="AB23" s="7" t="n">
-        <v>144</v>
+        <v>51</v>
       </c>
       <c r="AC23" s="7" t="inlineStr">
         <is>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="AD23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="AB24" s="4" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="AC24" s="4" t="inlineStr">
         <is>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="AD24" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="AB25" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC25" s="7" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="AD25" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="AB26" s="4" t="n">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="AC26" s="4" t="inlineStr">
         <is>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="AD26" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -3220,16 +3220,16 @@
         </is>
       </c>
       <c r="AB27" s="7" t="n">
-        <v>515</v>
+        <v>3</v>
       </c>
       <c r="AC27" s="7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="AD27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -3279,16 +3279,16 @@
         </is>
       </c>
       <c r="AB28" s="4" t="n">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="AC28" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="AD28" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -3338,16 +3338,16 @@
         </is>
       </c>
       <c r="AB29" s="7" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="AC29" s="7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="AD29" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="AB30" s="4" t="n">
-        <v>42</v>
+        <v>515</v>
       </c>
       <c r="AC30" s="4" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="AD30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
         </is>
       </c>
       <c r="AB31" s="7" t="n">
-        <v>123</v>
+        <v>28</v>
       </c>
       <c r="AC31" s="7" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="AD31" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="AB32" s="4" t="n">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="AC32" s="4" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="AD32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3597,7 @@
         </is>
       </c>
       <c r="AB33" s="7" t="n">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="AC33" s="7" t="inlineStr">
         <is>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="AD33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -3638,16 +3638,16 @@
         </is>
       </c>
       <c r="AB34" s="4" t="n">
-        <v>453</v>
+        <v>42</v>
       </c>
       <c r="AC34" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="AD34" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -3679,16 +3679,16 @@
         </is>
       </c>
       <c r="AB35" s="7" t="n">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="AC35" s="7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="AD35" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -3720,16 +3720,16 @@
         </is>
       </c>
       <c r="AB36" s="4" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="AC36" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="AD36" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -3761,16 +3761,16 @@
         </is>
       </c>
       <c r="AB37" s="7" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="AC37" s="7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="AD37" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="AB38" s="4" t="n">
-        <v>147</v>
+        <v>453</v>
       </c>
       <c r="AC38" s="4" t="inlineStr">
         <is>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="AD38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="AB39" s="7" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AC39" s="7" t="inlineStr">
         <is>
@@ -3852,7 +3852,7 @@
       </c>
       <c r="AD39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="AB40" s="4" t="n">
-        <v>5</v>
+        <v>136</v>
       </c>
       <c r="AC40" s="4" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="AD40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -3925,7 +3925,7 @@
         </is>
       </c>
       <c r="AB41" s="7" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="AC41" s="7" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="AD41" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -3966,16 +3966,16 @@
         </is>
       </c>
       <c r="AB42" s="4" t="n">
-        <v>518</v>
+        <v>45</v>
       </c>
       <c r="AC42" s="4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="AD42" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -4007,16 +4007,16 @@
         </is>
       </c>
       <c r="AB43" s="7" t="n">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="AC43" s="7" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="AD43" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -4048,16 +4048,16 @@
         </is>
       </c>
       <c r="AB44" s="4" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="AC44" s="4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="AD44" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -4089,16 +4089,16 @@
         </is>
       </c>
       <c r="AB45" s="7" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="AC45" s="7" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="AD45" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -4130,16 +4130,16 @@
         </is>
       </c>
       <c r="AB46" s="4" t="n">
-        <v>127</v>
+        <v>2</v>
       </c>
       <c r="AC46" s="4" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="AD46" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="AB47" s="7" t="n">
-        <v>1</v>
+        <v>518</v>
       </c>
       <c r="AC47" s="7" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="AD47" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="AB48" s="4" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="AC48" s="4" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="AD48" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
         </is>
       </c>
       <c r="AB49" s="7" t="n">
-        <v>1</v>
+        <v>126</v>
       </c>
       <c r="AC49" s="7" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
       </c>
       <c r="AD49" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -4294,16 +4294,16 @@
         </is>
       </c>
       <c r="AB50" s="4" t="n">
-        <v>474</v>
+        <v>57</v>
       </c>
       <c r="AC50" s="4" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD50" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -4335,16 +4335,16 @@
         </is>
       </c>
       <c r="AB51" s="7" t="n">
-        <v>138</v>
+        <v>47</v>
       </c>
       <c r="AC51" s="7" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -4376,16 +4376,16 @@
         </is>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>53</v>
+        <v>127</v>
       </c>
       <c r="AC52" s="4" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -4417,16 +4417,16 @@
         </is>
       </c>
       <c r="AB53" s="7" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="AC53" s="7" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -4458,16 +4458,16 @@
         </is>
       </c>
       <c r="AB54" s="4" t="n">
-        <v>129</v>
+        <v>4</v>
       </c>
       <c r="AC54" s="4" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD54" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -4499,16 +4499,16 @@
         </is>
       </c>
       <c r="AB55" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC55" s="7" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="AD55" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="AB56" s="4" t="n">
-        <v>1</v>
+        <v>474</v>
       </c>
       <c r="AC56" s="4" t="inlineStr">
         <is>
@@ -4549,7 +4549,7 @@
       </c>
       <c r="AD56" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
         </is>
       </c>
       <c r="AB57" s="7" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AC57" s="7" t="inlineStr">
         <is>
@@ -4590,7 +4590,7 @@
       </c>
       <c r="AD57" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -4622,16 +4622,16 @@
         </is>
       </c>
       <c r="AB58" s="4" t="n">
-        <v>430</v>
+        <v>138</v>
       </c>
       <c r="AC58" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD58" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -4663,16 +4663,16 @@
         </is>
       </c>
       <c r="AB59" s="7" t="n">
-        <v>163</v>
+        <v>53</v>
       </c>
       <c r="AC59" s="7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD59" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -4704,16 +4704,16 @@
         </is>
       </c>
       <c r="AB60" s="4" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="AC60" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD60" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -4745,16 +4745,16 @@
         </is>
       </c>
       <c r="AB61" s="7" t="n">
-        <v>59</v>
+        <v>129</v>
       </c>
       <c r="AC61" s="7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -4786,16 +4786,16 @@
         </is>
       </c>
       <c r="AB62" s="4" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="AC62" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -4827,16 +4827,16 @@
         </is>
       </c>
       <c r="AB63" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC63" s="7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -4868,16 +4868,16 @@
         </is>
       </c>
       <c r="AB64" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC64" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="AD64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
         </is>
       </c>
       <c r="AB65" s="7" t="n">
-        <v>2</v>
+        <v>430</v>
       </c>
       <c r="AC65" s="7" t="inlineStr">
         <is>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="AD65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -4950,16 +4950,16 @@
         </is>
       </c>
       <c r="AB66" s="4" t="n">
-        <v>478</v>
+        <v>27</v>
       </c>
       <c r="AC66" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD66" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -4991,11 +4991,11 @@
         </is>
       </c>
       <c r="AB67" s="7" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="AC67" s="7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD67" s="7" t="inlineStr">
@@ -5032,11 +5032,11 @@
         </is>
       </c>
       <c r="AB68" s="4" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="AC68" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD68" s="4" t="inlineStr">
@@ -5073,11 +5073,11 @@
         </is>
       </c>
       <c r="AB69" s="7" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="AC69" s="7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD69" s="7" t="inlineStr">
@@ -5114,11 +5114,11 @@
         </is>
       </c>
       <c r="AB70" s="4" t="n">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="AC70" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD70" s="4" t="inlineStr">
@@ -5155,11 +5155,11 @@
         </is>
       </c>
       <c r="AB71" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC71" s="7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD71" s="7" t="inlineStr">
@@ -5196,11 +5196,11 @@
         </is>
       </c>
       <c r="AB72" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AC72" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD72" s="4" t="inlineStr">
@@ -5237,11 +5237,11 @@
         </is>
       </c>
       <c r="AB73" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC73" s="7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="AD73" s="7" t="inlineStr">
@@ -5278,11 +5278,11 @@
         </is>
       </c>
       <c r="AB74" s="4" t="n">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="AC74" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD74" s="4" t="inlineStr">
@@ -5319,16 +5319,16 @@
         </is>
       </c>
       <c r="AB75" s="7" t="n">
-        <v>150</v>
+        <v>23</v>
       </c>
       <c r="AC75" s="7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD75" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -5360,16 +5360,16 @@
         </is>
       </c>
       <c r="AB76" s="4" t="n">
-        <v>58</v>
+        <v>162</v>
       </c>
       <c r="AC76" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -5401,16 +5401,16 @@
         </is>
       </c>
       <c r="AB77" s="7" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="AC77" s="7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -5442,16 +5442,16 @@
         </is>
       </c>
       <c r="AB78" s="4" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="AC78" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD78" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -5483,11 +5483,11 @@
         </is>
       </c>
       <c r="AB79" s="7" t="n">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="AC79" s="7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD79" s="7" t="inlineStr">
@@ -5524,11 +5524,11 @@
         </is>
       </c>
       <c r="AB80" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC80" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD80" s="4" t="inlineStr">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="AB81" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC81" s="7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD81" s="7" t="inlineStr">
@@ -5606,11 +5606,11 @@
         </is>
       </c>
       <c r="AB82" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC82" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="AD82" s="4" t="inlineStr">
@@ -5647,11 +5647,11 @@
         </is>
       </c>
       <c r="AB83" s="7" t="n">
-        <v>324</v>
+        <v>443</v>
       </c>
       <c r="AC83" s="7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD83" s="7" t="inlineStr">
@@ -5688,16 +5688,16 @@
         </is>
       </c>
       <c r="AB84" s="4" t="n">
-        <v>195</v>
+        <v>36</v>
       </c>
       <c r="AC84" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD84" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -5729,16 +5729,16 @@
         </is>
       </c>
       <c r="AB85" s="7" t="n">
-        <v>52</v>
+        <v>150</v>
       </c>
       <c r="AC85" s="7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD85" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -5770,16 +5770,16 @@
         </is>
       </c>
       <c r="AB86" s="4" t="n">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="AC86" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD86" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -5811,16 +5811,16 @@
         </is>
       </c>
       <c r="AB87" s="7" t="n">
-        <v>136</v>
+        <v>36</v>
       </c>
       <c r="AC87" s="7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD87" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -5856,12 +5856,12 @@
       </c>
       <c r="AC88" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD88" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
     </row>
@@ -5893,16 +5893,16 @@
         </is>
       </c>
       <c r="AB89" s="7" t="n">
-        <v>8</v>
+        <v>129</v>
       </c>
       <c r="AC89" s="7" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD89" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -5938,12 +5938,12 @@
       </c>
       <c r="AC90" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD90" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -5975,16 +5975,16 @@
         </is>
       </c>
       <c r="AB91" s="7" t="n">
-        <v>327</v>
+        <v>7</v>
       </c>
       <c r="AC91" s="7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD91" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -6016,16 +6016,16 @@
         </is>
       </c>
       <c r="AB92" s="4" t="n">
-        <v>176</v>
+        <v>2</v>
       </c>
       <c r="AC92" s="4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="AD92" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -6057,16 +6057,16 @@
         </is>
       </c>
       <c r="AB93" s="7" t="n">
-        <v>51</v>
+        <v>324</v>
       </c>
       <c r="AC93" s="7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD93" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -6098,16 +6098,16 @@
         </is>
       </c>
       <c r="AB94" s="4" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="AC94" s="4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD94" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -6139,16 +6139,16 @@
         </is>
       </c>
       <c r="AB95" s="7" t="n">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="AC95" s="7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD95" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -6180,16 +6180,16 @@
         </is>
       </c>
       <c r="AB96" s="4" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="AC96" s="4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD96" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -6221,16 +6221,16 @@
         </is>
       </c>
       <c r="AB97" s="7" t="n">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="AC97" s="7" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD97" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -6262,16 +6262,16 @@
         </is>
       </c>
       <c r="AB98" s="4" t="n">
-        <v>2</v>
+        <v>136</v>
       </c>
       <c r="AC98" s="4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD98" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -6303,16 +6303,16 @@
         </is>
       </c>
       <c r="AB99" s="7" t="n">
-        <v>319</v>
+        <v>1</v>
       </c>
       <c r="AC99" s="7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD99" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -6344,16 +6344,16 @@
         </is>
       </c>
       <c r="AB100" s="4" t="n">
-        <v>172</v>
+        <v>8</v>
       </c>
       <c r="AC100" s="4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD100" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -6385,16 +6385,16 @@
         </is>
       </c>
       <c r="AB101" s="7" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AC101" s="7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="AD101" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -6426,16 +6426,16 @@
         </is>
       </c>
       <c r="AB102" s="4" t="n">
-        <v>31</v>
+        <v>327</v>
       </c>
       <c r="AC102" s="4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD102" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -6467,16 +6467,16 @@
         </is>
       </c>
       <c r="AB103" s="7" t="n">
-        <v>140</v>
+        <v>26</v>
       </c>
       <c r="AC103" s="7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD103" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -6508,16 +6508,16 @@
         </is>
       </c>
       <c r="AB104" s="4" t="n">
-        <v>3</v>
+        <v>176</v>
       </c>
       <c r="AC104" s="4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD104" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -6549,16 +6549,16 @@
         </is>
       </c>
       <c r="AB105" s="7" t="n">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="AC105" s="7" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD105" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -6590,16 +6590,16 @@
         </is>
       </c>
       <c r="AB106" s="4" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="AC106" s="4" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD106" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -6631,16 +6631,16 @@
         </is>
       </c>
       <c r="AB107" s="7" t="n">
-        <v>332</v>
+        <v>156</v>
       </c>
       <c r="AC107" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD107" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -6672,16 +6672,16 @@
         </is>
       </c>
       <c r="AB108" s="4" t="n">
-        <v>158</v>
+        <v>1</v>
       </c>
       <c r="AC108" s="4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD108" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -6713,16 +6713,16 @@
         </is>
       </c>
       <c r="AB109" s="7" t="n">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="AC109" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD109" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -6754,16 +6754,16 @@
         </is>
       </c>
       <c r="AB110" s="4" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="AC110" s="4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="AD110" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -6795,16 +6795,16 @@
         </is>
       </c>
       <c r="AB111" s="7" t="n">
-        <v>141</v>
+        <v>319</v>
       </c>
       <c r="AC111" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD111" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -6836,16 +6836,16 @@
         </is>
       </c>
       <c r="AB112" s="4" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="AC112" s="4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD112" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -6877,16 +6877,16 @@
         </is>
       </c>
       <c r="AB113" s="7" t="n">
-        <v>6</v>
+        <v>172</v>
       </c>
       <c r="AC113" s="7" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD113" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -6918,16 +6918,16 @@
         </is>
       </c>
       <c r="AB114" s="4" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="AC114" s="4" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD114" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -6959,16 +6959,16 @@
         </is>
       </c>
       <c r="AB115" s="7" t="n">
-        <v>323</v>
+        <v>31</v>
       </c>
       <c r="AC115" s="7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD115" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -7000,16 +7000,16 @@
         </is>
       </c>
       <c r="AB116" s="4" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="AC116" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD116" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -7041,16 +7041,16 @@
         </is>
       </c>
       <c r="AB117" s="7" t="n">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="AC117" s="7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD117" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -7082,16 +7082,16 @@
         </is>
       </c>
       <c r="AB118" s="4" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="AC118" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD118" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -7123,16 +7123,16 @@
         </is>
       </c>
       <c r="AB119" s="7" t="n">
-        <v>146</v>
+        <v>1</v>
       </c>
       <c r="AC119" s="7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="AD119" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -7164,16 +7164,16 @@
         </is>
       </c>
       <c r="AB120" s="4" t="n">
-        <v>3</v>
+        <v>332</v>
       </c>
       <c r="AC120" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD120" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -7205,16 +7205,16 @@
         </is>
       </c>
       <c r="AB121" s="7" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="AC121" s="7" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD121" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -7246,16 +7246,16 @@
         </is>
       </c>
       <c r="AB122" s="4" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="AC122" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD122" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -7287,16 +7287,16 @@
         </is>
       </c>
       <c r="AB123" s="7" t="n">
-        <v>350</v>
+        <v>54</v>
       </c>
       <c r="AC123" s="7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD123" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -7328,16 +7328,16 @@
         </is>
       </c>
       <c r="AB124" s="4" t="n">
-        <v>152</v>
+        <v>30</v>
       </c>
       <c r="AC124" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD124" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -7369,16 +7369,16 @@
         </is>
       </c>
       <c r="AB125" s="7" t="n">
-        <v>44</v>
+        <v>141</v>
       </c>
       <c r="AC125" s="7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD125" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -7410,16 +7410,16 @@
         </is>
       </c>
       <c r="AB126" s="4" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="AC126" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD126" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -7451,16 +7451,16 @@
         </is>
       </c>
       <c r="AB127" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AC127" s="7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD127" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -7492,16 +7492,16 @@
         </is>
       </c>
       <c r="AB128" s="4" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="AC128" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="AD128" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -7533,16 +7533,16 @@
         </is>
       </c>
       <c r="AB129" s="7" t="n">
-        <v>3</v>
+        <v>323</v>
       </c>
       <c r="AC129" s="7" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD129" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -7574,16 +7574,16 @@
         </is>
       </c>
       <c r="AB130" s="4" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="AC130" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD130" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -7615,16 +7615,16 @@
         </is>
       </c>
       <c r="AB131" s="7" t="n">
-        <v>319</v>
+        <v>132</v>
       </c>
       <c r="AC131" s="7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD131" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="AB132" s="4" t="n">
-        <v>140</v>
+        <v>39</v>
       </c>
       <c r="AC132" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD132" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -7697,16 +7697,16 @@
         </is>
       </c>
       <c r="AB133" s="7" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="AC133" s="7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD133" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -7738,16 +7738,16 @@
         </is>
       </c>
       <c r="AB134" s="4" t="n">
-        <v>42</v>
+        <v>146</v>
       </c>
       <c r="AC134" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD134" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -7779,16 +7779,16 @@
         </is>
       </c>
       <c r="AB135" s="7" t="n">
-        <v>128</v>
+        <v>3</v>
       </c>
       <c r="AC135" s="7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD135" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -7820,16 +7820,16 @@
         </is>
       </c>
       <c r="AB136" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC136" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD136" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -7861,16 +7861,16 @@
         </is>
       </c>
       <c r="AB137" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AC137" s="7" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="AD137" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
     </row>
@@ -7902,16 +7902,16 @@
         </is>
       </c>
       <c r="AB138" s="4" t="n">
-        <v>2</v>
+        <v>350</v>
       </c>
       <c r="AC138" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD138" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -7943,16 +7943,16 @@
         </is>
       </c>
       <c r="AB139" s="7" t="n">
-        <v>325</v>
+        <v>23</v>
       </c>
       <c r="AC139" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD139" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -7984,11 +7984,11 @@
         </is>
       </c>
       <c r="AB140" s="4" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="AC140" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD140" s="4" t="inlineStr">
@@ -8025,11 +8025,11 @@
         </is>
       </c>
       <c r="AB141" s="7" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="AC141" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD141" s="7" t="inlineStr">
@@ -8066,11 +8066,11 @@
         </is>
       </c>
       <c r="AB142" s="4" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="AC142" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD142" s="4" t="inlineStr">
@@ -8107,16 +8107,16 @@
         </is>
       </c>
       <c r="AB143" s="7" t="n">
-        <v>110</v>
+        <v>1</v>
       </c>
       <c r="AC143" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD143" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
     </row>
@@ -8148,16 +8148,16 @@
         </is>
       </c>
       <c r="AB144" s="4" t="n">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="AC144" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD144" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -8189,16 +8189,16 @@
         </is>
       </c>
       <c r="AB145" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AC145" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD145" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
     </row>
@@ -8230,16 +8230,16 @@
         </is>
       </c>
       <c r="AB146" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC146" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="AD146" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
     </row>
@@ -8270,9 +8270,19 @@
           <t>com.logistics.rider.foody</t>
         </is>
       </c>
-      <c r="AB147" s="7" t="n"/>
-      <c r="AC147" s="7" t="n"/>
-      <c r="AD147" s="7" t="n"/>
+      <c r="AB147" s="7" t="n">
+        <v>319</v>
+      </c>
+      <c r="AC147" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD147" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="T148" s="4" t="inlineStr">
@@ -8291,9 +8301,19 @@
       <c r="X148" s="4" t="n"/>
       <c r="Y148" s="4" t="n"/>
       <c r="Z148" s="4" t="n"/>
-      <c r="AB148" s="4" t="n"/>
-      <c r="AC148" s="4" t="n"/>
-      <c r="AD148" s="4" t="n"/>
+      <c r="AB148" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="AC148" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD148" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="T149" s="7" t="inlineStr">
@@ -8312,9 +8332,19 @@
       <c r="X149" s="7" t="n"/>
       <c r="Y149" s="7" t="n"/>
       <c r="Z149" s="7" t="n"/>
-      <c r="AB149" s="7" t="n"/>
-      <c r="AC149" s="7" t="n"/>
-      <c r="AD149" s="7" t="n"/>
+      <c r="AB149" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="AC149" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD149" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="T150" s="4" t="inlineStr">
@@ -8333,9 +8363,19 @@
       <c r="X150" s="4" t="n"/>
       <c r="Y150" s="4" t="n"/>
       <c r="Z150" s="4" t="n"/>
-      <c r="AB150" s="4" t="n"/>
-      <c r="AC150" s="4" t="n"/>
-      <c r="AD150" s="4" t="n"/>
+      <c r="AB150" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="AC150" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD150" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="T151" s="7" t="inlineStr">
@@ -8354,9 +8394,19 @@
       <c r="X151" s="7" t="n"/>
       <c r="Y151" s="7" t="n"/>
       <c r="Z151" s="7" t="n"/>
-      <c r="AB151" s="7" t="n"/>
-      <c r="AC151" s="7" t="n"/>
-      <c r="AD151" s="7" t="n"/>
+      <c r="AB151" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="AC151" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD151" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="T152" s="4" t="inlineStr">
@@ -8375,9 +8425,19 @@
       <c r="X152" s="4" t="n"/>
       <c r="Y152" s="4" t="n"/>
       <c r="Z152" s="4" t="n"/>
-      <c r="AB152" s="4" t="n"/>
-      <c r="AC152" s="4" t="n"/>
-      <c r="AD152" s="4" t="n"/>
+      <c r="AB152" s="4" t="n">
+        <v>128</v>
+      </c>
+      <c r="AC152" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD152" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="T153" s="7" t="inlineStr">
@@ -8396,9 +8456,19 @@
       <c r="X153" s="7" t="n"/>
       <c r="Y153" s="7" t="n"/>
       <c r="Z153" s="7" t="n"/>
-      <c r="AB153" s="7" t="n"/>
-      <c r="AC153" s="7" t="n"/>
-      <c r="AD153" s="7" t="n"/>
+      <c r="AB153" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC153" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD153" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="T154" s="4" t="inlineStr">
@@ -8417,9 +8487,19 @@
       <c r="X154" s="4" t="n"/>
       <c r="Y154" s="4" t="n"/>
       <c r="Z154" s="4" t="n"/>
-      <c r="AB154" s="4" t="n"/>
-      <c r="AC154" s="4" t="n"/>
-      <c r="AD154" s="4" t="n"/>
+      <c r="AB154" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC154" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD154" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="T155" s="7" t="inlineStr">
@@ -8438,9 +8518,19 @@
       <c r="X155" s="7" t="n"/>
       <c r="Y155" s="7" t="n"/>
       <c r="Z155" s="7" t="n"/>
-      <c r="AB155" s="7" t="n"/>
-      <c r="AC155" s="7" t="n"/>
-      <c r="AD155" s="7" t="n"/>
+      <c r="AB155" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC155" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="AD155" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="T156" s="4" t="inlineStr">
@@ -8459,9 +8549,19 @@
       <c r="X156" s="4" t="n"/>
       <c r="Y156" s="4" t="n"/>
       <c r="Z156" s="4" t="n"/>
-      <c r="AB156" s="4" t="n"/>
-      <c r="AC156" s="4" t="n"/>
-      <c r="AD156" s="4" t="n"/>
+      <c r="AB156" s="4" t="n">
+        <v>325</v>
+      </c>
+      <c r="AC156" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD156" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="T157" s="7" t="inlineStr">
@@ -8480,9 +8580,19 @@
       <c r="X157" s="7" t="n"/>
       <c r="Y157" s="7" t="n"/>
       <c r="Z157" s="7" t="n"/>
-      <c r="AB157" s="7" t="n"/>
-      <c r="AC157" s="7" t="n"/>
-      <c r="AD157" s="7" t="n"/>
+      <c r="AB157" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="AC157" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD157" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="T158" s="4" t="inlineStr">
@@ -8501,9 +8611,19 @@
       <c r="X158" s="4" t="n"/>
       <c r="Y158" s="4" t="n"/>
       <c r="Z158" s="4" t="n"/>
-      <c r="AB158" s="4" t="n"/>
-      <c r="AC158" s="4" t="n"/>
-      <c r="AD158" s="4" t="n"/>
+      <c r="AB158" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="AC158" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD158" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="T159" s="7" t="inlineStr">
@@ -8522,9 +8642,19 @@
       <c r="X159" s="7" t="n"/>
       <c r="Y159" s="7" t="n"/>
       <c r="Z159" s="7" t="n"/>
-      <c r="AB159" s="7" t="n"/>
-      <c r="AC159" s="7" t="n"/>
-      <c r="AD159" s="7" t="n"/>
+      <c r="AB159" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="AC159" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD159" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="T160" s="4" t="inlineStr">
@@ -8543,9 +8673,19 @@
       <c r="X160" s="4" t="n"/>
       <c r="Y160" s="4" t="n"/>
       <c r="Z160" s="4" t="n"/>
-      <c r="AB160" s="4" t="n"/>
-      <c r="AC160" s="4" t="n"/>
-      <c r="AD160" s="4" t="n"/>
+      <c r="AB160" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="AC160" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD160" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="T161" s="7" t="inlineStr">
@@ -8564,9 +8704,19 @@
       <c r="X161" s="7" t="n"/>
       <c r="Y161" s="7" t="n"/>
       <c r="Z161" s="7" t="n"/>
-      <c r="AB161" s="7" t="n"/>
-      <c r="AC161" s="7" t="n"/>
-      <c r="AD161" s="7" t="n"/>
+      <c r="AB161" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="AC161" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD161" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="T162" s="4" t="inlineStr">
@@ -8585,9 +8735,19 @@
       <c r="X162" s="4" t="n"/>
       <c r="Y162" s="4" t="n"/>
       <c r="Z162" s="4" t="n"/>
-      <c r="AB162" s="4" t="n"/>
-      <c r="AC162" s="4" t="n"/>
-      <c r="AD162" s="4" t="n"/>
+      <c r="AB162" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC162" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD162" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="T163" s="7" t="inlineStr">
@@ -8606,9 +8766,19 @@
       <c r="X163" s="7" t="n"/>
       <c r="Y163" s="7" t="n"/>
       <c r="Z163" s="7" t="n"/>
-      <c r="AB163" s="7" t="n"/>
-      <c r="AC163" s="7" t="n"/>
-      <c r="AD163" s="7" t="n"/>
+      <c r="AB163" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC163" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD163" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="T164" s="4" t="inlineStr">
@@ -8627,9 +8797,19 @@
       <c r="X164" s="4" t="n"/>
       <c r="Y164" s="4" t="n"/>
       <c r="Z164" s="4" t="n"/>
-      <c r="AB164" s="4" t="n"/>
-      <c r="AC164" s="4" t="n"/>
-      <c r="AD164" s="4" t="n"/>
+      <c r="AB164" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC164" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="AD164" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="T165" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Fixed auto generated report issue
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -699,11 +699,11 @@
         </is>
       </c>
       <c r="B2" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A2&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A2&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*"),M2))*100,2)</f>
         <v/>
       </c>
       <c r="C2" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A2&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A2&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A2&amp;"*"),M2))*100,2)</f>
         <v/>
       </c>
       <c r="D2" s="4" t="n">
@@ -735,11 +735,11 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A3&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A3&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*"),M3))*100,2)</f>
         <v/>
       </c>
       <c r="C3" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A3&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A3&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A3&amp;"*"),M3))*100,2)</f>
         <v/>
       </c>
       <c r="D3" s="7" t="n">
@@ -771,11 +771,11 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A4&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A4&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*"),M4))*100,2)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A4&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A4&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A4&amp;"*"),M4))*100,2)</f>
         <v/>
       </c>
       <c r="D4" s="4" t="n">
@@ -807,11 +807,11 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A5&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A5&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*"),M5))*100,2)</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A5&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A5&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A5&amp;"*"),M5))*100,2)</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
@@ -843,11 +843,11 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A6&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A6&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*"),M6))*100,2)</f>
         <v/>
       </c>
       <c r="C6" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A6&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A6&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A6&amp;"*"),M6))*100,2)</f>
         <v/>
       </c>
       <c r="D6" s="4" t="n">
@@ -879,11 +879,11 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A7&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A7&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*"),M7))*100,2)</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A7&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A7&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A7&amp;"*"),M7))*100,2)</f>
         <v/>
       </c>
       <c r="D7" s="7" t="n">
@@ -915,11 +915,11 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A8&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A8&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*"),M8))*100,2)</f>
         <v/>
       </c>
       <c r="C8" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A8&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A8&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A8&amp;"*"),M8))*100,2)</f>
         <v/>
       </c>
       <c r="D8" s="4" t="n">
@@ -951,11 +951,11 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A9&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A9&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*"),M9))*100,2)</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A9&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A9&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A9&amp;"*"),M9))*100,2)</f>
         <v/>
       </c>
       <c r="D9" s="7" t="n">
@@ -987,11 +987,11 @@
         </is>
       </c>
       <c r="B10" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A10&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A10&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*"),M10))*100,2)</f>
         <v/>
       </c>
       <c r="C10" s="4">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A10&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A10&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A10&amp;"*"),M10))*100,2)</f>
         <v/>
       </c>
       <c r="D10" s="4" t="n">
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A11&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$X:$X,Dashboard!$Z:$Z,"*"&amp;$A11&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*"),M11))*100,2)</f>
         <v/>
       </c>
       <c r="C11" s="7">
-        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A11&amp;"*")/SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(Dashboard!$AB:$AB,Dashboard!$AD:$AD,"*"&amp;$A11&amp;"*")/IF(SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*")&gt;0,SUMIFS(Dashboard!$V:$V,Dashboard!$U:$U,"*"&amp;$A11&amp;"*"),M11))*100,2)</f>
         <v/>
       </c>
       <c r="D11" s="7" t="n">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="F2" s="4" t="n"/>
       <c r="G2" s="4">
-        <f>ROUND((1-E2/D2)*100,2)</f>
+        <f>ROUND((1-E2/IF(D2&gt;0,D2,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H2" s="4">
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="L2" s="4">
-        <f>ROUND(100*(1-K2/D2),2)</f>
+        <f>ROUND(100*(1-K2/IF(D2&gt;0,D2,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M2" s="4">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="F3" s="7" t="n"/>
       <c r="G3" s="7">
-        <f>ROUND((1-E3/D3)*100,2)</f>
+        <f>ROUND((1-E3/IF(D3&gt;0,D3,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H3" s="7">
@@ -1418,7 +1418,7 @@
         <v/>
       </c>
       <c r="L3" s="7">
-        <f>ROUND(100*(1-K3/D3),2)</f>
+        <f>ROUND(100*(1-K3/IF(D3&gt;0,D3,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M3" s="7">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4">
-        <f>ROUND((1-E4/D4)*100,2)</f>
+        <f>ROUND((1-E4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H4" s="4">
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="L4" s="4">
-        <f>ROUND(100*(1-K4/D4),2)</f>
+        <f>ROUND(100*(1-K4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M4" s="4">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="7">
-        <f>ROUND((1-E5/D5)*100,2)</f>
+        <f>ROUND((1-E5/IF(D5&gt;0,D5,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H5" s="7">
@@ -1582,7 +1582,7 @@
         <v/>
       </c>
       <c r="L5" s="7">
-        <f>ROUND(100*(1-K5/D5),2)</f>
+        <f>ROUND(100*(1-K5/IF(D5&gt;0,D5,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M5" s="7">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4">
-        <f>ROUND((1-E6/D6)*100,2)</f>
+        <f>ROUND((1-E6/IF(D6&gt;0,D6,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H6" s="4">
@@ -1667,7 +1667,7 @@
         <v/>
       </c>
       <c r="L6" s="4">
-        <f>ROUND(100*(1-K6/D6),2)</f>
+        <f>ROUND(100*(1-K6/IF(D6&gt;0,D6,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M6" s="4">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7">
-        <f>ROUND((1-E7/D7)*100,2)</f>
+        <f>ROUND((1-E7/IF(D7&gt;0,D7,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H7" s="7">
@@ -1752,7 +1752,7 @@
         <v/>
       </c>
       <c r="L7" s="7">
-        <f>ROUND(100*(1-K7/D7),2)</f>
+        <f>ROUND(100*(1-K7/IF(D7&gt;0,D7,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M7" s="7">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4">
-        <f>ROUND((1-E8/D8)*100,2)</f>
+        <f>ROUND((1-E8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H8" s="4">
@@ -1837,7 +1837,7 @@
         <v/>
       </c>
       <c r="L8" s="4">
-        <f>ROUND(100*(1-K8/D8),2)</f>
+        <f>ROUND(100*(1-K8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M8" s="4">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7">
-        <f>ROUND((1-E9/D9)*100,2)</f>
+        <f>ROUND((1-E9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H9" s="7">
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="L9" s="7">
-        <f>ROUND(100*(1-K9/D9),2)</f>
+        <f>ROUND(100*(1-K9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M9" s="7">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4">
-        <f>ROUND((1-E10/D10)*100,2)</f>
+        <f>ROUND((1-E10/IF(D10&gt;0,D10,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H10" s="4">
@@ -2003,7 +2003,7 @@
         <v/>
       </c>
       <c r="L10" s="4">
-        <f>ROUND(100*(1-K10/D10),2)</f>
+        <f>ROUND(100*(1-K10/IF(D10&gt;0,D10,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M10" s="4">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="7">
-        <f>ROUND((1-E11/D11)*100,2)</f>
+        <f>ROUND((1-E11/IF(D11&gt;0,D11,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H11" s="7">
@@ -2082,7 +2082,7 @@
         <v/>
       </c>
       <c r="L11" s="7">
-        <f>ROUND(100*(1-K11/D11),2)</f>
+        <f>ROUND(100*(1-K11/IF(D11&gt;0,D11,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M11" s="7">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4">
-        <f>ROUND((1-E12/D12)*100,2)</f>
+        <f>ROUND((1-E12/IF(D12&gt;0,D12,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H12" s="4">
@@ -2161,7 +2161,7 @@
         <v/>
       </c>
       <c r="L12" s="4">
-        <f>ROUND(100*(1-K12/D12),2)</f>
+        <f>ROUND(100*(1-K12/IF(D12&gt;0,D12,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M12" s="4">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="7">
-        <f>ROUND((1-E13/D13)*100,2)</f>
+        <f>ROUND((1-E13/IF(D13&gt;0,D13,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H13" s="7">
@@ -2240,7 +2240,7 @@
         <v/>
       </c>
       <c r="L13" s="7">
-        <f>ROUND(100*(1-K13/D13),2)</f>
+        <f>ROUND(100*(1-K13/IF(D13&gt;0,D13,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M13" s="7">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4">
-        <f>ROUND((1-E14/D14)*100,2)</f>
+        <f>ROUND((1-E14/IF(D14&gt;0,D14,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H14" s="4">
@@ -2319,7 +2319,7 @@
         <v/>
       </c>
       <c r="L14" s="4">
-        <f>ROUND(100*(1-K14/D14),2)</f>
+        <f>ROUND(100*(1-K14/IF(D14&gt;0,D14,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M14" s="4">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="7">
-        <f>ROUND((1-E15/D15)*100,2)</f>
+        <f>ROUND((1-E15/IF(D15&gt;0,D15,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H15" s="7">
@@ -2398,7 +2398,7 @@
         <v/>
       </c>
       <c r="L15" s="7">
-        <f>ROUND(100*(1-K15/D15),2)</f>
+        <f>ROUND(100*(1-K15/IF(D15&gt;0,D15,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M15" s="7">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4">
-        <f>ROUND((1-E16/D16)*100,2)</f>
+        <f>ROUND((1-E16/IF(D16&gt;0,D16,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H16" s="4">
@@ -2477,7 +2477,7 @@
         <v/>
       </c>
       <c r="L16" s="4">
-        <f>ROUND(100*(1-K16/D16),2)</f>
+        <f>ROUND(100*(1-K16/IF(D16&gt;0,D16,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M16" s="4">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="7">
-        <f>ROUND((1-E17/D17)*100,2)</f>
+        <f>ROUND((1-E17/IF(D17&gt;0,D17,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H17" s="7">
@@ -2556,7 +2556,7 @@
         <v/>
       </c>
       <c r="L17" s="7">
-        <f>ROUND(100*(1-K17/D17),2)</f>
+        <f>ROUND(100*(1-K17/IF(D17&gt;0,D17,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M17" s="7">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4">
-        <f>ROUND((1-E18/D18)*100,2)</f>
+        <f>ROUND((1-E18/IF(D18&gt;0,D18,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H18" s="4">
@@ -2635,7 +2635,7 @@
         <v/>
       </c>
       <c r="L18" s="4">
-        <f>ROUND(100*(1-K18/D18),2)</f>
+        <f>ROUND(100*(1-K18/IF(D18&gt;0,D18,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M18" s="4">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="7">
-        <f>ROUND((1-E19/D19)*100,2)</f>
+        <f>ROUND((1-E19/IF(D19&gt;0,D19,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H19" s="7">
@@ -2714,7 +2714,7 @@
         <v/>
       </c>
       <c r="L19" s="7">
-        <f>ROUND(100*(1-K19/D19),2)</f>
+        <f>ROUND(100*(1-K19/IF(D19&gt;0,D19,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M19" s="7">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4">
-        <f>ROUND((1-E20/D20)*100,2)</f>
+        <f>ROUND((1-E20/IF(D20&gt;0,D20,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H20" s="4">
@@ -2793,7 +2793,7 @@
         <v/>
       </c>
       <c r="L20" s="4">
-        <f>ROUND(100*(1-K20/D20),2)</f>
+        <f>ROUND(100*(1-K20/IF(D20&gt;0,D20,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M20" s="4">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7">
-        <f>ROUND((1-E21/D21)*100,2)</f>
+        <f>ROUND((1-E21/IF(D21&gt;0,D21,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H21" s="7">
@@ -2872,7 +2872,7 @@
         <v/>
       </c>
       <c r="L21" s="7">
-        <f>ROUND(100*(1-K21/D21),2)</f>
+        <f>ROUND(100*(1-K21/IF(D21&gt;0,D21,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M21" s="7">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4">
-        <f>ROUND((1-E22/D22)*100,2)</f>
+        <f>ROUND((1-E22/IF(D22&gt;0,D22,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H22" s="4">
@@ -2951,7 +2951,7 @@
         <v/>
       </c>
       <c r="L22" s="4">
-        <f>ROUND(100*(1-K22/D22),2)</f>
+        <f>ROUND(100*(1-K22/IF(D22&gt;0,D22,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M22" s="4">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="7">
-        <f>ROUND((1-E23/D23)*100,2)</f>
+        <f>ROUND((1-E23/IF(D23&gt;0,D23,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H23" s="7">
@@ -3030,7 +3030,7 @@
         <v/>
       </c>
       <c r="L23" s="7">
-        <f>ROUND(100*(1-K23/D23),2)</f>
+        <f>ROUND(100*(1-K23/IF(D23&gt;0,D23,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M23" s="7">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4">
-        <f>ROUND((1-E24/D24)*100,2)</f>
+        <f>ROUND((1-E24/IF(D24&gt;0,D24,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H24" s="4">
@@ -3109,7 +3109,7 @@
         <v/>
       </c>
       <c r="L24" s="4">
-        <f>ROUND(100*(1-K24/D24),2)</f>
+        <f>ROUND(100*(1-K24/IF(D24&gt;0,D24,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M24" s="4">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="7">
-        <f>ROUND((1-E25/D25)*100,2)</f>
+        <f>ROUND((1-E25/IF(D25&gt;0,D25,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H25" s="7">
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="L25" s="7">
-        <f>ROUND(100*(1-K25/D25),2)</f>
+        <f>ROUND(100*(1-K25/IF(D25&gt;0,D25,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M25" s="7">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4">
-        <f>ROUND((1-E26/D26)*100,2)</f>
+        <f>ROUND((1-E26/IF(D26&gt;0,D26,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100,2)</f>
         <v/>
       </c>
       <c r="H26" s="4">
@@ -3267,7 +3267,7 @@
         <v/>
       </c>
       <c r="L26" s="4">
-        <f>ROUND(100*(1-K26/D26),2)</f>
+        <f>ROUND(100*(1-K26/IF(D26&gt;0,D26,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)),2)</f>
         <v/>
       </c>
       <c r="M26" s="4">
@@ -3685,7 +3685,7 @@
       <c r="E33" s="27" t="n"/>
       <c r="F33" s="27" t="n"/>
       <c r="G33" s="28">
-        <f>TRUNC((1-SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*")/SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*")/IF(SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*")&gt;0,SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*"),SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")))*100,2)</f>
         <v/>
       </c>
       <c r="H33" s="29">
@@ -3699,7 +3699,7 @@
       <c r="J33" s="27" t="n"/>
       <c r="K33" s="27" t="n"/>
       <c r="L33" s="28">
-        <f>TRUNC((1-SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*")/SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*"))*100,2)</f>
+        <f>TRUNC((1-SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*")/IF(SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*")&gt;0,SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*"),SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")))*100,2)</f>
         <v/>
       </c>
       <c r="M33" s="29">

</xml_diff>

<commit_message>
Updated STTI number, by excluding 4.2624.1, as the release was faulty
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -627,7 +627,7 @@
         <v>4.47</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.63</v>
@@ -663,7 +663,7 @@
         <v>4.47</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0.63</v>
@@ -699,7 +699,7 @@
         <v>4.47</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0.63</v>
@@ -735,7 +735,7 @@
         <v>4.47</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0.63</v>
@@ -771,7 +771,7 @@
         <v>4.47</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0.63</v>
@@ -807,7 +807,7 @@
         <v>4.47</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.63</v>
@@ -843,7 +843,7 @@
         <v>4.47</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.63</v>
@@ -879,7 +879,7 @@
         <v>4.47</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.63</v>
@@ -915,7 +915,7 @@
         <v>4.47</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0.63</v>
@@ -951,7 +951,7 @@
         <v>4.47</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.63</v>

</xml_diff>

<commit_message>
Added device class for hangs and crash reporting to be able to compare based on class distribution
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -719,7 +719,7 @@
         <v>0.74</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>78203</v>
@@ -755,7 +755,7 @@
         <v>0.74</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14946</v>
@@ -791,7 +791,7 @@
         <v>0.74</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>16988</v>
@@ -827,7 +827,7 @@
         <v>0.74</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>20641</v>
@@ -863,7 +863,7 @@
         <v>0.74</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>10630</v>
@@ -899,7 +899,7 @@
         <v>0.74</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>2186</v>
@@ -935,7 +935,7 @@
         <v>0.74</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>46896</v>
@@ -971,7 +971,7 @@
         <v>0.74</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>731</v>
@@ -1007,7 +1007,7 @@
         <v>0.74</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5258</v>
@@ -1043,7 +1043,7 @@
         <v>0.74</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1.28</v>
+        <v>1.3</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>729</v>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD66"/>
+  <dimension ref="A1:AD79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1728,29 +1728,49 @@
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
+      <c r="D7" s="7">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="7">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C7)</f>
+        <v/>
+      </c>
       <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="G7" s="7">
+        <f>ROUND(MAX(0,MIN(100,(1-E7/IF(D7&gt;0,D7,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7">
+        <f>MIN(1,(G7-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
+      <c r="K7" s="7">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="7">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K7/IF(D7&gt;0,D7,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>MAX(0,(L7-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N7" s="7">
+        <f>$B$2+H7+M7</f>
+        <v/>
+      </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="U7" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U7" s="7" t="inlineStr"/>
       <c r="V7" s="7" t="n">
-        <v>5504</v>
+        <v>1</v>
       </c>
       <c r="X7" s="7" t="n">
         <v>95</v>
@@ -1806,7 +1826,7 @@
       <c r="N8" s="4" t="n"/>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
@@ -1815,7 +1835,7 @@
         </is>
       </c>
       <c r="V8" s="4" t="n">
-        <v>5352</v>
+        <v>5504</v>
       </c>
       <c r="X8" s="4" t="n">
         <v>13</v>
@@ -1865,7 +1885,7 @@
       <c r="N9" s="7" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
@@ -1874,7 +1894,7 @@
         </is>
       </c>
       <c r="V9" s="7" t="n">
-        <v>5324</v>
+        <v>5352</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>3</v>
@@ -1932,7 +1952,7 @@
       <c r="N10" s="4" t="n"/>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1941,7 +1961,7 @@
         </is>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5091</v>
+        <v>5324</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>117</v>
@@ -1991,7 +2011,7 @@
       <c r="N11" s="7" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -2000,7 +2020,7 @@
         </is>
       </c>
       <c r="V11" s="7" t="n">
-        <v>4961</v>
+        <v>5091</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>18</v>
@@ -2050,16 +2070,16 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>15599</v>
+        <v>4961</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>71</v>
@@ -2109,16 +2129,16 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>14943</v>
+        <v>5646</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>26</v>
@@ -2168,7 +2188,7 @@
       <c r="N14" s="4" t="n"/>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -2177,7 +2197,7 @@
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>14930</v>
+        <v>15599</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>20</v>
@@ -2227,7 +2247,7 @@
       <c r="N15" s="7" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
@@ -2236,10 +2256,10 @@
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>14111</v>
+        <v>14943</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Y15" s="7" t="inlineStr">
         <is>
@@ -2286,7 +2306,7 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2295,7 +2315,7 @@
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>14130</v>
+        <v>14930</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>11</v>
@@ -2345,16 +2365,16 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>82921</v>
+        <v>14111</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>3</v>
@@ -2404,16 +2424,16 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>80613</v>
+        <v>14130</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>139</v>
@@ -2463,16 +2483,16 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>82716</v>
+        <v>14512</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>14</v>
@@ -2522,7 +2542,7 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2531,7 +2551,7 @@
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>79024</v>
+        <v>82921</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>68</v>
@@ -2581,7 +2601,7 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
@@ -2590,7 +2610,7 @@
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>79116</v>
+        <v>80613</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>28</v>
@@ -2640,16 +2660,16 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>756</v>
+        <v>82716</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>17</v>
@@ -2699,16 +2719,16 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>708</v>
+        <v>79024</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>106</v>
@@ -2758,16 +2778,16 @@
       <c r="N24" s="4" t="n"/>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>733</v>
+        <v>79116</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2817,16 +2837,16 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>662</v>
+        <v>80620</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>9</v>
@@ -2876,7 +2896,7 @@
       <c r="N26" s="4" t="n"/>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
@@ -2885,7 +2905,7 @@
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>678</v>
+        <v>756</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>3</v>
@@ -2935,16 +2955,16 @@
       <c r="N27" s="7" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>48266</v>
+        <v>708</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>145</v>
@@ -2994,16 +3014,16 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V28" s="4" t="n">
-        <v>50405</v>
+        <v>733</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>20</v>
@@ -3053,16 +3073,16 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>48886</v>
+        <v>662</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>73</v>
@@ -3112,16 +3132,16 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>47253</v>
+        <v>678</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>31</v>
@@ -3171,16 +3191,16 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>46972</v>
+        <v>700</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>16</v>
@@ -3235,11 +3255,11 @@
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>1</v>
+        <v>48266</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>108</v>
@@ -3303,11 +3323,11 @@
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>1</v>
+        <v>50405</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>13</v>
@@ -3338,7 +3358,7 @@
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D6)</f>
+        <f>AVERAGE(D2:D7)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3348,7 +3368,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H6)</f>
+        <f>AVERAGE(H2:H7)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3376,11 +3396,11 @@
       </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>1</v>
+        <v>48886</v>
       </c>
       <c r="X34" s="4" t="n">
         <v>2</v>
@@ -3417,11 +3437,11 @@
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>1</v>
+        <v>47253</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>105</v>
@@ -3458,11 +3478,11 @@
       </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>1</v>
+        <v>46972</v>
       </c>
       <c r="X36" s="4" t="n">
         <v>18</v>
@@ -3494,16 +3514,16 @@
     <row r="37">
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>1</v>
+        <v>48667</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>54</v>
@@ -3535,12 +3555,12 @@
     <row r="38">
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
@@ -3576,12 +3596,12 @@
     <row r="39">
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
@@ -3617,12 +3637,12 @@
     <row r="40">
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
@@ -3658,12 +3678,12 @@
     <row r="41">
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V41" s="7" t="n">
@@ -3699,16 +3719,16 @@
     <row r="42">
       <c r="T42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V42" s="4" t="n">
-        <v>10655</v>
+        <v>1</v>
       </c>
       <c r="X42" s="4" t="n">
         <v>9</v>
@@ -3740,16 +3760,16 @@
     <row r="43">
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V43" s="7" t="n">
-        <v>10413</v>
+        <v>1</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>1</v>
@@ -3781,20 +3801,30 @@
     <row r="44">
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V44" s="4" t="n">
-        <v>10036</v>
-      </c>
-      <c r="X44" s="4" t="n"/>
-      <c r="Y44" s="4" t="n"/>
-      <c r="Z44" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X44" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB44" s="4" t="n">
         <v>2</v>
       </c>
@@ -3812,20 +3842,30 @@
     <row r="45">
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V45" s="7" t="n">
-        <v>9869</v>
-      </c>
-      <c r="X45" s="7" t="n"/>
-      <c r="Y45" s="7" t="n"/>
-      <c r="Z45" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X45" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y45" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z45" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB45" s="7" t="n">
         <v>2</v>
       </c>
@@ -3843,20 +3883,30 @@
     <row r="46">
       <c r="T46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U46" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V46" s="4" t="n">
-        <v>10072</v>
-      </c>
-      <c r="X46" s="4" t="n"/>
-      <c r="Y46" s="4" t="n"/>
-      <c r="Z46" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X46" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y46" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z46" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB46" s="4" t="n">
         <v>4</v>
       </c>
@@ -3874,205 +3924,335 @@
     <row r="47">
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V47" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X47" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y47" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z47" s="7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V47" s="7" t="n">
-        <v>23063</v>
-      </c>
-      <c r="X47" s="7" t="n"/>
-      <c r="Y47" s="7" t="n"/>
-      <c r="Z47" s="7" t="n"/>
-      <c r="AB47" s="7" t="n"/>
-      <c r="AC47" s="7" t="n"/>
-      <c r="AD47" s="7" t="n"/>
+      <c r="AB47" s="7" t="n">
+        <v>388</v>
+      </c>
+      <c r="AC47" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD47" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U48" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V48" s="4" t="n">
-        <v>23168</v>
-      </c>
-      <c r="X48" s="4" t="n"/>
-      <c r="Y48" s="4" t="n"/>
-      <c r="Z48" s="4" t="n"/>
-      <c r="AB48" s="4" t="n"/>
-      <c r="AC48" s="4" t="n"/>
-      <c r="AD48" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X48" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y48" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z48" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB48" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="AC48" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD48" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V49" s="7" t="n">
-        <v>24394</v>
-      </c>
-      <c r="X49" s="7" t="n"/>
-      <c r="Y49" s="7" t="n"/>
-      <c r="Z49" s="7" t="n"/>
-      <c r="AB49" s="7" t="n"/>
-      <c r="AC49" s="7" t="n"/>
-      <c r="AD49" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X49" s="7" t="n">
+        <v>115</v>
+      </c>
+      <c r="Y49" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z49" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB49" s="7" t="n">
+        <v>176</v>
+      </c>
+      <c r="AC49" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD49" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="T50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V50" s="4" t="n">
+        <v>10655</v>
+      </c>
+      <c r="X50" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="Z50" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB50" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD50" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V50" s="4" t="n">
-        <v>21980</v>
-      </c>
-      <c r="X50" s="4" t="n"/>
-      <c r="Y50" s="4" t="n"/>
-      <c r="Z50" s="4" t="n"/>
-      <c r="AB50" s="4" t="n"/>
-      <c r="AC50" s="4" t="n"/>
-      <c r="AD50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V51" s="7" t="n">
-        <v>21517</v>
+        <v>10413</v>
       </c>
       <c r="X51" s="7" t="n"/>
       <c r="Y51" s="7" t="n"/>
       <c r="Z51" s="7" t="n"/>
-      <c r="AB51" s="7" t="n"/>
-      <c r="AC51" s="7" t="n"/>
-      <c r="AD51" s="7" t="n"/>
+      <c r="AB51" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="AC51" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD51" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="T52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V52" s="4" t="n">
-        <v>17887</v>
+        <v>10036</v>
       </c>
       <c r="X52" s="4" t="n"/>
       <c r="Y52" s="4" t="n"/>
       <c r="Z52" s="4" t="n"/>
-      <c r="AB52" s="4" t="n"/>
-      <c r="AC52" s="4" t="n"/>
-      <c r="AD52" s="4" t="n"/>
+      <c r="AB52" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="AC52" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD52" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V53" s="7" t="n">
-        <v>17641</v>
+        <v>9869</v>
       </c>
       <c r="X53" s="7" t="n"/>
       <c r="Y53" s="7" t="n"/>
       <c r="Z53" s="7" t="n"/>
-      <c r="AB53" s="7" t="n"/>
-      <c r="AC53" s="7" t="n"/>
-      <c r="AD53" s="7" t="n"/>
+      <c r="AB53" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC53" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD53" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="T54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V54" s="4" t="n">
-        <v>17144</v>
+        <v>10072</v>
       </c>
       <c r="X54" s="4" t="n"/>
       <c r="Y54" s="4" t="n"/>
       <c r="Z54" s="4" t="n"/>
-      <c r="AB54" s="4" t="n"/>
-      <c r="AC54" s="4" t="n"/>
-      <c r="AD54" s="4" t="n"/>
+      <c r="AB54" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD54" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V55" s="7" t="n">
-        <v>17159</v>
+        <v>10125</v>
       </c>
       <c r="X55" s="7" t="n"/>
       <c r="Y55" s="7" t="n"/>
       <c r="Z55" s="7" t="n"/>
-      <c r="AB55" s="7" t="n"/>
-      <c r="AC55" s="7" t="n"/>
-      <c r="AD55" s="7" t="n"/>
+      <c r="AB55" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC55" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="AD55" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V56" s="4" t="n">
-        <v>17724</v>
+        <v>23063</v>
       </c>
       <c r="X56" s="4" t="n"/>
       <c r="Y56" s="4" t="n"/>
@@ -4084,16 +4264,16 @@
     <row r="57">
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V57" s="7" t="n">
-        <v>700</v>
+        <v>23168</v>
       </c>
       <c r="X57" s="7" t="n"/>
       <c r="Y57" s="7" t="n"/>
@@ -4105,16 +4285,16 @@
     <row r="58">
       <c r="T58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U58" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V58" s="4" t="n">
-        <v>686</v>
+        <v>24394</v>
       </c>
       <c r="X58" s="4" t="n"/>
       <c r="Y58" s="4" t="n"/>
@@ -4126,16 +4306,16 @@
     <row r="59">
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V59" s="7" t="n">
-        <v>698</v>
+        <v>21980</v>
       </c>
       <c r="X59" s="7" t="n"/>
       <c r="Y59" s="7" t="n"/>
@@ -4147,16 +4327,16 @@
     <row r="60">
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U60" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V60" s="4" t="n">
-        <v>687</v>
+        <v>21517</v>
       </c>
       <c r="X60" s="4" t="n"/>
       <c r="Y60" s="4" t="n"/>
@@ -4168,16 +4348,16 @@
     <row r="61">
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V61" s="7" t="n">
-        <v>716</v>
+        <v>22785</v>
       </c>
       <c r="X61" s="7" t="n"/>
       <c r="Y61" s="7" t="n"/>
@@ -4194,11 +4374,11 @@
       </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V62" s="4" t="n">
-        <v>2290</v>
+        <v>17887</v>
       </c>
       <c r="X62" s="4" t="n"/>
       <c r="Y62" s="4" t="n"/>
@@ -4215,11 +4395,11 @@
       </c>
       <c r="U63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V63" s="7" t="n">
-        <v>2092</v>
+        <v>17641</v>
       </c>
       <c r="X63" s="7" t="n"/>
       <c r="Y63" s="7" t="n"/>
@@ -4236,11 +4416,11 @@
       </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V64" s="4" t="n">
-        <v>2043</v>
+        <v>17144</v>
       </c>
       <c r="X64" s="4" t="n"/>
       <c r="Y64" s="4" t="n"/>
@@ -4257,11 +4437,11 @@
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V65" s="7" t="n">
-        <v>1969</v>
+        <v>17159</v>
       </c>
       <c r="X65" s="7" t="n"/>
       <c r="Y65" s="7" t="n"/>
@@ -4278,11 +4458,11 @@
       </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V66" s="4" t="n">
-        <v>1938</v>
+        <v>17724</v>
       </c>
       <c r="X66" s="4" t="n"/>
       <c r="Y66" s="4" t="n"/>
@@ -4290,6 +4470,279 @@
       <c r="AB66" s="4" t="n"/>
       <c r="AC66" s="4" t="n"/>
       <c r="AD66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="T67" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U67" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V67" s="7" t="n">
+        <v>17829</v>
+      </c>
+      <c r="X67" s="7" t="n"/>
+      <c r="Y67" s="7" t="n"/>
+      <c r="Z67" s="7" t="n"/>
+      <c r="AB67" s="7" t="n"/>
+      <c r="AC67" s="7" t="n"/>
+      <c r="AD67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="T68" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U68" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V68" s="4" t="n">
+        <v>700</v>
+      </c>
+      <c r="X68" s="4" t="n"/>
+      <c r="Y68" s="4" t="n"/>
+      <c r="Z68" s="4" t="n"/>
+      <c r="AB68" s="4" t="n"/>
+      <c r="AC68" s="4" t="n"/>
+      <c r="AD68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="T69" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U69" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V69" s="7" t="n">
+        <v>686</v>
+      </c>
+      <c r="X69" s="7" t="n"/>
+      <c r="Y69" s="7" t="n"/>
+      <c r="Z69" s="7" t="n"/>
+      <c r="AB69" s="7" t="n"/>
+      <c r="AC69" s="7" t="n"/>
+      <c r="AD69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="T70" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U70" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V70" s="4" t="n">
+        <v>698</v>
+      </c>
+      <c r="X70" s="4" t="n"/>
+      <c r="Y70" s="4" t="n"/>
+      <c r="Z70" s="4" t="n"/>
+      <c r="AB70" s="4" t="n"/>
+      <c r="AC70" s="4" t="n"/>
+      <c r="AD70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="T71" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U71" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V71" s="7" t="n">
+        <v>687</v>
+      </c>
+      <c r="X71" s="7" t="n"/>
+      <c r="Y71" s="7" t="n"/>
+      <c r="Z71" s="7" t="n"/>
+      <c r="AB71" s="7" t="n"/>
+      <c r="AC71" s="7" t="n"/>
+      <c r="AD71" s="7" t="n"/>
+    </row>
+    <row r="72">
+      <c r="T72" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U72" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V72" s="4" t="n">
+        <v>716</v>
+      </c>
+      <c r="X72" s="4" t="n"/>
+      <c r="Y72" s="4" t="n"/>
+      <c r="Z72" s="4" t="n"/>
+      <c r="AB72" s="4" t="n"/>
+      <c r="AC72" s="4" t="n"/>
+      <c r="AD72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="T73" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U73" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V73" s="7" t="n">
+        <v>719</v>
+      </c>
+      <c r="X73" s="7" t="n"/>
+      <c r="Y73" s="7" t="n"/>
+      <c r="Z73" s="7" t="n"/>
+      <c r="AB73" s="7" t="n"/>
+      <c r="AC73" s="7" t="n"/>
+      <c r="AD73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="T74" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U74" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V74" s="4" t="n">
+        <v>2290</v>
+      </c>
+      <c r="X74" s="4" t="n"/>
+      <c r="Y74" s="4" t="n"/>
+      <c r="Z74" s="4" t="n"/>
+      <c r="AB74" s="4" t="n"/>
+      <c r="AC74" s="4" t="n"/>
+      <c r="AD74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="T75" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U75" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V75" s="7" t="n">
+        <v>2092</v>
+      </c>
+      <c r="X75" s="7" t="n"/>
+      <c r="Y75" s="7" t="n"/>
+      <c r="Z75" s="7" t="n"/>
+      <c r="AB75" s="7" t="n"/>
+      <c r="AC75" s="7" t="n"/>
+      <c r="AD75" s="7" t="n"/>
+    </row>
+    <row r="76">
+      <c r="T76" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U76" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V76" s="4" t="n">
+        <v>2043</v>
+      </c>
+      <c r="X76" s="4" t="n"/>
+      <c r="Y76" s="4" t="n"/>
+      <c r="Z76" s="4" t="n"/>
+      <c r="AB76" s="4" t="n"/>
+      <c r="AC76" s="4" t="n"/>
+      <c r="AD76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="T77" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U77" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V77" s="7" t="n">
+        <v>1969</v>
+      </c>
+      <c r="X77" s="7" t="n"/>
+      <c r="Y77" s="7" t="n"/>
+      <c r="Z77" s="7" t="n"/>
+      <c r="AB77" s="7" t="n"/>
+      <c r="AC77" s="7" t="n"/>
+      <c r="AD77" s="7" t="n"/>
+    </row>
+    <row r="78">
+      <c r="T78" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U78" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V78" s="4" t="n">
+        <v>1938</v>
+      </c>
+      <c r="X78" s="4" t="n"/>
+      <c r="Y78" s="4" t="n"/>
+      <c r="Z78" s="4" t="n"/>
+      <c r="AB78" s="4" t="n"/>
+      <c r="AC78" s="4" t="n"/>
+      <c r="AD78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="T79" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U79" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V79" s="7" t="n">
+        <v>2048</v>
+      </c>
+      <c r="X79" s="7" t="n"/>
+      <c r="Y79" s="7" t="n"/>
+      <c r="Z79" s="7" t="n"/>
+      <c r="AB79" s="7" t="n"/>
+      <c r="AC79" s="7" t="n"/>
+      <c r="AD79" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Updated hang categories for location and camera hangs
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -716,10 +716,10 @@
         <v>0.84</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>78203</v>
@@ -752,10 +752,10 @@
         <v>0.84</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14946</v>
@@ -788,10 +788,10 @@
         <v>0.84</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>16988</v>
@@ -824,10 +824,10 @@
         <v>0.84</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>20641</v>
@@ -860,10 +860,10 @@
         <v>0.84</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>10630</v>
@@ -896,10 +896,10 @@
         <v>0.84</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>2186</v>
@@ -932,10 +932,10 @@
         <v>0.84</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>46896</v>
@@ -968,10 +968,10 @@
         <v>0.84</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>731</v>
@@ -1004,10 +1004,10 @@
         <v>0.84</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5258</v>
@@ -1040,10 +1040,10 @@
         <v>0.84</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1.3</v>
+        <v>1.31</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>729</v>
@@ -1094,31 +1094,31 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((B12-99.7)/(99.9-99.7))*50)+50))*0.35,2)</f>
+        <f>MIN(100,MAX(0,(((B12-99.7)/(99.9-99.7))*50)+50))*35%</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((C12-99.7)/(99.9-99.7))*50)+50))*0.25,2)</f>
+        <f>MIN(100,MAX(0,(((C12-99.7)/(99.9-99.7))*50)+50))*25%</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((D12-75)/(60-75))*50)+50))*0.02,2)</f>
+        <f>MIN(100,MAX(0,(((D12-75)/(60-75))*50)+50))*2%</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((E12-4)/(2-4))*50)+50))*0.10,2)</f>
+        <f>MIN(100,MAX(0,(((E12-4)/(2-4))*50)+50))*10%</f>
         <v/>
       </c>
       <c r="F13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((F12-1.5)/(0.5-1.5))*50)+50))*0.10,2)</f>
+        <f>MIN(100,MAX(0,(((F12-1.5)/(0.5-1.5))*50)+50))*10%</f>
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((G12-3)/(1-3))*50)+50))*0.13,2)</f>
+        <f>MIN(100,MAX(0,(((G12-3)/(1-3))*50)+50))*13%</f>
         <v/>
       </c>
       <c r="H13" s="12">
-        <f>ROUND(MIN(100,MAX(0,(((H12-2)/(1-2))*50)+50))*0.05,2)</f>
+        <f>MIN(100,MAX(0,(((H12-2)/(1-2))*50)+50))*5%</f>
         <v/>
       </c>
       <c r="M13" s="11">
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD79"/>
+  <dimension ref="A1:AD92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1813,29 +1813,49 @@
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
+      <c r="D8" s="4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C8)</f>
+        <v/>
+      </c>
       <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
+      <c r="G8" s="4">
+        <f>ROUND(MAX(0,MIN(100,(1-E8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>MIN(1,(G8-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4" t="n"/>
+      <c r="K8" s="4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>MAX(0,(L8-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>$B$2+H8+M8</f>
+        <v/>
+      </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr"/>
       <c r="V8" s="4" t="n">
-        <v>5504</v>
+        <v>1</v>
       </c>
       <c r="X8" s="4" t="n">
         <v>13</v>
@@ -1885,7 +1905,7 @@
       <c r="N9" s="7" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
@@ -1894,7 +1914,7 @@
         </is>
       </c>
       <c r="V9" s="7" t="n">
-        <v>5352</v>
+        <v>5504</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>3</v>
@@ -1952,7 +1972,7 @@
       <c r="N10" s="4" t="n"/>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1961,7 +1981,7 @@
         </is>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5324</v>
+        <v>5352</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>117</v>
@@ -2011,7 +2031,7 @@
       <c r="N11" s="7" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -2020,7 +2040,7 @@
         </is>
       </c>
       <c r="V11" s="7" t="n">
-        <v>5091</v>
+        <v>5324</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>18</v>
@@ -2070,7 +2090,7 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -2079,7 +2099,7 @@
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>4961</v>
+        <v>5091</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>71</v>
@@ -2129,7 +2149,7 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
@@ -2138,7 +2158,7 @@
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>5646</v>
+        <v>4961</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>26</v>
@@ -2188,16 +2208,16 @@
       <c r="N14" s="4" t="n"/>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>15599</v>
+        <v>5646</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>20</v>
@@ -2247,16 +2267,16 @@
       <c r="N15" s="7" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>14943</v>
+        <v>5436</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>81</v>
@@ -2306,7 +2326,7 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2315,7 +2335,7 @@
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>14930</v>
+        <v>15599</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>11</v>
@@ -2365,7 +2385,7 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
@@ -2374,7 +2394,7 @@
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>14111</v>
+        <v>14943</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>3</v>
@@ -2424,7 +2444,7 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
@@ -2433,7 +2453,7 @@
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>14130</v>
+        <v>14930</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>139</v>
@@ -2483,7 +2503,7 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
@@ -2492,7 +2512,7 @@
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>14512</v>
+        <v>14111</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>14</v>
@@ -2542,16 +2562,16 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>82921</v>
+        <v>14130</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>68</v>
@@ -2601,16 +2621,16 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>80613</v>
+        <v>14512</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>28</v>
@@ -2660,16 +2680,16 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>82716</v>
+        <v>14749</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>17</v>
@@ -2719,7 +2739,7 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
@@ -2728,7 +2748,7 @@
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>79024</v>
+        <v>82921</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>106</v>
@@ -2778,7 +2798,7 @@
       <c r="N24" s="4" t="n"/>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -2787,7 +2807,7 @@
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>79116</v>
+        <v>80613</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2837,7 +2857,7 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
@@ -2846,7 +2866,7 @@
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>80620</v>
+        <v>82716</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>9</v>
@@ -2896,16 +2916,16 @@
       <c r="N26" s="4" t="n"/>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>756</v>
+        <v>79024</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>3</v>
@@ -2955,16 +2975,16 @@
       <c r="N27" s="7" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>708</v>
+        <v>79116</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>145</v>
@@ -3014,16 +3034,16 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V28" s="4" t="n">
-        <v>733</v>
+        <v>80620</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>20</v>
@@ -3073,16 +3093,16 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>662</v>
+        <v>80878</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>73</v>
@@ -3132,7 +3152,7 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3141,7 +3161,7 @@
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>678</v>
+        <v>756</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>31</v>
@@ -3191,7 +3211,7 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
@@ -3200,7 +3220,7 @@
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>16</v>
@@ -3250,16 +3270,16 @@
       <c r="N32" s="4" t="n"/>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>48266</v>
+        <v>733</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>108</v>
@@ -3318,16 +3338,16 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>50405</v>
+        <v>662</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>13</v>
@@ -3358,7 +3378,7 @@
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D7)</f>
+        <f>AVERAGE(D2:D8)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3368,7 +3388,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H7)</f>
+        <f>AVERAGE(H2:H8)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3391,16 +3411,16 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>48886</v>
+        <v>678</v>
       </c>
       <c r="X34" s="4" t="n">
         <v>2</v>
@@ -3432,16 +3452,16 @@
     <row r="35">
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>47253</v>
+        <v>700</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>105</v>
@@ -3473,16 +3493,16 @@
     <row r="36">
       <c r="T36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>46972</v>
+        <v>683</v>
       </c>
       <c r="X36" s="4" t="n">
         <v>18</v>
@@ -3514,7 +3534,7 @@
     <row r="37">
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
@@ -3523,7 +3543,7 @@
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>48667</v>
+        <v>48266</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>54</v>
@@ -3555,16 +3575,16 @@
     <row r="38">
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>1</v>
+        <v>50405</v>
       </c>
       <c r="X38" s="4" t="n">
         <v>27</v>
@@ -3596,16 +3616,16 @@
     <row r="39">
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
-        <v>1</v>
+        <v>48886</v>
       </c>
       <c r="X39" s="7" t="n">
         <v>13</v>
@@ -3637,19 +3657,19 @@
     <row r="40">
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>1</v>
+        <v>47253</v>
       </c>
       <c r="X40" s="4" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Y40" s="4" t="inlineStr">
         <is>
@@ -3678,16 +3698,16 @@
     <row r="41">
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V41" s="7" t="n">
-        <v>1</v>
+        <v>46972</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>1</v>
@@ -3719,16 +3739,16 @@
     <row r="42">
       <c r="T42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V42" s="4" t="n">
-        <v>1</v>
+        <v>48667</v>
       </c>
       <c r="X42" s="4" t="n">
         <v>9</v>
@@ -3760,16 +3780,16 @@
     <row r="43">
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V43" s="7" t="n">
-        <v>1</v>
+        <v>48109</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>1</v>
@@ -3806,7 +3826,7 @@
       </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V44" s="4" t="n">
@@ -3847,7 +3867,7 @@
       </c>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V45" s="7" t="n">
@@ -3888,7 +3908,7 @@
       </c>
       <c r="U46" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V46" s="4" t="n">
@@ -3929,7 +3949,7 @@
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V47" s="7" t="n">
@@ -3970,7 +3990,7 @@
       </c>
       <c r="U48" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V48" s="4" t="n">
@@ -4011,7 +4031,7 @@
       </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V49" s="7" t="n">
@@ -4047,16 +4067,16 @@
     <row r="50">
       <c r="T50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V50" s="4" t="n">
-        <v>10655</v>
+        <v>1</v>
       </c>
       <c r="X50" s="4" t="n">
         <v>3</v>
@@ -4088,20 +4108,30 @@
     <row r="51">
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V51" s="7" t="n">
-        <v>10413</v>
-      </c>
-      <c r="X51" s="7" t="n"/>
-      <c r="Y51" s="7" t="n"/>
-      <c r="Z51" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X51" s="7" t="n">
+        <v>127</v>
+      </c>
+      <c r="Y51" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z51" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB51" s="7" t="n">
         <v>37</v>
       </c>
@@ -4119,20 +4149,30 @@
     <row r="52">
       <c r="T52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V52" s="4" t="n">
-        <v>10036</v>
-      </c>
-      <c r="X52" s="4" t="n"/>
-      <c r="Y52" s="4" t="n"/>
-      <c r="Z52" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X52" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y52" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z52" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB52" s="4" t="n">
         <v>178</v>
       </c>
@@ -4150,20 +4190,30 @@
     <row r="53">
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V53" s="7" t="n">
-        <v>9869</v>
-      </c>
-      <c r="X53" s="7" t="n"/>
-      <c r="Y53" s="7" t="n"/>
-      <c r="Z53" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X53" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="Y53" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z53" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB53" s="7" t="n">
         <v>1</v>
       </c>
@@ -4181,20 +4231,30 @@
     <row r="54">
       <c r="T54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V54" s="4" t="n">
-        <v>10072</v>
-      </c>
-      <c r="X54" s="4" t="n"/>
-      <c r="Y54" s="4" t="n"/>
-      <c r="Z54" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X54" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB54" s="4" t="n">
         <v>4</v>
       </c>
@@ -4212,20 +4272,30 @@
     <row r="55">
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X55" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y55" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z55" s="7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
-      <c r="V55" s="7" t="n">
-        <v>10125</v>
-      </c>
-      <c r="X55" s="7" t="n"/>
-      <c r="Y55" s="7" t="n"/>
-      <c r="Z55" s="7" t="n"/>
       <c r="AB55" s="7" t="n">
         <v>3</v>
       </c>
@@ -4243,205 +4313,325 @@
     <row r="56">
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V56" s="4" t="n">
-        <v>23063</v>
-      </c>
-      <c r="X56" s="4" t="n"/>
-      <c r="Y56" s="4" t="n"/>
-      <c r="Z56" s="4" t="n"/>
-      <c r="AB56" s="4" t="n"/>
-      <c r="AC56" s="4" t="n"/>
-      <c r="AD56" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X56" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB56" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V57" s="7" t="n">
-        <v>23168</v>
-      </c>
-      <c r="X57" s="7" t="n"/>
-      <c r="Y57" s="7" t="n"/>
-      <c r="Z57" s="7" t="n"/>
-      <c r="AB57" s="7" t="n"/>
-      <c r="AC57" s="7" t="n"/>
-      <c r="AD57" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y57" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z57" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="AB57" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="AC57" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD57" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="T58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U58" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V58" s="4" t="n">
-        <v>24394</v>
-      </c>
-      <c r="X58" s="4" t="n"/>
-      <c r="Y58" s="4" t="n"/>
-      <c r="Z58" s="4" t="n"/>
-      <c r="AB58" s="4" t="n"/>
-      <c r="AC58" s="4" t="n"/>
-      <c r="AD58" s="4" t="n"/>
+        <v>10655</v>
+      </c>
+      <c r="X58" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y58" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="Z58" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB58" s="4" t="n">
+        <v>176</v>
+      </c>
+      <c r="AC58" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD58" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V59" s="7" t="n">
-        <v>21980</v>
+        <v>10413</v>
       </c>
       <c r="X59" s="7" t="n"/>
       <c r="Y59" s="7" t="n"/>
       <c r="Z59" s="7" t="n"/>
-      <c r="AB59" s="7" t="n"/>
-      <c r="AC59" s="7" t="n"/>
-      <c r="AD59" s="7" t="n"/>
+      <c r="AB59" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="AC59" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD59" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U60" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V60" s="4" t="n">
-        <v>21517</v>
+        <v>10036</v>
       </c>
       <c r="X60" s="4" t="n"/>
       <c r="Y60" s="4" t="n"/>
       <c r="Z60" s="4" t="n"/>
-      <c r="AB60" s="4" t="n"/>
-      <c r="AC60" s="4" t="n"/>
-      <c r="AD60" s="4" t="n"/>
+      <c r="AB60" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="AC60" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD60" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V61" s="7" t="n">
-        <v>22785</v>
+        <v>9869</v>
       </c>
       <c r="X61" s="7" t="n"/>
       <c r="Y61" s="7" t="n"/>
       <c r="Z61" s="7" t="n"/>
-      <c r="AB61" s="7" t="n"/>
-      <c r="AC61" s="7" t="n"/>
-      <c r="AD61" s="7" t="n"/>
+      <c r="AB61" s="7" t="n">
+        <v>152</v>
+      </c>
+      <c r="AC61" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD61" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="T62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V62" s="4" t="n">
-        <v>17887</v>
+        <v>10072</v>
       </c>
       <c r="X62" s="4" t="n"/>
       <c r="Y62" s="4" t="n"/>
       <c r="Z62" s="4" t="n"/>
-      <c r="AB62" s="4" t="n"/>
-      <c r="AC62" s="4" t="n"/>
-      <c r="AD62" s="4" t="n"/>
+      <c r="AB62" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC62" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD62" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="T63" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V63" s="7" t="n">
-        <v>17641</v>
+        <v>10125</v>
       </c>
       <c r="X63" s="7" t="n"/>
       <c r="Y63" s="7" t="n"/>
       <c r="Z63" s="7" t="n"/>
-      <c r="AB63" s="7" t="n"/>
-      <c r="AC63" s="7" t="n"/>
-      <c r="AD63" s="7" t="n"/>
+      <c r="AB63" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC63" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD63" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="T64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V64" s="4" t="n">
-        <v>17144</v>
+        <v>10161</v>
       </c>
       <c r="X64" s="4" t="n"/>
       <c r="Y64" s="4" t="n"/>
       <c r="Z64" s="4" t="n"/>
-      <c r="AB64" s="4" t="n"/>
-      <c r="AC64" s="4" t="n"/>
-      <c r="AD64" s="4" t="n"/>
+      <c r="AB64" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC64" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="AD64" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="T65" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V65" s="7" t="n">
-        <v>17159</v>
+        <v>23063</v>
       </c>
       <c r="X65" s="7" t="n"/>
       <c r="Y65" s="7" t="n"/>
@@ -4453,16 +4643,16 @@
     <row r="66">
       <c r="T66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V66" s="4" t="n">
-        <v>17724</v>
+        <v>23168</v>
       </c>
       <c r="X66" s="4" t="n"/>
       <c r="Y66" s="4" t="n"/>
@@ -4474,16 +4664,16 @@
     <row r="67">
       <c r="T67" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U67" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V67" s="7" t="n">
-        <v>17829</v>
+        <v>24394</v>
       </c>
       <c r="X67" s="7" t="n"/>
       <c r="Y67" s="7" t="n"/>
@@ -4495,16 +4685,16 @@
     <row r="68">
       <c r="T68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U68" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V68" s="4" t="n">
-        <v>700</v>
+        <v>21980</v>
       </c>
       <c r="X68" s="4" t="n"/>
       <c r="Y68" s="4" t="n"/>
@@ -4516,16 +4706,16 @@
     <row r="69">
       <c r="T69" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U69" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V69" s="7" t="n">
-        <v>686</v>
+        <v>21517</v>
       </c>
       <c r="X69" s="7" t="n"/>
       <c r="Y69" s="7" t="n"/>
@@ -4537,16 +4727,16 @@
     <row r="70">
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U70" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V70" s="4" t="n">
-        <v>698</v>
+        <v>22785</v>
       </c>
       <c r="X70" s="4" t="n"/>
       <c r="Y70" s="4" t="n"/>
@@ -4558,16 +4748,16 @@
     <row r="71">
       <c r="T71" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U71" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V71" s="7" t="n">
-        <v>687</v>
+        <v>24108</v>
       </c>
       <c r="X71" s="7" t="n"/>
       <c r="Y71" s="7" t="n"/>
@@ -4579,16 +4769,16 @@
     <row r="72">
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U72" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V72" s="4" t="n">
-        <v>716</v>
+        <v>17887</v>
       </c>
       <c r="X72" s="4" t="n"/>
       <c r="Y72" s="4" t="n"/>
@@ -4600,16 +4790,16 @@
     <row r="73">
       <c r="T73" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U73" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V73" s="7" t="n">
-        <v>719</v>
+        <v>17641</v>
       </c>
       <c r="X73" s="7" t="n"/>
       <c r="Y73" s="7" t="n"/>
@@ -4621,16 +4811,16 @@
     <row r="74">
       <c r="T74" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U74" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V74" s="4" t="n">
-        <v>2290</v>
+        <v>17144</v>
       </c>
       <c r="X74" s="4" t="n"/>
       <c r="Y74" s="4" t="n"/>
@@ -4642,16 +4832,16 @@
     <row r="75">
       <c r="T75" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U75" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V75" s="7" t="n">
-        <v>2092</v>
+        <v>17159</v>
       </c>
       <c r="X75" s="7" t="n"/>
       <c r="Y75" s="7" t="n"/>
@@ -4663,16 +4853,16 @@
     <row r="76">
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V76" s="4" t="n">
-        <v>2043</v>
+        <v>17724</v>
       </c>
       <c r="X76" s="4" t="n"/>
       <c r="Y76" s="4" t="n"/>
@@ -4684,16 +4874,16 @@
     <row r="77">
       <c r="T77" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V77" s="7" t="n">
-        <v>1969</v>
+        <v>17829</v>
       </c>
       <c r="X77" s="7" t="n"/>
       <c r="Y77" s="7" t="n"/>
@@ -4705,16 +4895,16 @@
     <row r="78">
       <c r="T78" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U78" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V78" s="4" t="n">
-        <v>1938</v>
+        <v>18088</v>
       </c>
       <c r="X78" s="4" t="n"/>
       <c r="Y78" s="4" t="n"/>
@@ -4726,16 +4916,16 @@
     <row r="79">
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U79" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V79" s="7" t="n">
-        <v>2048</v>
+        <v>700</v>
       </c>
       <c r="X79" s="7" t="n"/>
       <c r="Y79" s="7" t="n"/>
@@ -4743,6 +4933,279 @@
       <c r="AB79" s="7" t="n"/>
       <c r="AC79" s="7" t="n"/>
       <c r="AD79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="T80" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U80" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V80" s="4" t="n">
+        <v>686</v>
+      </c>
+      <c r="X80" s="4" t="n"/>
+      <c r="Y80" s="4" t="n"/>
+      <c r="Z80" s="4" t="n"/>
+      <c r="AB80" s="4" t="n"/>
+      <c r="AC80" s="4" t="n"/>
+      <c r="AD80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="T81" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U81" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V81" s="7" t="n">
+        <v>698</v>
+      </c>
+      <c r="X81" s="7" t="n"/>
+      <c r="Y81" s="7" t="n"/>
+      <c r="Z81" s="7" t="n"/>
+      <c r="AB81" s="7" t="n"/>
+      <c r="AC81" s="7" t="n"/>
+      <c r="AD81" s="7" t="n"/>
+    </row>
+    <row r="82">
+      <c r="T82" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U82" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V82" s="4" t="n">
+        <v>687</v>
+      </c>
+      <c r="X82" s="4" t="n"/>
+      <c r="Y82" s="4" t="n"/>
+      <c r="Z82" s="4" t="n"/>
+      <c r="AB82" s="4" t="n"/>
+      <c r="AC82" s="4" t="n"/>
+      <c r="AD82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="T83" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U83" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V83" s="7" t="n">
+        <v>716</v>
+      </c>
+      <c r="X83" s="7" t="n"/>
+      <c r="Y83" s="7" t="n"/>
+      <c r="Z83" s="7" t="n"/>
+      <c r="AB83" s="7" t="n"/>
+      <c r="AC83" s="7" t="n"/>
+      <c r="AD83" s="7" t="n"/>
+    </row>
+    <row r="84">
+      <c r="T84" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U84" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V84" s="4" t="n">
+        <v>719</v>
+      </c>
+      <c r="X84" s="4" t="n"/>
+      <c r="Y84" s="4" t="n"/>
+      <c r="Z84" s="4" t="n"/>
+      <c r="AB84" s="4" t="n"/>
+      <c r="AC84" s="4" t="n"/>
+      <c r="AD84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="T85" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U85" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V85" s="7" t="n">
+        <v>724</v>
+      </c>
+      <c r="X85" s="7" t="n"/>
+      <c r="Y85" s="7" t="n"/>
+      <c r="Z85" s="7" t="n"/>
+      <c r="AB85" s="7" t="n"/>
+      <c r="AC85" s="7" t="n"/>
+      <c r="AD85" s="7" t="n"/>
+    </row>
+    <row r="86">
+      <c r="T86" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U86" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V86" s="4" t="n">
+        <v>2290</v>
+      </c>
+      <c r="X86" s="4" t="n"/>
+      <c r="Y86" s="4" t="n"/>
+      <c r="Z86" s="4" t="n"/>
+      <c r="AB86" s="4" t="n"/>
+      <c r="AC86" s="4" t="n"/>
+      <c r="AD86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="T87" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U87" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V87" s="7" t="n">
+        <v>2092</v>
+      </c>
+      <c r="X87" s="7" t="n"/>
+      <c r="Y87" s="7" t="n"/>
+      <c r="Z87" s="7" t="n"/>
+      <c r="AB87" s="7" t="n"/>
+      <c r="AC87" s="7" t="n"/>
+      <c r="AD87" s="7" t="n"/>
+    </row>
+    <row r="88">
+      <c r="T88" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U88" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V88" s="4" t="n">
+        <v>2043</v>
+      </c>
+      <c r="X88" s="4" t="n"/>
+      <c r="Y88" s="4" t="n"/>
+      <c r="Z88" s="4" t="n"/>
+      <c r="AB88" s="4" t="n"/>
+      <c r="AC88" s="4" t="n"/>
+      <c r="AD88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="T89" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U89" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V89" s="7" t="n">
+        <v>1969</v>
+      </c>
+      <c r="X89" s="7" t="n"/>
+      <c r="Y89" s="7" t="n"/>
+      <c r="Z89" s="7" t="n"/>
+      <c r="AB89" s="7" t="n"/>
+      <c r="AC89" s="7" t="n"/>
+      <c r="AD89" s="7" t="n"/>
+    </row>
+    <row r="90">
+      <c r="T90" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U90" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V90" s="4" t="n">
+        <v>1938</v>
+      </c>
+      <c r="X90" s="4" t="n"/>
+      <c r="Y90" s="4" t="n"/>
+      <c r="Z90" s="4" t="n"/>
+      <c r="AB90" s="4" t="n"/>
+      <c r="AC90" s="4" t="n"/>
+      <c r="AD90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="T91" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U91" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V91" s="7" t="n">
+        <v>2048</v>
+      </c>
+      <c r="X91" s="7" t="n"/>
+      <c r="Y91" s="7" t="n"/>
+      <c r="Z91" s="7" t="n"/>
+      <c r="AB91" s="7" t="n"/>
+      <c r="AC91" s="7" t="n"/>
+      <c r="AD91" s="7" t="n"/>
+    </row>
+    <row r="92">
+      <c r="T92" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U92" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V92" s="4" t="n">
+        <v>2033</v>
+      </c>
+      <c r="X92" s="4" t="n"/>
+      <c r="Y92" s="4" t="n"/>
+      <c r="Z92" s="4" t="n"/>
+      <c r="AB92" s="4" t="n"/>
+      <c r="AC92" s="4" t="n"/>
+      <c r="AD92" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Added 4.2828.3 release, as peya has release 4.2828.3
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -716,7 +716,7 @@
         <v>0.84</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>1.31</v>
@@ -752,7 +752,7 @@
         <v>0.84</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>1.31</v>
@@ -788,7 +788,7 @@
         <v>0.84</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>1.31</v>
@@ -824,7 +824,7 @@
         <v>0.84</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>1.31</v>
@@ -860,7 +860,7 @@
         <v>0.84</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>1.31</v>
@@ -896,7 +896,7 @@
         <v>0.84</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>1.31</v>
@@ -932,7 +932,7 @@
         <v>0.84</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>1.31</v>
@@ -968,7 +968,7 @@
         <v>0.84</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>1.31</v>
@@ -1004,7 +1004,7 @@
         <v>0.84</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>1.31</v>
@@ -1040,7 +1040,7 @@
         <v>0.84</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>1.31</v>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD92"/>
+  <dimension ref="A1:AD105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1892,29 +1892,49 @@
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="D9" s="7">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C9)</f>
+        <v/>
+      </c>
       <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="G9" s="7">
+        <f>ROUND(MAX(0,MIN(100,(1-E9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7">
+        <f>MIN(1,(G9-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
+      <c r="K9" s="7">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>MAX(0,(L9-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="7">
+        <f>$B$2+H9+M9</f>
+        <v/>
+      </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="U9" s="7" t="inlineStr"/>
       <c r="V9" s="7" t="n">
-        <v>5504</v>
+        <v>1</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>3</v>
@@ -1972,7 +1992,7 @@
       <c r="N10" s="4" t="n"/>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1981,7 +2001,7 @@
         </is>
       </c>
       <c r="V10" s="4" t="n">
-        <v>5352</v>
+        <v>5504</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>117</v>
@@ -2031,7 +2051,7 @@
       <c r="N11" s="7" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -2040,7 +2060,7 @@
         </is>
       </c>
       <c r="V11" s="7" t="n">
-        <v>5324</v>
+        <v>5352</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>18</v>
@@ -2090,7 +2110,7 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -2099,7 +2119,7 @@
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5091</v>
+        <v>5324</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>71</v>
@@ -2149,7 +2169,7 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>4961</v>
+        <v>5091</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>26</v>
@@ -2208,7 +2228,7 @@
       <c r="N14" s="4" t="n"/>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -2217,7 +2237,7 @@
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>5646</v>
+        <v>4961</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>20</v>
@@ -2267,7 +2287,7 @@
       <c r="N15" s="7" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
@@ -2276,7 +2296,7 @@
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>5436</v>
+        <v>5646</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>81</v>
@@ -2326,16 +2346,16 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>15599</v>
+        <v>5436</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>11</v>
@@ -2385,16 +2405,16 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>14943</v>
+        <v>5678</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>3</v>
@@ -2444,7 +2464,7 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
@@ -2453,7 +2473,7 @@
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>14930</v>
+        <v>15599</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>139</v>
@@ -2503,7 +2523,7 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
@@ -2512,7 +2532,7 @@
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>14111</v>
+        <v>14943</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>14</v>
@@ -2562,7 +2582,7 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2571,7 +2591,7 @@
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>14130</v>
+        <v>14930</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>68</v>
@@ -2621,7 +2641,7 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
@@ -2630,7 +2650,7 @@
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>14512</v>
+        <v>14111</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>28</v>
@@ -2680,7 +2700,7 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2689,7 +2709,7 @@
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>14749</v>
+        <v>14130</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>17</v>
@@ -2739,16 +2759,16 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>82921</v>
+        <v>14512</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>106</v>
@@ -2798,16 +2818,16 @@
       <c r="N24" s="4" t="n"/>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>80613</v>
+        <v>14749</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2857,16 +2877,16 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>82716</v>
+        <v>15293</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>9</v>
@@ -2916,7 +2936,7 @@
       <c r="N26" s="4" t="n"/>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
@@ -2925,7 +2945,7 @@
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>79024</v>
+        <v>82921</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>3</v>
@@ -2975,7 +2995,7 @@
       <c r="N27" s="7" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
@@ -2984,7 +3004,7 @@
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>79116</v>
+        <v>80613</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>145</v>
@@ -3034,7 +3054,7 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
@@ -3043,7 +3063,7 @@
         </is>
       </c>
       <c r="V28" s="4" t="n">
-        <v>80620</v>
+        <v>82716</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>20</v>
@@ -3093,7 +3113,7 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
@@ -3102,7 +3122,7 @@
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>80878</v>
+        <v>79024</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>73</v>
@@ -3152,16 +3172,16 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>756</v>
+        <v>79116</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>31</v>
@@ -3211,16 +3231,16 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>708</v>
+        <v>80620</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>16</v>
@@ -3270,16 +3290,16 @@
       <c r="N32" s="4" t="n"/>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>733</v>
+        <v>80878</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>108</v>
@@ -3338,16 +3358,16 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>662</v>
+        <v>81522</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>13</v>
@@ -3378,7 +3398,7 @@
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D8)</f>
+        <f>AVERAGE(D2:D9)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3388,7 +3408,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H8)</f>
+        <f>AVERAGE(H2:H9)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3411,7 +3431,7 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -3420,7 +3440,7 @@
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>678</v>
+        <v>756</v>
       </c>
       <c r="X34" s="4" t="n">
         <v>2</v>
@@ -3452,7 +3472,7 @@
     <row r="35">
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
@@ -3461,7 +3481,7 @@
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>105</v>
@@ -3493,7 +3513,7 @@
     <row r="36">
       <c r="T36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -3502,7 +3522,7 @@
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>683</v>
+        <v>733</v>
       </c>
       <c r="X36" s="4" t="n">
         <v>18</v>
@@ -3534,16 +3554,16 @@
     <row r="37">
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>48266</v>
+        <v>662</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>54</v>
@@ -3575,16 +3595,16 @@
     <row r="38">
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>50405</v>
+        <v>678</v>
       </c>
       <c r="X38" s="4" t="n">
         <v>27</v>
@@ -3616,16 +3636,16 @@
     <row r="39">
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
-        <v>48886</v>
+        <v>700</v>
       </c>
       <c r="X39" s="7" t="n">
         <v>13</v>
@@ -3657,16 +3677,16 @@
     <row r="40">
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>47253</v>
+        <v>683</v>
       </c>
       <c r="X40" s="4" t="n">
         <v>89</v>
@@ -3698,16 +3718,16 @@
     <row r="41">
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V41" s="7" t="n">
-        <v>46972</v>
+        <v>720</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>1</v>
@@ -3739,7 +3759,7 @@
     <row r="42">
       <c r="T42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
@@ -3748,7 +3768,7 @@
         </is>
       </c>
       <c r="V42" s="4" t="n">
-        <v>48667</v>
+        <v>48266</v>
       </c>
       <c r="X42" s="4" t="n">
         <v>9</v>
@@ -3780,7 +3800,7 @@
     <row r="43">
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
@@ -3789,7 +3809,7 @@
         </is>
       </c>
       <c r="V43" s="7" t="n">
-        <v>48109</v>
+        <v>50405</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>1</v>
@@ -3821,16 +3841,16 @@
     <row r="44">
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V44" s="4" t="n">
-        <v>1</v>
+        <v>48886</v>
       </c>
       <c r="X44" s="4" t="n">
         <v>135</v>
@@ -3862,16 +3882,16 @@
     <row r="45">
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V45" s="7" t="n">
-        <v>1</v>
+        <v>47253</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>8</v>
@@ -3903,16 +3923,16 @@
     <row r="46">
       <c r="T46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U46" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V46" s="4" t="n">
-        <v>1</v>
+        <v>46972</v>
       </c>
       <c r="X46" s="4" t="n">
         <v>60</v>
@@ -3944,16 +3964,16 @@
     <row r="47">
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V47" s="7" t="n">
-        <v>1</v>
+        <v>48667</v>
       </c>
       <c r="X47" s="7" t="n">
         <v>19</v>
@@ -3985,16 +4005,16 @@
     <row r="48">
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U48" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V48" s="4" t="n">
-        <v>1</v>
+        <v>48109</v>
       </c>
       <c r="X48" s="4" t="n">
         <v>20</v>
@@ -4026,16 +4046,16 @@
     <row r="49">
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V49" s="7" t="n">
-        <v>1</v>
+        <v>48852</v>
       </c>
       <c r="X49" s="7" t="n">
         <v>115</v>
@@ -4067,7 +4087,7 @@
     <row r="50">
       <c r="T50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr">
@@ -4108,12 +4128,12 @@
     <row r="51">
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V51" s="7" t="n">
@@ -4149,12 +4169,12 @@
     <row r="52">
       <c r="T52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V52" s="4" t="n">
@@ -4190,12 +4210,12 @@
     <row r="53">
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V53" s="7" t="n">
@@ -4231,12 +4251,12 @@
     <row r="54">
       <c r="T54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V54" s="4" t="n">
@@ -4272,12 +4292,12 @@
     <row r="55">
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V55" s="7" t="n">
@@ -4313,12 +4333,12 @@
     <row r="56">
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V56" s="4" t="n">
@@ -4354,12 +4374,12 @@
     <row r="57">
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V57" s="7" t="n">
@@ -4400,11 +4420,11 @@
       </c>
       <c r="U58" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V58" s="4" t="n">
-        <v>10655</v>
+        <v>1</v>
       </c>
       <c r="X58" s="4" t="n">
         <v>8</v>
@@ -4441,15 +4461,25 @@
       </c>
       <c r="U59" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V59" s="7" t="n">
-        <v>10413</v>
-      </c>
-      <c r="X59" s="7" t="n"/>
-      <c r="Y59" s="7" t="n"/>
-      <c r="Z59" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X59" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y59" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z59" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB59" s="7" t="n">
         <v>56</v>
       </c>
@@ -4472,15 +4502,25 @@
       </c>
       <c r="U60" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V60" s="4" t="n">
-        <v>10036</v>
-      </c>
-      <c r="X60" s="4" t="n"/>
-      <c r="Y60" s="4" t="n"/>
-      <c r="Z60" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X60" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y60" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z60" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB60" s="4" t="n">
         <v>41</v>
       </c>
@@ -4503,15 +4543,25 @@
       </c>
       <c r="U61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V61" s="7" t="n">
-        <v>9869</v>
-      </c>
-      <c r="X61" s="7" t="n"/>
-      <c r="Y61" s="7" t="n"/>
-      <c r="Z61" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X61" s="7" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y61" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z61" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB61" s="7" t="n">
         <v>152</v>
       </c>
@@ -4534,15 +4584,25 @@
       </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V62" s="4" t="n">
-        <v>10072</v>
-      </c>
-      <c r="X62" s="4" t="n"/>
-      <c r="Y62" s="4" t="n"/>
-      <c r="Z62" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X62" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="Y62" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z62" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB62" s="4" t="n">
         <v>3</v>
       </c>
@@ -4565,15 +4625,25 @@
       </c>
       <c r="U63" s="7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V63" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X63" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y63" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z63" s="7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
-      <c r="V63" s="7" t="n">
-        <v>10125</v>
-      </c>
-      <c r="X63" s="7" t="n"/>
-      <c r="Y63" s="7" t="n"/>
-      <c r="Z63" s="7" t="n"/>
       <c r="AB63" s="7" t="n">
         <v>7</v>
       </c>
@@ -4596,15 +4666,25 @@
       </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V64" s="4" t="n">
-        <v>10161</v>
-      </c>
-      <c r="X64" s="4" t="n"/>
-      <c r="Y64" s="4" t="n"/>
-      <c r="Z64" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X64" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="Y64" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z64" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB64" s="4" t="n">
         <v>3</v>
       </c>
@@ -4622,205 +4702,325 @@
     <row r="65">
       <c r="T65" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V65" s="7" t="n">
-        <v>23063</v>
-      </c>
-      <c r="X65" s="7" t="n"/>
-      <c r="Y65" s="7" t="n"/>
-      <c r="Z65" s="7" t="n"/>
-      <c r="AB65" s="7" t="n"/>
-      <c r="AC65" s="7" t="n"/>
-      <c r="AD65" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X65" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y65" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z65" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="AB65" s="7" t="n">
+        <v>362</v>
+      </c>
+      <c r="AC65" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD65" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="T66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V66" s="4" t="n">
-        <v>23168</v>
-      </c>
-      <c r="X66" s="4" t="n"/>
-      <c r="Y66" s="4" t="n"/>
-      <c r="Z66" s="4" t="n"/>
-      <c r="AB66" s="4" t="n"/>
-      <c r="AC66" s="4" t="n"/>
-      <c r="AD66" s="4" t="n"/>
+        <v>10655</v>
+      </c>
+      <c r="X66" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y66" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z66" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB66" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="AC66" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD66" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="T67" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U67" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V67" s="7" t="n">
-        <v>24394</v>
-      </c>
-      <c r="X67" s="7" t="n"/>
-      <c r="Y67" s="7" t="n"/>
-      <c r="Z67" s="7" t="n"/>
-      <c r="AB67" s="7" t="n"/>
-      <c r="AC67" s="7" t="n"/>
-      <c r="AD67" s="7" t="n"/>
+        <v>10413</v>
+      </c>
+      <c r="X67" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y67" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="Z67" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="AB67" s="7" t="n">
+        <v>188</v>
+      </c>
+      <c r="AC67" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD67" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="T68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U68" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V68" s="4" t="n">
-        <v>21980</v>
+        <v>10036</v>
       </c>
       <c r="X68" s="4" t="n"/>
       <c r="Y68" s="4" t="n"/>
       <c r="Z68" s="4" t="n"/>
-      <c r="AB68" s="4" t="n"/>
-      <c r="AC68" s="4" t="n"/>
-      <c r="AD68" s="4" t="n"/>
+      <c r="AB68" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AC68" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD68" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="T69" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U69" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V69" s="7" t="n">
-        <v>21517</v>
+        <v>9869</v>
       </c>
       <c r="X69" s="7" t="n"/>
       <c r="Y69" s="7" t="n"/>
       <c r="Z69" s="7" t="n"/>
-      <c r="AB69" s="7" t="n"/>
-      <c r="AC69" s="7" t="n"/>
-      <c r="AD69" s="7" t="n"/>
+      <c r="AB69" s="7" t="n">
+        <v>47</v>
+      </c>
+      <c r="AC69" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD69" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U70" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V70" s="4" t="n">
-        <v>22785</v>
+        <v>10072</v>
       </c>
       <c r="X70" s="4" t="n"/>
       <c r="Y70" s="4" t="n"/>
       <c r="Z70" s="4" t="n"/>
-      <c r="AB70" s="4" t="n"/>
-      <c r="AC70" s="4" t="n"/>
-      <c r="AD70" s="4" t="n"/>
+      <c r="AB70" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="AC70" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD70" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="T71" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U71" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V71" s="7" t="n">
-        <v>24108</v>
+        <v>10125</v>
       </c>
       <c r="X71" s="7" t="n"/>
       <c r="Y71" s="7" t="n"/>
       <c r="Z71" s="7" t="n"/>
-      <c r="AB71" s="7" t="n"/>
-      <c r="AC71" s="7" t="n"/>
-      <c r="AD71" s="7" t="n"/>
+      <c r="AB71" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC71" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD71" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U72" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V72" s="4" t="n">
-        <v>17887</v>
+        <v>10161</v>
       </c>
       <c r="X72" s="4" t="n"/>
       <c r="Y72" s="4" t="n"/>
       <c r="Z72" s="4" t="n"/>
-      <c r="AB72" s="4" t="n"/>
-      <c r="AC72" s="4" t="n"/>
-      <c r="AD72" s="4" t="n"/>
+      <c r="AB72" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC72" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD72" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="T73" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U73" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V73" s="7" t="n">
-        <v>17641</v>
+        <v>10341</v>
       </c>
       <c r="X73" s="7" t="n"/>
       <c r="Y73" s="7" t="n"/>
       <c r="Z73" s="7" t="n"/>
-      <c r="AB73" s="7" t="n"/>
-      <c r="AC73" s="7" t="n"/>
-      <c r="AD73" s="7" t="n"/>
+      <c r="AB73" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC73" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="AD73" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="T74" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U74" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V74" s="4" t="n">
-        <v>17144</v>
+        <v>23063</v>
       </c>
       <c r="X74" s="4" t="n"/>
       <c r="Y74" s="4" t="n"/>
@@ -4832,16 +5032,16 @@
     <row r="75">
       <c r="T75" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U75" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V75" s="7" t="n">
-        <v>17159</v>
+        <v>23168</v>
       </c>
       <c r="X75" s="7" t="n"/>
       <c r="Y75" s="7" t="n"/>
@@ -4853,16 +5053,16 @@
     <row r="76">
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V76" s="4" t="n">
-        <v>17724</v>
+        <v>24394</v>
       </c>
       <c r="X76" s="4" t="n"/>
       <c r="Y76" s="4" t="n"/>
@@ -4874,16 +5074,16 @@
     <row r="77">
       <c r="T77" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V77" s="7" t="n">
-        <v>17829</v>
+        <v>21980</v>
       </c>
       <c r="X77" s="7" t="n"/>
       <c r="Y77" s="7" t="n"/>
@@ -4895,16 +5095,16 @@
     <row r="78">
       <c r="T78" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U78" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V78" s="4" t="n">
-        <v>18088</v>
+        <v>21517</v>
       </c>
       <c r="X78" s="4" t="n"/>
       <c r="Y78" s="4" t="n"/>
@@ -4916,16 +5116,16 @@
     <row r="79">
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U79" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V79" s="7" t="n">
-        <v>700</v>
+        <v>22785</v>
       </c>
       <c r="X79" s="7" t="n"/>
       <c r="Y79" s="7" t="n"/>
@@ -4937,16 +5137,16 @@
     <row r="80">
       <c r="T80" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U80" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V80" s="4" t="n">
-        <v>686</v>
+        <v>24108</v>
       </c>
       <c r="X80" s="4" t="n"/>
       <c r="Y80" s="4" t="n"/>
@@ -4958,16 +5158,16 @@
     <row r="81">
       <c r="T81" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U81" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V81" s="7" t="n">
-        <v>698</v>
+        <v>23330</v>
       </c>
       <c r="X81" s="7" t="n"/>
       <c r="Y81" s="7" t="n"/>
@@ -4979,16 +5179,16 @@
     <row r="82">
       <c r="T82" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U82" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V82" s="4" t="n">
-        <v>687</v>
+        <v>17887</v>
       </c>
       <c r="X82" s="4" t="n"/>
       <c r="Y82" s="4" t="n"/>
@@ -5000,16 +5200,16 @@
     <row r="83">
       <c r="T83" s="7" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U83" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V83" s="7" t="n">
-        <v>716</v>
+        <v>17641</v>
       </c>
       <c r="X83" s="7" t="n"/>
       <c r="Y83" s="7" t="n"/>
@@ -5021,16 +5221,16 @@
     <row r="84">
       <c r="T84" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U84" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V84" s="4" t="n">
-        <v>719</v>
+        <v>17144</v>
       </c>
       <c r="X84" s="4" t="n"/>
       <c r="Y84" s="4" t="n"/>
@@ -5042,16 +5242,16 @@
     <row r="85">
       <c r="T85" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U85" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V85" s="7" t="n">
-        <v>724</v>
+        <v>17159</v>
       </c>
       <c r="X85" s="7" t="n"/>
       <c r="Y85" s="7" t="n"/>
@@ -5063,16 +5263,16 @@
     <row r="86">
       <c r="T86" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U86" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V86" s="4" t="n">
-        <v>2290</v>
+        <v>17724</v>
       </c>
       <c r="X86" s="4" t="n"/>
       <c r="Y86" s="4" t="n"/>
@@ -5084,16 +5284,16 @@
     <row r="87">
       <c r="T87" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U87" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V87" s="7" t="n">
-        <v>2092</v>
+        <v>17829</v>
       </c>
       <c r="X87" s="7" t="n"/>
       <c r="Y87" s="7" t="n"/>
@@ -5105,16 +5305,16 @@
     <row r="88">
       <c r="T88" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U88" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V88" s="4" t="n">
-        <v>2043</v>
+        <v>18088</v>
       </c>
       <c r="X88" s="4" t="n"/>
       <c r="Y88" s="4" t="n"/>
@@ -5126,16 +5326,16 @@
     <row r="89">
       <c r="T89" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U89" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V89" s="7" t="n">
-        <v>1969</v>
+        <v>17869</v>
       </c>
       <c r="X89" s="7" t="n"/>
       <c r="Y89" s="7" t="n"/>
@@ -5147,16 +5347,16 @@
     <row r="90">
       <c r="T90" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U90" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V90" s="4" t="n">
-        <v>1938</v>
+        <v>700</v>
       </c>
       <c r="X90" s="4" t="n"/>
       <c r="Y90" s="4" t="n"/>
@@ -5168,16 +5368,16 @@
     <row r="91">
       <c r="T91" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U91" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V91" s="7" t="n">
-        <v>2048</v>
+        <v>686</v>
       </c>
       <c r="X91" s="7" t="n"/>
       <c r="Y91" s="7" t="n"/>
@@ -5189,16 +5389,16 @@
     <row r="92">
       <c r="T92" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U92" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V92" s="4" t="n">
-        <v>2033</v>
+        <v>698</v>
       </c>
       <c r="X92" s="4" t="n"/>
       <c r="Y92" s="4" t="n"/>
@@ -5206,6 +5406,279 @@
       <c r="AB92" s="4" t="n"/>
       <c r="AC92" s="4" t="n"/>
       <c r="AD92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="T93" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U93" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V93" s="7" t="n">
+        <v>687</v>
+      </c>
+      <c r="X93" s="7" t="n"/>
+      <c r="Y93" s="7" t="n"/>
+      <c r="Z93" s="7" t="n"/>
+      <c r="AB93" s="7" t="n"/>
+      <c r="AC93" s="7" t="n"/>
+      <c r="AD93" s="7" t="n"/>
+    </row>
+    <row r="94">
+      <c r="T94" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U94" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V94" s="4" t="n">
+        <v>716</v>
+      </c>
+      <c r="X94" s="4" t="n"/>
+      <c r="Y94" s="4" t="n"/>
+      <c r="Z94" s="4" t="n"/>
+      <c r="AB94" s="4" t="n"/>
+      <c r="AC94" s="4" t="n"/>
+      <c r="AD94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="T95" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U95" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V95" s="7" t="n">
+        <v>719</v>
+      </c>
+      <c r="X95" s="7" t="n"/>
+      <c r="Y95" s="7" t="n"/>
+      <c r="Z95" s="7" t="n"/>
+      <c r="AB95" s="7" t="n"/>
+      <c r="AC95" s="7" t="n"/>
+      <c r="AD95" s="7" t="n"/>
+    </row>
+    <row r="96">
+      <c r="T96" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U96" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V96" s="4" t="n">
+        <v>724</v>
+      </c>
+      <c r="X96" s="4" t="n"/>
+      <c r="Y96" s="4" t="n"/>
+      <c r="Z96" s="4" t="n"/>
+      <c r="AB96" s="4" t="n"/>
+      <c r="AC96" s="4" t="n"/>
+      <c r="AD96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="T97" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="U97" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V97" s="7" t="n">
+        <v>701</v>
+      </c>
+      <c r="X97" s="7" t="n"/>
+      <c r="Y97" s="7" t="n"/>
+      <c r="Z97" s="7" t="n"/>
+      <c r="AB97" s="7" t="n"/>
+      <c r="AC97" s="7" t="n"/>
+      <c r="AD97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="T98" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U98" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V98" s="4" t="n">
+        <v>2290</v>
+      </c>
+      <c r="X98" s="4" t="n"/>
+      <c r="Y98" s="4" t="n"/>
+      <c r="Z98" s="4" t="n"/>
+      <c r="AB98" s="4" t="n"/>
+      <c r="AC98" s="4" t="n"/>
+      <c r="AD98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="T99" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U99" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V99" s="7" t="n">
+        <v>2092</v>
+      </c>
+      <c r="X99" s="7" t="n"/>
+      <c r="Y99" s="7" t="n"/>
+      <c r="Z99" s="7" t="n"/>
+      <c r="AB99" s="7" t="n"/>
+      <c r="AC99" s="7" t="n"/>
+      <c r="AD99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="T100" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U100" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V100" s="4" t="n">
+        <v>2043</v>
+      </c>
+      <c r="X100" s="4" t="n"/>
+      <c r="Y100" s="4" t="n"/>
+      <c r="Z100" s="4" t="n"/>
+      <c r="AB100" s="4" t="n"/>
+      <c r="AC100" s="4" t="n"/>
+      <c r="AD100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="T101" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U101" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V101" s="7" t="n">
+        <v>1969</v>
+      </c>
+      <c r="X101" s="7" t="n"/>
+      <c r="Y101" s="7" t="n"/>
+      <c r="Z101" s="7" t="n"/>
+      <c r="AB101" s="7" t="n"/>
+      <c r="AC101" s="7" t="n"/>
+      <c r="AD101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="T102" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U102" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V102" s="4" t="n">
+        <v>1938</v>
+      </c>
+      <c r="X102" s="4" t="n"/>
+      <c r="Y102" s="4" t="n"/>
+      <c r="Z102" s="4" t="n"/>
+      <c r="AB102" s="4" t="n"/>
+      <c r="AC102" s="4" t="n"/>
+      <c r="AD102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="T103" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U103" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V103" s="7" t="n">
+        <v>2048</v>
+      </c>
+      <c r="X103" s="7" t="n"/>
+      <c r="Y103" s="7" t="n"/>
+      <c r="Z103" s="7" t="n"/>
+      <c r="AB103" s="7" t="n"/>
+      <c r="AC103" s="7" t="n"/>
+      <c r="AD103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="T104" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U104" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V104" s="4" t="n">
+        <v>2033</v>
+      </c>
+      <c r="X104" s="4" t="n"/>
+      <c r="Y104" s="4" t="n"/>
+      <c r="Z104" s="4" t="n"/>
+      <c r="AB104" s="4" t="n"/>
+      <c r="AC104" s="4" t="n"/>
+      <c r="AD104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="T105" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="U105" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V105" s="7" t="n">
+        <v>2242</v>
+      </c>
+      <c r="X105" s="7" t="n"/>
+      <c r="Y105" s="7" t="n"/>
+      <c r="Z105" s="7" t="n"/>
+      <c r="AB105" s="7" t="n"/>
+      <c r="AC105" s="7" t="n"/>
+      <c r="AD105" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Fixed auto generate issue and updated ASTI and TTI numbers for July
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -710,16 +710,16 @@
         <v>77.5</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>78203</v>
@@ -746,16 +746,16 @@
         <v>80.7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14946</v>
@@ -782,16 +782,16 @@
         <v>77.59999999999999</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>16988</v>
@@ -818,16 +818,16 @@
         <v>67.8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>20641</v>
@@ -854,16 +854,16 @@
         <v>77.59999999999999</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>10630</v>
@@ -890,16 +890,16 @@
         <v>77.5</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>2186</v>
@@ -926,16 +926,16 @@
         <v>77.5</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>46896</v>
@@ -962,16 +962,16 @@
         <v>77.2</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>731</v>
@@ -998,16 +998,16 @@
         <v>67.7</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5258</v>
@@ -1034,16 +1034,16 @@
         <v>67.7</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4.47</v>
+        <v>4.54</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.84</v>
+        <v>1.18</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>729</v>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD157"/>
+  <dimension ref="A1:AD170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2295,29 +2295,49 @@
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
+      <c r="D14" s="4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C14)</f>
+        <v/>
+      </c>
       <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
+      <c r="G14" s="4">
+        <f>ROUND(MAX(0,MIN(100,(1-E14/IF(D14&gt;0,D14,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>MIN(1,(G14-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="n"/>
-      <c r="N14" s="4" t="n"/>
+      <c r="K14" s="4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K14/IF(D14&gt;0,D14,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M14" s="4">
+        <f>MAX(0,(L14-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N14" s="4">
+        <f>$B$2+H14+M14</f>
+        <v/>
+      </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="U14" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr"/>
       <c r="V14" s="4" t="n">
-        <v>5504</v>
+        <v>1</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>15</v>
@@ -2367,7 +2387,7 @@
       <c r="N15" s="7" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
@@ -2376,7 +2396,7 @@
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>5352</v>
+        <v>5504</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>57</v>
@@ -2426,7 +2446,7 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
@@ -2435,7 +2455,7 @@
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>5324</v>
+        <v>5352</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>11</v>
@@ -2485,7 +2505,7 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>5091</v>
+        <v>5324</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>3</v>
@@ -2544,7 +2564,7 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
@@ -2553,7 +2573,7 @@
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>4961</v>
+        <v>5091</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>109</v>
@@ -2603,7 +2623,7 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
@@ -2612,7 +2632,7 @@
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>5646</v>
+        <v>4961</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>13</v>
@@ -2662,7 +2682,7 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
@@ -2671,7 +2691,7 @@
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>5436</v>
+        <v>5646</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>52</v>
@@ -2721,7 +2741,7 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
@@ -2730,7 +2750,7 @@
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>5678</v>
+        <v>5436</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>20</v>
@@ -2780,7 +2800,7 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
@@ -2789,7 +2809,7 @@
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>5512</v>
+        <v>5678</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>16</v>
@@ -2839,7 +2859,7 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
@@ -2848,7 +2868,7 @@
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>5450</v>
+        <v>5512</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>73</v>
@@ -2898,7 +2918,7 @@
       <c r="N24" s="4" t="n"/>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -2907,7 +2927,7 @@
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>5116</v>
+        <v>5450</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2957,7 +2977,7 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
@@ -2966,7 +2986,7 @@
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>5004</v>
+        <v>5116</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>9</v>
@@ -3016,16 +3036,16 @@
       <c r="N26" s="4" t="n"/>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>15599</v>
+        <v>5004</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>3</v>
@@ -3075,16 +3095,16 @@
       <c r="N27" s="7" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>14943</v>
+        <v>5765</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>118</v>
@@ -3134,7 +3154,7 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
@@ -3143,7 +3163,7 @@
         </is>
       </c>
       <c r="V28" s="4" t="n">
-        <v>14930</v>
+        <v>15599</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>18</v>
@@ -3193,7 +3213,7 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
@@ -3202,7 +3222,7 @@
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>14111</v>
+        <v>14943</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>59</v>
@@ -3252,7 +3272,7 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3261,7 +3281,7 @@
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>14130</v>
+        <v>14930</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>25</v>
@@ -3311,7 +3331,7 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
@@ -3320,7 +3340,7 @@
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>14512</v>
+        <v>14111</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>14</v>
@@ -3370,7 +3390,7 @@
       <c r="N32" s="4" t="n"/>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -3379,7 +3399,7 @@
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>14749</v>
+        <v>14130</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>76</v>
@@ -3438,7 +3458,7 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
@@ -3447,7 +3467,7 @@
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>15293</v>
+        <v>14512</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>13</v>
@@ -3478,7 +3498,7 @@
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D13)</f>
+        <f>AVERAGE(D2:D14)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3488,7 +3508,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H13)</f>
+        <f>AVERAGE(H2:H14)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3511,7 +3531,7 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -3520,7 +3540,7 @@
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>14634</v>
+        <v>14749</v>
       </c>
       <c r="X34" s="4" t="n">
         <v>2</v>
@@ -3552,7 +3572,7 @@
     <row r="35">
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
@@ -3561,7 +3581,7 @@
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>14782</v>
+        <v>15293</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>74</v>
@@ -3593,7 +3613,7 @@
     <row r="36">
       <c r="T36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
@@ -3602,7 +3622,7 @@
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>14108</v>
+        <v>14634</v>
       </c>
       <c r="X36" s="4" t="n">
         <v>18</v>
@@ -3634,7 +3654,7 @@
     <row r="37">
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
@@ -3643,7 +3663,7 @@
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>13970</v>
+        <v>14782</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>44</v>
@@ -3675,16 +3695,16 @@
     <row r="38">
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>82921</v>
+        <v>14108</v>
       </c>
       <c r="X38" s="4" t="n">
         <v>23</v>
@@ -3716,16 +3736,16 @@
     <row r="39">
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
-        <v>80613</v>
+        <v>13970</v>
       </c>
       <c r="X39" s="7" t="n">
         <v>10</v>
@@ -3757,16 +3777,16 @@
     <row r="40">
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>82716</v>
+        <v>14738</v>
       </c>
       <c r="X40" s="4" t="n">
         <v>69</v>
@@ -3798,7 +3818,7 @@
     <row r="41">
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
@@ -3807,7 +3827,7 @@
         </is>
       </c>
       <c r="V41" s="7" t="n">
-        <v>79024</v>
+        <v>82921</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>1</v>
@@ -3839,7 +3859,7 @@
     <row r="42">
       <c r="T42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
@@ -3848,7 +3868,7 @@
         </is>
       </c>
       <c r="V42" s="4" t="n">
-        <v>79116</v>
+        <v>80613</v>
       </c>
       <c r="X42" s="4" t="n">
         <v>9</v>
@@ -3880,7 +3900,7 @@
     <row r="43">
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
@@ -3889,7 +3909,7 @@
         </is>
       </c>
       <c r="V43" s="7" t="n">
-        <v>80620</v>
+        <v>82716</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>113</v>
@@ -3921,7 +3941,7 @@
     <row r="44">
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr">
@@ -3930,7 +3950,7 @@
         </is>
       </c>
       <c r="V44" s="4" t="n">
-        <v>80878</v>
+        <v>79024</v>
       </c>
       <c r="X44" s="4" t="n">
         <v>5</v>
@@ -3962,7 +3982,7 @@
     <row r="45">
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
@@ -3971,7 +3991,7 @@
         </is>
       </c>
       <c r="V45" s="7" t="n">
-        <v>81522</v>
+        <v>79116</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>48</v>
@@ -4003,7 +4023,7 @@
     <row r="46">
       <c r="T46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U46" s="4" t="inlineStr">
@@ -4012,7 +4032,7 @@
         </is>
       </c>
       <c r="V46" s="4" t="n">
-        <v>81556</v>
+        <v>80620</v>
       </c>
       <c r="X46" s="4" t="n">
         <v>19</v>
@@ -4044,7 +4064,7 @@
     <row r="47">
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
@@ -4053,7 +4073,7 @@
         </is>
       </c>
       <c r="V47" s="7" t="n">
-        <v>78444</v>
+        <v>80878</v>
       </c>
       <c r="X47" s="7" t="n">
         <v>18</v>
@@ -4085,7 +4105,7 @@
     <row r="48">
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U48" s="4" t="inlineStr">
@@ -4094,7 +4114,7 @@
         </is>
       </c>
       <c r="V48" s="4" t="n">
-        <v>73979</v>
+        <v>81522</v>
       </c>
       <c r="X48" s="4" t="n">
         <v>86</v>
@@ -4126,7 +4146,7 @@
     <row r="49">
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
@@ -4135,7 +4155,7 @@
         </is>
       </c>
       <c r="V49" s="7" t="n">
-        <v>77997</v>
+        <v>81556</v>
       </c>
       <c r="X49" s="7" t="n">
         <v>3</v>
@@ -4167,16 +4187,16 @@
     <row r="50">
       <c r="T50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V50" s="4" t="n">
-        <v>756</v>
+        <v>78444</v>
       </c>
       <c r="X50" s="4" t="n">
         <v>102</v>
@@ -4208,16 +4228,16 @@
     <row r="51">
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V51" s="7" t="n">
-        <v>708</v>
+        <v>73979</v>
       </c>
       <c r="X51" s="7" t="n">
         <v>10</v>
@@ -4249,16 +4269,16 @@
     <row r="52">
       <c r="T52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V52" s="4" t="n">
-        <v>733</v>
+        <v>77997</v>
       </c>
       <c r="X52" s="4" t="n">
         <v>62</v>
@@ -4290,16 +4310,16 @@
     <row r="53">
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V53" s="7" t="n">
-        <v>662</v>
+        <v>81861</v>
       </c>
       <c r="X53" s="7" t="n">
         <v>17</v>
@@ -4331,7 +4351,7 @@
     <row r="54">
       <c r="T54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
@@ -4340,7 +4360,7 @@
         </is>
       </c>
       <c r="V54" s="4" t="n">
-        <v>678</v>
+        <v>756</v>
       </c>
       <c r="X54" s="4" t="n">
         <v>11</v>
@@ -4372,7 +4392,7 @@
     <row r="55">
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
@@ -4381,7 +4401,7 @@
         </is>
       </c>
       <c r="V55" s="7" t="n">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="X55" s="7" t="n">
         <v>62</v>
@@ -4413,7 +4433,7 @@
     <row r="56">
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
@@ -4422,7 +4442,7 @@
         </is>
       </c>
       <c r="V56" s="4" t="n">
-        <v>683</v>
+        <v>733</v>
       </c>
       <c r="X56" s="4" t="n">
         <v>1</v>
@@ -4454,7 +4474,7 @@
     <row r="57">
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
@@ -4463,7 +4483,7 @@
         </is>
       </c>
       <c r="V57" s="7" t="n">
-        <v>720</v>
+        <v>662</v>
       </c>
       <c r="X57" s="7" t="n">
         <v>7</v>
@@ -4495,7 +4515,7 @@
     <row r="58">
       <c r="T58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U58" s="4" t="inlineStr">
@@ -4504,7 +4524,7 @@
         </is>
       </c>
       <c r="V58" s="4" t="n">
-        <v>695</v>
+        <v>678</v>
       </c>
       <c r="X58" s="4" t="n">
         <v>76</v>
@@ -4536,7 +4556,7 @@
     <row r="59">
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
@@ -4545,7 +4565,7 @@
         </is>
       </c>
       <c r="V59" s="7" t="n">
-        <v>707</v>
+        <v>700</v>
       </c>
       <c r="X59" s="7" t="n">
         <v>8</v>
@@ -4577,7 +4597,7 @@
     <row r="60">
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U60" s="4" t="inlineStr">
@@ -4586,7 +4606,7 @@
         </is>
       </c>
       <c r="V60" s="4" t="n">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="X60" s="4" t="n">
         <v>46</v>
@@ -4618,7 +4638,7 @@
     <row r="61">
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
@@ -4627,7 +4647,7 @@
         </is>
       </c>
       <c r="V61" s="7" t="n">
-        <v>660</v>
+        <v>720</v>
       </c>
       <c r="X61" s="7" t="n">
         <v>41</v>
@@ -4659,16 +4679,16 @@
     <row r="62">
       <c r="T62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V62" s="4" t="n">
-        <v>48266</v>
+        <v>695</v>
       </c>
       <c r="X62" s="4" t="n">
         <v>11</v>
@@ -4700,16 +4720,16 @@
     <row r="63">
       <c r="T63" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V63" s="7" t="n">
-        <v>50405</v>
+        <v>707</v>
       </c>
       <c r="X63" s="7" t="n">
         <v>65</v>
@@ -4741,16 +4761,16 @@
     <row r="64">
       <c r="T64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V64" s="4" t="n">
-        <v>48886</v>
+        <v>677</v>
       </c>
       <c r="X64" s="4" t="n">
         <v>1</v>
@@ -4782,16 +4802,16 @@
     <row r="65">
       <c r="T65" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V65" s="7" t="n">
-        <v>47253</v>
+        <v>660</v>
       </c>
       <c r="X65" s="7" t="n">
         <v>11</v>
@@ -4823,16 +4843,16 @@
     <row r="66">
       <c r="T66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V66" s="4" t="n">
-        <v>46972</v>
+        <v>719</v>
       </c>
       <c r="X66" s="4" t="n">
         <v>1</v>
@@ -4864,7 +4884,7 @@
     <row r="67">
       <c r="T67" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U67" s="7" t="inlineStr">
@@ -4873,7 +4893,7 @@
         </is>
       </c>
       <c r="V67" s="7" t="n">
-        <v>48667</v>
+        <v>48266</v>
       </c>
       <c r="X67" s="7" t="n">
         <v>92</v>
@@ -4905,7 +4925,7 @@
     <row r="68">
       <c r="T68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U68" s="4" t="inlineStr">
@@ -4914,7 +4934,7 @@
         </is>
       </c>
       <c r="V68" s="4" t="n">
-        <v>48109</v>
+        <v>50405</v>
       </c>
       <c r="X68" s="4" t="n">
         <v>5</v>
@@ -4946,7 +4966,7 @@
     <row r="69">
       <c r="T69" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U69" s="7" t="inlineStr">
@@ -4955,7 +4975,7 @@
         </is>
       </c>
       <c r="V69" s="7" t="n">
-        <v>48852</v>
+        <v>48886</v>
       </c>
       <c r="X69" s="7" t="n">
         <v>62</v>
@@ -4987,7 +5007,7 @@
     <row r="70">
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U70" s="4" t="inlineStr">
@@ -4996,7 +5016,7 @@
         </is>
       </c>
       <c r="V70" s="4" t="n">
-        <v>50001</v>
+        <v>47253</v>
       </c>
       <c r="X70" s="4" t="n">
         <v>31</v>
@@ -5028,7 +5048,7 @@
     <row r="71">
       <c r="T71" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U71" s="7" t="inlineStr">
@@ -5037,7 +5057,7 @@
         </is>
       </c>
       <c r="V71" s="7" t="n">
-        <v>49282</v>
+        <v>46972</v>
       </c>
       <c r="X71" s="7" t="n">
         <v>18</v>
@@ -5069,7 +5089,7 @@
     <row r="72">
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U72" s="4" t="inlineStr">
@@ -5078,7 +5098,7 @@
         </is>
       </c>
       <c r="V72" s="4" t="n">
-        <v>47782</v>
+        <v>48667</v>
       </c>
       <c r="X72" s="4" t="n">
         <v>57</v>
@@ -5110,7 +5130,7 @@
     <row r="73">
       <c r="T73" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U73" s="7" t="inlineStr">
@@ -5119,7 +5139,7 @@
         </is>
       </c>
       <c r="V73" s="7" t="n">
-        <v>47775</v>
+        <v>48109</v>
       </c>
       <c r="X73" s="7" t="n">
         <v>14</v>
@@ -5151,16 +5171,16 @@
     <row r="74">
       <c r="T74" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U74" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V74" s="4" t="n">
-        <v>1</v>
+        <v>48852</v>
       </c>
       <c r="X74" s="4" t="n">
         <v>1</v>
@@ -5192,16 +5212,16 @@
     <row r="75">
       <c r="T75" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U75" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V75" s="7" t="n">
-        <v>1</v>
+        <v>50001</v>
       </c>
       <c r="X75" s="7" t="n">
         <v>66</v>
@@ -5233,16 +5253,16 @@
     <row r="76">
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V76" s="4" t="n">
-        <v>1</v>
+        <v>49282</v>
       </c>
       <c r="X76" s="4" t="n">
         <v>8</v>
@@ -5274,16 +5294,16 @@
     <row r="77">
       <c r="T77" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V77" s="7" t="n">
-        <v>1</v>
+        <v>47782</v>
       </c>
       <c r="X77" s="7" t="n">
         <v>45</v>
@@ -5315,16 +5335,16 @@
     <row r="78">
       <c r="T78" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U78" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V78" s="4" t="n">
-        <v>1</v>
+        <v>47775</v>
       </c>
       <c r="X78" s="4" t="n">
         <v>33</v>
@@ -5356,16 +5376,16 @@
     <row r="79">
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U79" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V79" s="7" t="n">
-        <v>1</v>
+        <v>50744</v>
       </c>
       <c r="X79" s="7" t="n">
         <v>7</v>
@@ -5397,7 +5417,7 @@
     <row r="80">
       <c r="T80" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U80" s="4" t="inlineStr">
@@ -5438,7 +5458,7 @@
     <row r="81">
       <c r="T81" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U81" s="7" t="inlineStr">
@@ -5479,7 +5499,7 @@
     <row r="82">
       <c r="T82" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U82" s="4" t="inlineStr">
@@ -5520,7 +5540,7 @@
     <row r="83">
       <c r="T83" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U83" s="7" t="inlineStr">
@@ -5561,7 +5581,7 @@
     <row r="84">
       <c r="T84" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U84" s="4" t="inlineStr">
@@ -5602,7 +5622,7 @@
     <row r="85">
       <c r="T85" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U85" s="7" t="inlineStr">
@@ -5643,12 +5663,12 @@
     <row r="86">
       <c r="T86" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U86" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V86" s="4" t="n">
@@ -5684,12 +5704,12 @@
     <row r="87">
       <c r="T87" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U87" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V87" s="7" t="n">
@@ -5725,12 +5745,12 @@
     <row r="88">
       <c r="T88" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U88" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V88" s="4" t="n">
@@ -5766,12 +5786,12 @@
     <row r="89">
       <c r="T89" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U89" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V89" s="7" t="n">
@@ -5807,12 +5827,12 @@
     <row r="90">
       <c r="T90" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U90" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V90" s="4" t="n">
@@ -5848,12 +5868,12 @@
     <row r="91">
       <c r="T91" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U91" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V91" s="7" t="n">
@@ -5889,12 +5909,12 @@
     <row r="92">
       <c r="T92" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U92" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V92" s="4" t="n">
@@ -5930,7 +5950,7 @@
     <row r="93">
       <c r="T93" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U93" s="7" t="inlineStr">
@@ -5971,7 +5991,7 @@
     <row r="94">
       <c r="T94" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U94" s="4" t="inlineStr">
@@ -6012,7 +6032,7 @@
     <row r="95">
       <c r="T95" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U95" s="7" t="inlineStr">
@@ -6053,7 +6073,7 @@
     <row r="96">
       <c r="T96" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U96" s="4" t="inlineStr">
@@ -6094,7 +6114,7 @@
     <row r="97">
       <c r="T97" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U97" s="7" t="inlineStr">
@@ -6135,16 +6155,16 @@
     <row r="98">
       <c r="T98" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U98" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V98" s="4" t="n">
-        <v>10655</v>
+        <v>1</v>
       </c>
       <c r="X98" s="4" t="n">
         <v>8</v>
@@ -6176,16 +6196,16 @@
     <row r="99">
       <c r="T99" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U99" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V99" s="7" t="n">
-        <v>10413</v>
+        <v>1</v>
       </c>
       <c r="X99" s="7" t="n">
         <v>1</v>
@@ -6217,20 +6237,30 @@
     <row r="100">
       <c r="T100" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U100" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V100" s="4" t="n">
-        <v>10036</v>
-      </c>
-      <c r="X100" s="4" t="n"/>
-      <c r="Y100" s="4" t="n"/>
-      <c r="Z100" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X100" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="Y100" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z100" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB100" s="4" t="n">
         <v>6</v>
       </c>
@@ -6248,20 +6278,30 @@
     <row r="101">
       <c r="T101" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U101" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V101" s="7" t="n">
-        <v>9869</v>
-      </c>
-      <c r="X101" s="7" t="n"/>
-      <c r="Y101" s="7" t="n"/>
-      <c r="Z101" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X101" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y101" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z101" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB101" s="7" t="n">
         <v>2</v>
       </c>
@@ -6279,20 +6319,30 @@
     <row r="102">
       <c r="T102" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U102" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V102" s="4" t="n">
-        <v>10072</v>
-      </c>
-      <c r="X102" s="4" t="n"/>
-      <c r="Y102" s="4" t="n"/>
-      <c r="Z102" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X102" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="Y102" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z102" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB102" s="4" t="n">
         <v>443</v>
       </c>
@@ -6310,20 +6360,30 @@
     <row r="103">
       <c r="T103" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U103" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V103" s="7" t="n">
-        <v>10125</v>
-      </c>
-      <c r="X103" s="7" t="n"/>
-      <c r="Y103" s="7" t="n"/>
-      <c r="Z103" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X103" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y103" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z103" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB103" s="7" t="n">
         <v>29</v>
       </c>
@@ -6341,20 +6401,30 @@
     <row r="104">
       <c r="T104" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U104" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V104" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X104" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Y104" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z104" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
-      <c r="V104" s="4" t="n">
-        <v>10161</v>
-      </c>
-      <c r="X104" s="4" t="n"/>
-      <c r="Y104" s="4" t="n"/>
-      <c r="Z104" s="4" t="n"/>
       <c r="AB104" s="4" t="n">
         <v>162</v>
       </c>
@@ -6372,20 +6442,30 @@
     <row r="105">
       <c r="T105" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U105" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V105" s="7" t="n">
-        <v>10341</v>
-      </c>
-      <c r="X105" s="7" t="n"/>
-      <c r="Y105" s="7" t="n"/>
-      <c r="Z105" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X105" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y105" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z105" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB105" s="7" t="n">
         <v>52</v>
       </c>
@@ -6403,7 +6483,7 @@
     <row r="106">
       <c r="T106" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U106" s="4" t="inlineStr">
@@ -6412,11 +6492,21 @@
         </is>
       </c>
       <c r="V106" s="4" t="n">
-        <v>10448</v>
-      </c>
-      <c r="X106" s="4" t="n"/>
-      <c r="Y106" s="4" t="n"/>
-      <c r="Z106" s="4" t="n"/>
+        <v>10655</v>
+      </c>
+      <c r="X106" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y106" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z106" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB106" s="4" t="n">
         <v>54</v>
       </c>
@@ -6434,7 +6524,7 @@
     <row r="107">
       <c r="T107" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U107" s="7" t="inlineStr">
@@ -6443,13 +6533,23 @@
         </is>
       </c>
       <c r="V107" s="7" t="n">
-        <v>10118</v>
-      </c>
-      <c r="X107" s="7" t="n"/>
-      <c r="Y107" s="7" t="n"/>
-      <c r="Z107" s="7" t="n"/>
+        <v>10413</v>
+      </c>
+      <c r="X107" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y107" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="Z107" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
       <c r="AB107" s="7" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AC107" s="7" t="inlineStr">
         <is>
@@ -6465,7 +6565,7 @@
     <row r="108">
       <c r="T108" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U108" s="4" t="inlineStr">
@@ -6474,7 +6574,7 @@
         </is>
       </c>
       <c r="V108" s="4" t="n">
-        <v>9869</v>
+        <v>10036</v>
       </c>
       <c r="X108" s="4" t="n"/>
       <c r="Y108" s="4" t="n"/>
@@ -6496,7 +6596,7 @@
     <row r="109">
       <c r="T109" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U109" s="7" t="inlineStr">
@@ -6505,7 +6605,7 @@
         </is>
       </c>
       <c r="V109" s="7" t="n">
-        <v>10116</v>
+        <v>9869</v>
       </c>
       <c r="X109" s="7" t="n"/>
       <c r="Y109" s="7" t="n"/>
@@ -6527,16 +6627,16 @@
     <row r="110">
       <c r="T110" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U110" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V110" s="4" t="n">
-        <v>23063</v>
+        <v>10072</v>
       </c>
       <c r="X110" s="4" t="n"/>
       <c r="Y110" s="4" t="n"/>
@@ -6558,175 +6658,255 @@
     <row r="111">
       <c r="T111" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U111" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V111" s="7" t="n">
-        <v>23168</v>
+        <v>10125</v>
       </c>
       <c r="X111" s="7" t="n"/>
       <c r="Y111" s="7" t="n"/>
       <c r="Z111" s="7" t="n"/>
-      <c r="AB111" s="7" t="n"/>
-      <c r="AC111" s="7" t="n"/>
-      <c r="AD111" s="7" t="n"/>
+      <c r="AB111" s="7" t="n">
+        <v>366</v>
+      </c>
+      <c r="AC111" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD111" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="T112" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U112" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V112" s="4" t="n">
-        <v>24394</v>
+        <v>10161</v>
       </c>
       <c r="X112" s="4" t="n"/>
       <c r="Y112" s="4" t="n"/>
       <c r="Z112" s="4" t="n"/>
-      <c r="AB112" s="4" t="n"/>
-      <c r="AC112" s="4" t="n"/>
-      <c r="AD112" s="4" t="n"/>
+      <c r="AB112" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="AC112" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD112" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="T113" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U113" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V113" s="7" t="n">
-        <v>21980</v>
+        <v>10341</v>
       </c>
       <c r="X113" s="7" t="n"/>
       <c r="Y113" s="7" t="n"/>
       <c r="Z113" s="7" t="n"/>
-      <c r="AB113" s="7" t="n"/>
-      <c r="AC113" s="7" t="n"/>
-      <c r="AD113" s="7" t="n"/>
+      <c r="AB113" s="7" t="n">
+        <v>170</v>
+      </c>
+      <c r="AC113" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD113" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="T114" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U114" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V114" s="4" t="n">
-        <v>21517</v>
+        <v>10448</v>
       </c>
       <c r="X114" s="4" t="n"/>
       <c r="Y114" s="4" t="n"/>
       <c r="Z114" s="4" t="n"/>
-      <c r="AB114" s="4" t="n"/>
-      <c r="AC114" s="4" t="n"/>
-      <c r="AD114" s="4" t="n"/>
+      <c r="AB114" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="AC114" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD114" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="T115" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U115" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V115" s="7" t="n">
-        <v>22785</v>
+        <v>10118</v>
       </c>
       <c r="X115" s="7" t="n"/>
       <c r="Y115" s="7" t="n"/>
       <c r="Z115" s="7" t="n"/>
-      <c r="AB115" s="7" t="n"/>
-      <c r="AC115" s="7" t="n"/>
-      <c r="AD115" s="7" t="n"/>
+      <c r="AB115" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="AC115" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD115" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="T116" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U116" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V116" s="4" t="n">
-        <v>24108</v>
+        <v>9869</v>
       </c>
       <c r="X116" s="4" t="n"/>
       <c r="Y116" s="4" t="n"/>
       <c r="Z116" s="4" t="n"/>
-      <c r="AB116" s="4" t="n"/>
-      <c r="AC116" s="4" t="n"/>
-      <c r="AD116" s="4" t="n"/>
+      <c r="AB116" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="AC116" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD116" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="T117" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U117" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V117" s="7" t="n">
-        <v>23330</v>
+        <v>10116</v>
       </c>
       <c r="X117" s="7" t="n"/>
       <c r="Y117" s="7" t="n"/>
       <c r="Z117" s="7" t="n"/>
-      <c r="AB117" s="7" t="n"/>
-      <c r="AC117" s="7" t="n"/>
-      <c r="AD117" s="7" t="n"/>
+      <c r="AB117" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC117" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD117" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="T118" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U118" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V118" s="4" t="n">
-        <v>22973</v>
+        <v>10451</v>
       </c>
       <c r="X118" s="4" t="n"/>
       <c r="Y118" s="4" t="n"/>
       <c r="Z118" s="4" t="n"/>
-      <c r="AB118" s="4" t="n"/>
-      <c r="AC118" s="4" t="n"/>
-      <c r="AD118" s="4" t="n"/>
+      <c r="AB118" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC118" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD118" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="T119" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U119" s="7" t="inlineStr">
@@ -6735,19 +6915,29 @@
         </is>
       </c>
       <c r="V119" s="7" t="n">
-        <v>23457</v>
+        <v>23063</v>
       </c>
       <c r="X119" s="7" t="n"/>
       <c r="Y119" s="7" t="n"/>
       <c r="Z119" s="7" t="n"/>
-      <c r="AB119" s="7" t="n"/>
-      <c r="AC119" s="7" t="n"/>
-      <c r="AD119" s="7" t="n"/>
+      <c r="AB119" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC119" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="AD119" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="T120" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U120" s="4" t="inlineStr">
@@ -6756,7 +6946,7 @@
         </is>
       </c>
       <c r="V120" s="4" t="n">
-        <v>24804</v>
+        <v>23168</v>
       </c>
       <c r="X120" s="4" t="n"/>
       <c r="Y120" s="4" t="n"/>
@@ -6768,7 +6958,7 @@
     <row r="121">
       <c r="T121" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U121" s="7" t="inlineStr">
@@ -6777,7 +6967,7 @@
         </is>
       </c>
       <c r="V121" s="7" t="n">
-        <v>21635</v>
+        <v>24394</v>
       </c>
       <c r="X121" s="7" t="n"/>
       <c r="Y121" s="7" t="n"/>
@@ -6789,16 +6979,16 @@
     <row r="122">
       <c r="T122" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U122" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V122" s="4" t="n">
-        <v>17887</v>
+        <v>21980</v>
       </c>
       <c r="X122" s="4" t="n"/>
       <c r="Y122" s="4" t="n"/>
@@ -6810,16 +7000,16 @@
     <row r="123">
       <c r="T123" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U123" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V123" s="7" t="n">
-        <v>17641</v>
+        <v>21517</v>
       </c>
       <c r="X123" s="7" t="n"/>
       <c r="Y123" s="7" t="n"/>
@@ -6831,16 +7021,16 @@
     <row r="124">
       <c r="T124" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U124" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V124" s="4" t="n">
-        <v>17144</v>
+        <v>22785</v>
       </c>
       <c r="X124" s="4" t="n"/>
       <c r="Y124" s="4" t="n"/>
@@ -6852,16 +7042,16 @@
     <row r="125">
       <c r="T125" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U125" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V125" s="7" t="n">
-        <v>17159</v>
+        <v>24108</v>
       </c>
       <c r="X125" s="7" t="n"/>
       <c r="Y125" s="7" t="n"/>
@@ -6873,16 +7063,16 @@
     <row r="126">
       <c r="T126" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U126" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V126" s="4" t="n">
-        <v>17724</v>
+        <v>23330</v>
       </c>
       <c r="X126" s="4" t="n"/>
       <c r="Y126" s="4" t="n"/>
@@ -6894,16 +7084,16 @@
     <row r="127">
       <c r="T127" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U127" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V127" s="7" t="n">
-        <v>17829</v>
+        <v>22973</v>
       </c>
       <c r="X127" s="7" t="n"/>
       <c r="Y127" s="7" t="n"/>
@@ -6915,16 +7105,16 @@
     <row r="128">
       <c r="T128" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U128" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V128" s="4" t="n">
-        <v>18088</v>
+        <v>23457</v>
       </c>
       <c r="X128" s="4" t="n"/>
       <c r="Y128" s="4" t="n"/>
@@ -6936,16 +7126,16 @@
     <row r="129">
       <c r="T129" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U129" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V129" s="7" t="n">
-        <v>17869</v>
+        <v>24804</v>
       </c>
       <c r="X129" s="7" t="n"/>
       <c r="Y129" s="7" t="n"/>
@@ -6957,16 +7147,16 @@
     <row r="130">
       <c r="T130" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U130" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V130" s="4" t="n">
-        <v>17862</v>
+        <v>21635</v>
       </c>
       <c r="X130" s="4" t="n"/>
       <c r="Y130" s="4" t="n"/>
@@ -6978,16 +7168,16 @@
     <row r="131">
       <c r="T131" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U131" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V131" s="7" t="n">
-        <v>17228</v>
+        <v>23338</v>
       </c>
       <c r="X131" s="7" t="n"/>
       <c r="Y131" s="7" t="n"/>
@@ -6999,7 +7189,7 @@
     <row r="132">
       <c r="T132" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U132" s="4" t="inlineStr">
@@ -7008,7 +7198,7 @@
         </is>
       </c>
       <c r="V132" s="4" t="n">
-        <v>17411</v>
+        <v>17887</v>
       </c>
       <c r="X132" s="4" t="n"/>
       <c r="Y132" s="4" t="n"/>
@@ -7020,7 +7210,7 @@
     <row r="133">
       <c r="T133" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U133" s="7" t="inlineStr">
@@ -7029,7 +7219,7 @@
         </is>
       </c>
       <c r="V133" s="7" t="n">
-        <v>17610</v>
+        <v>17641</v>
       </c>
       <c r="X133" s="7" t="n"/>
       <c r="Y133" s="7" t="n"/>
@@ -7041,16 +7231,16 @@
     <row r="134">
       <c r="T134" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U134" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V134" s="4" t="n">
-        <v>700</v>
+        <v>17144</v>
       </c>
       <c r="X134" s="4" t="n"/>
       <c r="Y134" s="4" t="n"/>
@@ -7062,16 +7252,16 @@
     <row r="135">
       <c r="T135" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U135" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V135" s="7" t="n">
-        <v>686</v>
+        <v>17159</v>
       </c>
       <c r="X135" s="7" t="n"/>
       <c r="Y135" s="7" t="n"/>
@@ -7083,16 +7273,16 @@
     <row r="136">
       <c r="T136" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U136" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V136" s="4" t="n">
-        <v>698</v>
+        <v>17724</v>
       </c>
       <c r="X136" s="4" t="n"/>
       <c r="Y136" s="4" t="n"/>
@@ -7104,16 +7294,16 @@
     <row r="137">
       <c r="T137" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U137" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V137" s="7" t="n">
-        <v>687</v>
+        <v>17829</v>
       </c>
       <c r="X137" s="7" t="n"/>
       <c r="Y137" s="7" t="n"/>
@@ -7125,16 +7315,16 @@
     <row r="138">
       <c r="T138" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U138" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V138" s="4" t="n">
-        <v>716</v>
+        <v>18088</v>
       </c>
       <c r="X138" s="4" t="n"/>
       <c r="Y138" s="4" t="n"/>
@@ -7146,16 +7336,16 @@
     <row r="139">
       <c r="T139" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U139" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V139" s="7" t="n">
-        <v>719</v>
+        <v>17869</v>
       </c>
       <c r="X139" s="7" t="n"/>
       <c r="Y139" s="7" t="n"/>
@@ -7167,16 +7357,16 @@
     <row r="140">
       <c r="T140" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U140" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V140" s="4" t="n">
-        <v>724</v>
+        <v>17862</v>
       </c>
       <c r="X140" s="4" t="n"/>
       <c r="Y140" s="4" t="n"/>
@@ -7188,16 +7378,16 @@
     <row r="141">
       <c r="T141" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U141" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V141" s="7" t="n">
-        <v>701</v>
+        <v>17228</v>
       </c>
       <c r="X141" s="7" t="n"/>
       <c r="Y141" s="7" t="n"/>
@@ -7209,16 +7399,16 @@
     <row r="142">
       <c r="T142" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U142" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V142" s="4" t="n">
-        <v>736</v>
+        <v>17411</v>
       </c>
       <c r="X142" s="4" t="n"/>
       <c r="Y142" s="4" t="n"/>
@@ -7230,16 +7420,16 @@
     <row r="143">
       <c r="T143" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U143" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V143" s="7" t="n">
-        <v>722</v>
+        <v>17610</v>
       </c>
       <c r="X143" s="7" t="n"/>
       <c r="Y143" s="7" t="n"/>
@@ -7251,16 +7441,16 @@
     <row r="144">
       <c r="T144" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U144" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V144" s="4" t="n">
-        <v>684</v>
+        <v>17791</v>
       </c>
       <c r="X144" s="4" t="n"/>
       <c r="Y144" s="4" t="n"/>
@@ -7272,7 +7462,7 @@
     <row r="145">
       <c r="T145" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="U145" s="7" t="inlineStr">
@@ -7281,7 +7471,7 @@
         </is>
       </c>
       <c r="V145" s="7" t="n">
-        <v>688</v>
+        <v>700</v>
       </c>
       <c r="X145" s="7" t="n"/>
       <c r="Y145" s="7" t="n"/>
@@ -7293,16 +7483,16 @@
     <row r="146">
       <c r="T146" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="U146" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V146" s="4" t="n">
-        <v>2290</v>
+        <v>686</v>
       </c>
       <c r="X146" s="4" t="n"/>
       <c r="Y146" s="4" t="n"/>
@@ -7314,16 +7504,16 @@
     <row r="147">
       <c r="T147" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="U147" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V147" s="7" t="n">
-        <v>2092</v>
+        <v>698</v>
       </c>
       <c r="X147" s="7" t="n"/>
       <c r="Y147" s="7" t="n"/>
@@ -7335,16 +7525,16 @@
     <row r="148">
       <c r="T148" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="U148" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V148" s="4" t="n">
-        <v>2043</v>
+        <v>687</v>
       </c>
       <c r="X148" s="4" t="n"/>
       <c r="Y148" s="4" t="n"/>
@@ -7356,16 +7546,16 @@
     <row r="149">
       <c r="T149" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="U149" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V149" s="7" t="n">
-        <v>1969</v>
+        <v>716</v>
       </c>
       <c r="X149" s="7" t="n"/>
       <c r="Y149" s="7" t="n"/>
@@ -7377,16 +7567,16 @@
     <row r="150">
       <c r="T150" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="U150" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V150" s="4" t="n">
-        <v>1938</v>
+        <v>719</v>
       </c>
       <c r="X150" s="4" t="n"/>
       <c r="Y150" s="4" t="n"/>
@@ -7398,16 +7588,16 @@
     <row r="151">
       <c r="T151" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="U151" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V151" s="7" t="n">
-        <v>2048</v>
+        <v>724</v>
       </c>
       <c r="X151" s="7" t="n"/>
       <c r="Y151" s="7" t="n"/>
@@ -7419,16 +7609,16 @@
     <row r="152">
       <c r="T152" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="U152" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V152" s="4" t="n">
-        <v>2033</v>
+        <v>701</v>
       </c>
       <c r="X152" s="4" t="n"/>
       <c r="Y152" s="4" t="n"/>
@@ -7440,16 +7630,16 @@
     <row r="153">
       <c r="T153" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U153" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V153" s="7" t="n">
-        <v>2242</v>
+        <v>736</v>
       </c>
       <c r="X153" s="7" t="n"/>
       <c r="Y153" s="7" t="n"/>
@@ -7461,16 +7651,16 @@
     <row r="154">
       <c r="T154" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="U154" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V154" s="4" t="n">
-        <v>2096</v>
+        <v>722</v>
       </c>
       <c r="X154" s="4" t="n"/>
       <c r="Y154" s="4" t="n"/>
@@ -7482,16 +7672,16 @@
     <row r="155">
       <c r="T155" s="7" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="U155" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V155" s="7" t="n">
-        <v>1979</v>
+        <v>684</v>
       </c>
       <c r="X155" s="7" t="n"/>
       <c r="Y155" s="7" t="n"/>
@@ -7503,16 +7693,16 @@
     <row r="156">
       <c r="T156" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="U156" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V156" s="4" t="n">
-        <v>1870</v>
+        <v>688</v>
       </c>
       <c r="X156" s="4" t="n"/>
       <c r="Y156" s="4" t="n"/>
@@ -7524,16 +7714,16 @@
     <row r="157">
       <c r="T157" s="7" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="U157" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
       <c r="V157" s="7" t="n">
-        <v>1877</v>
+        <v>700</v>
       </c>
       <c r="X157" s="7" t="n"/>
       <c r="Y157" s="7" t="n"/>
@@ -7541,6 +7731,279 @@
       <c r="AB157" s="7" t="n"/>
       <c r="AC157" s="7" t="n"/>
       <c r="AD157" s="7" t="n"/>
+    </row>
+    <row r="158">
+      <c r="T158" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="U158" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V158" s="4" t="n">
+        <v>2290</v>
+      </c>
+      <c r="X158" s="4" t="n"/>
+      <c r="Y158" s="4" t="n"/>
+      <c r="Z158" s="4" t="n"/>
+      <c r="AB158" s="4" t="n"/>
+      <c r="AC158" s="4" t="n"/>
+      <c r="AD158" s="4" t="n"/>
+    </row>
+    <row r="159">
+      <c r="T159" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="U159" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V159" s="7" t="n">
+        <v>2092</v>
+      </c>
+      <c r="X159" s="7" t="n"/>
+      <c r="Y159" s="7" t="n"/>
+      <c r="Z159" s="7" t="n"/>
+      <c r="AB159" s="7" t="n"/>
+      <c r="AC159" s="7" t="n"/>
+      <c r="AD159" s="7" t="n"/>
+    </row>
+    <row r="160">
+      <c r="T160" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="U160" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V160" s="4" t="n">
+        <v>2043</v>
+      </c>
+      <c r="X160" s="4" t="n"/>
+      <c r="Y160" s="4" t="n"/>
+      <c r="Z160" s="4" t="n"/>
+      <c r="AB160" s="4" t="n"/>
+      <c r="AC160" s="4" t="n"/>
+      <c r="AD160" s="4" t="n"/>
+    </row>
+    <row r="161">
+      <c r="T161" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="U161" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V161" s="7" t="n">
+        <v>1969</v>
+      </c>
+      <c r="X161" s="7" t="n"/>
+      <c r="Y161" s="7" t="n"/>
+      <c r="Z161" s="7" t="n"/>
+      <c r="AB161" s="7" t="n"/>
+      <c r="AC161" s="7" t="n"/>
+      <c r="AD161" s="7" t="n"/>
+    </row>
+    <row r="162">
+      <c r="T162" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="U162" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V162" s="4" t="n">
+        <v>1938</v>
+      </c>
+      <c r="X162" s="4" t="n"/>
+      <c r="Y162" s="4" t="n"/>
+      <c r="Z162" s="4" t="n"/>
+      <c r="AB162" s="4" t="n"/>
+      <c r="AC162" s="4" t="n"/>
+      <c r="AD162" s="4" t="n"/>
+    </row>
+    <row r="163">
+      <c r="T163" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="U163" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V163" s="7" t="n">
+        <v>2048</v>
+      </c>
+      <c r="X163" s="7" t="n"/>
+      <c r="Y163" s="7" t="n"/>
+      <c r="Z163" s="7" t="n"/>
+      <c r="AB163" s="7" t="n"/>
+      <c r="AC163" s="7" t="n"/>
+      <c r="AD163" s="7" t="n"/>
+    </row>
+    <row r="164">
+      <c r="T164" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="U164" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V164" s="4" t="n">
+        <v>2033</v>
+      </c>
+      <c r="X164" s="4" t="n"/>
+      <c r="Y164" s="4" t="n"/>
+      <c r="Z164" s="4" t="n"/>
+      <c r="AB164" s="4" t="n"/>
+      <c r="AC164" s="4" t="n"/>
+      <c r="AD164" s="4" t="n"/>
+    </row>
+    <row r="165">
+      <c r="T165" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="U165" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V165" s="7" t="n">
+        <v>2242</v>
+      </c>
+      <c r="X165" s="7" t="n"/>
+      <c r="Y165" s="7" t="n"/>
+      <c r="Z165" s="7" t="n"/>
+      <c r="AB165" s="7" t="n"/>
+      <c r="AC165" s="7" t="n"/>
+      <c r="AD165" s="7" t="n"/>
+    </row>
+    <row r="166">
+      <c r="T166" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="U166" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V166" s="4" t="n">
+        <v>2096</v>
+      </c>
+      <c r="X166" s="4" t="n"/>
+      <c r="Y166" s="4" t="n"/>
+      <c r="Z166" s="4" t="n"/>
+      <c r="AB166" s="4" t="n"/>
+      <c r="AC166" s="4" t="n"/>
+      <c r="AD166" s="4" t="n"/>
+    </row>
+    <row r="167">
+      <c r="T167" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="U167" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V167" s="7" t="n">
+        <v>1979</v>
+      </c>
+      <c r="X167" s="7" t="n"/>
+      <c r="Y167" s="7" t="n"/>
+      <c r="Z167" s="7" t="n"/>
+      <c r="AB167" s="7" t="n"/>
+      <c r="AC167" s="7" t="n"/>
+      <c r="AD167" s="7" t="n"/>
+    </row>
+    <row r="168">
+      <c r="T168" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="U168" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V168" s="4" t="n">
+        <v>1870</v>
+      </c>
+      <c r="X168" s="4" t="n"/>
+      <c r="Y168" s="4" t="n"/>
+      <c r="Z168" s="4" t="n"/>
+      <c r="AB168" s="4" t="n"/>
+      <c r="AC168" s="4" t="n"/>
+      <c r="AD168" s="4" t="n"/>
+    </row>
+    <row r="169">
+      <c r="T169" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="U169" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V169" s="7" t="n">
+        <v>1877</v>
+      </c>
+      <c r="X169" s="7" t="n"/>
+      <c r="Y169" s="7" t="n"/>
+      <c r="Z169" s="7" t="n"/>
+      <c r="AB169" s="7" t="n"/>
+      <c r="AC169" s="7" t="n"/>
+      <c r="AD169" s="7" t="n"/>
+    </row>
+    <row r="170">
+      <c r="T170" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="U170" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V170" s="4" t="n">
+        <v>2052</v>
+      </c>
+      <c r="X170" s="4" t="n"/>
+      <c r="Y170" s="4" t="n"/>
+      <c r="Z170" s="4" t="n"/>
+      <c r="AB170" s="4" t="n"/>
+      <c r="AC170" s="4" t="n"/>
+      <c r="AD170" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Updated hard coded info for the month and added 4.2632.4
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -716,7 +716,7 @@
         <v>1.23</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>1.26</v>
@@ -752,7 +752,7 @@
         <v>1.23</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>1.26</v>
@@ -788,7 +788,7 @@
         <v>1.23</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>1.26</v>
@@ -824,7 +824,7 @@
         <v>1.23</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>1.26</v>
@@ -860,7 +860,7 @@
         <v>1.23</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>1.26</v>
@@ -896,7 +896,7 @@
         <v>1.23</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>1.26</v>
@@ -932,7 +932,7 @@
         <v>1.23</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>1.26</v>
@@ -968,7 +968,7 @@
         <v>1.23</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>1.26</v>
@@ -1004,7 +1004,7 @@
         <v>1.23</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>1.26</v>
@@ -1040,7 +1040,7 @@
         <v>1.23</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>1.26</v>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD39"/>
+  <dimension ref="A1:AD52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1558,29 +1558,49 @@
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
+      <c r="D5" s="7">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="7">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C5)</f>
+        <v/>
+      </c>
       <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
+      <c r="G5" s="7">
+        <f>ROUND(MAX(0,MIN(100,(1-E5/IF(D5&gt;0,D5,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>MIN(1,(G5-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="n"/>
-      <c r="N5" s="7" t="n"/>
+      <c r="K5" s="7">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C5)</f>
+        <v/>
+      </c>
+      <c r="L5" s="7">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K5/IF(D5&gt;0,D5,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M5" s="7">
+        <f>MAX(0,(L5-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
+        <f>$B$2+H5+M5</f>
+        <v/>
+      </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="U5" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U5" s="7" t="inlineStr"/>
       <c r="V5" s="7" t="n">
-        <v>5034</v>
+        <v>1</v>
       </c>
       <c r="X5" s="7" t="n">
         <v>29</v>
@@ -1636,7 +1656,7 @@
       <c r="N6" s="4" t="n"/>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
@@ -1645,7 +1665,7 @@
         </is>
       </c>
       <c r="V6" s="4" t="n">
-        <v>4901</v>
+        <v>5034</v>
       </c>
       <c r="X6" s="4" t="n">
         <v>11</v>
@@ -1701,7 +1721,7 @@
       <c r="N7" s="7" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
@@ -1710,7 +1730,7 @@
         </is>
       </c>
       <c r="V7" s="7" t="n">
-        <v>5271</v>
+        <v>4901</v>
       </c>
       <c r="X7" s="7" t="n">
         <v>73</v>
@@ -1766,16 +1786,16 @@
       <c r="N8" s="4" t="n"/>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V8" s="4" t="n">
-        <v>14257</v>
+        <v>5271</v>
       </c>
       <c r="X8" s="4" t="n">
         <v>5</v>
@@ -1825,16 +1845,16 @@
       <c r="N9" s="7" t="n"/>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V9" s="7" t="n">
-        <v>14081</v>
+        <v>5154</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>3</v>
@@ -1892,7 +1912,7 @@
       <c r="N10" s="4" t="n"/>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1901,7 +1921,7 @@
         </is>
       </c>
       <c r="V10" s="4" t="n">
-        <v>14699</v>
+        <v>14257</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>89</v>
@@ -1951,16 +1971,16 @@
       <c r="N11" s="7" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V11" s="7" t="n">
-        <v>81268</v>
+        <v>14081</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>11</v>
@@ -2010,16 +2030,16 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>80831</v>
+        <v>14699</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>40</v>
@@ -2069,16 +2089,16 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>84226</v>
+        <v>14545</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>22</v>
@@ -2133,11 +2153,11 @@
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>693</v>
+        <v>81268</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>12</v>
@@ -2192,11 +2212,11 @@
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>688</v>
+        <v>80831</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>66</v>
@@ -2251,11 +2271,11 @@
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>730</v>
+        <v>84226</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>3</v>
@@ -2305,16 +2325,16 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>48099</v>
+        <v>83820</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>84</v>
@@ -2364,16 +2384,16 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>47253</v>
+        <v>693</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>11</v>
@@ -2423,16 +2443,16 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>49786</v>
+        <v>688</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>48</v>
@@ -2482,16 +2502,16 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>1</v>
+        <v>730</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>16</v>
@@ -2541,16 +2561,16 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>1</v>
+        <v>680</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>10</v>
@@ -2605,11 +2625,11 @@
       </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>1</v>
+        <v>48099</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>60</v>
@@ -2664,11 +2684,11 @@
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>1</v>
+        <v>47253</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>7</v>
@@ -2723,11 +2743,11 @@
       </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>1</v>
+        <v>49786</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2777,20 +2797,30 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>10611</v>
-      </c>
-      <c r="X25" s="7" t="n"/>
-      <c r="Y25" s="7" t="n"/>
-      <c r="Z25" s="7" t="n"/>
+        <v>48589</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>83</v>
+      </c>
+      <c r="Y25" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z25" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB25" s="7" t="n">
         <v>3</v>
       </c>
@@ -2831,15 +2861,25 @@
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>10454</v>
-      </c>
-      <c r="X26" s="4" t="n"/>
-      <c r="Y26" s="4" t="n"/>
-      <c r="Z26" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X26" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB26" s="4" t="n">
         <v>5</v>
       </c>
@@ -2880,15 +2920,25 @@
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>10645</v>
-      </c>
-      <c r="X27" s="7" t="n"/>
-      <c r="Y27" s="7" t="n"/>
-      <c r="Z27" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="Y27" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z27" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB27" s="7" t="n">
         <v>3</v>
       </c>
@@ -2924,23 +2974,43 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z28" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V28" s="4" t="n">
-        <v>23698</v>
-      </c>
-      <c r="X28" s="4" t="n"/>
-      <c r="Y28" s="4" t="n"/>
-      <c r="Z28" s="4" t="n"/>
-      <c r="AB28" s="4" t="n"/>
-      <c r="AC28" s="4" t="n"/>
-      <c r="AD28" s="4" t="n"/>
+      <c r="AB28" s="4" t="n">
+        <v>478</v>
+      </c>
+      <c r="AC28" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD28" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -2963,23 +3033,43 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>22677</v>
-      </c>
-      <c r="X29" s="7" t="n"/>
-      <c r="Y29" s="7" t="n"/>
-      <c r="Z29" s="7" t="n"/>
-      <c r="AB29" s="7" t="n"/>
-      <c r="AC29" s="7" t="n"/>
-      <c r="AD29" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z29" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB29" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="AC29" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD29" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -3002,23 +3092,43 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>24762</v>
-      </c>
-      <c r="X30" s="4" t="n"/>
-      <c r="Y30" s="4" t="n"/>
-      <c r="Z30" s="4" t="n"/>
-      <c r="AB30" s="4" t="n"/>
-      <c r="AC30" s="4" t="n"/>
-      <c r="AD30" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X30" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z30" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB30" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="AC30" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD30" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -3041,23 +3151,43 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>17282</v>
-      </c>
-      <c r="X31" s="7" t="n"/>
-      <c r="Y31" s="7" t="n"/>
-      <c r="Z31" s="7" t="n"/>
-      <c r="AB31" s="7" t="n"/>
-      <c r="AC31" s="7" t="n"/>
-      <c r="AD31" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X31" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z31" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB31" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="AC31" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD31" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -3080,23 +3210,43 @@
       <c r="N32" s="4" t="n"/>
       <c r="T32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>17424</v>
-      </c>
-      <c r="X32" s="4" t="n"/>
-      <c r="Y32" s="4" t="n"/>
-      <c r="Z32" s="4" t="n"/>
-      <c r="AB32" s="4" t="n"/>
-      <c r="AC32" s="4" t="n"/>
-      <c r="AD32" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="AB32" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="AC32" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD32" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="D33" s="24" t="n"/>
@@ -3128,27 +3278,37 @@
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>17603</v>
+        <v>10611</v>
       </c>
       <c r="X33" s="7" t="n"/>
       <c r="Y33" s="7" t="n"/>
       <c r="Z33" s="7" t="n"/>
-      <c r="AB33" s="7" t="n"/>
-      <c r="AC33" s="7" t="n"/>
-      <c r="AD33" s="7" t="n"/>
+      <c r="AB33" s="7" t="n">
+        <v>251</v>
+      </c>
+      <c r="AC33" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD33" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D4)</f>
+        <f>AVERAGE(D2:D5)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3158,7 +3318,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H4)</f>
+        <f>AVERAGE(H2:H5)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3181,65 +3341,95 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>721</v>
+        <v>10454</v>
       </c>
       <c r="X34" s="4" t="n"/>
       <c r="Y34" s="4" t="n"/>
       <c r="Z34" s="4" t="n"/>
-      <c r="AB34" s="4" t="n"/>
-      <c r="AC34" s="4" t="n"/>
-      <c r="AD34" s="4" t="n"/>
+      <c r="AB34" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC34" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD34" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>705</v>
+        <v>10645</v>
       </c>
       <c r="X35" s="7" t="n"/>
       <c r="Y35" s="7" t="n"/>
       <c r="Z35" s="7" t="n"/>
-      <c r="AB35" s="7" t="n"/>
-      <c r="AC35" s="7" t="n"/>
-      <c r="AD35" s="7" t="n"/>
+      <c r="AB35" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="AC35" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD35" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="T36" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>702</v>
+        <v>10506</v>
       </c>
       <c r="X36" s="4" t="n"/>
       <c r="Y36" s="4" t="n"/>
       <c r="Z36" s="4" t="n"/>
-      <c r="AB36" s="4" t="n"/>
-      <c r="AC36" s="4" t="n"/>
-      <c r="AD36" s="4" t="n"/>
+      <c r="AB36" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC36" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="AD36" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="T37" s="7" t="inlineStr">
@@ -3249,11 +3439,11 @@
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>2009</v>
+        <v>23698</v>
       </c>
       <c r="X37" s="7" t="n"/>
       <c r="Y37" s="7" t="n"/>
@@ -3270,11 +3460,11 @@
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>2036</v>
+        <v>22677</v>
       </c>
       <c r="X38" s="4" t="n"/>
       <c r="Y38" s="4" t="n"/>
@@ -3291,11 +3481,11 @@
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
-        <v>2188</v>
+        <v>24762</v>
       </c>
       <c r="X39" s="7" t="n"/>
       <c r="Y39" s="7" t="n"/>
@@ -3303,6 +3493,279 @@
       <c r="AB39" s="7" t="n"/>
       <c r="AC39" s="7" t="n"/>
       <c r="AD39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="n">
+        <v>24562</v>
+      </c>
+      <c r="X40" s="4" t="n"/>
+      <c r="Y40" s="4" t="n"/>
+      <c r="Z40" s="4" t="n"/>
+      <c r="AB40" s="4" t="n"/>
+      <c r="AC40" s="4" t="n"/>
+      <c r="AD40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="T41" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U41" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V41" s="7" t="n">
+        <v>17282</v>
+      </c>
+      <c r="X41" s="7" t="n"/>
+      <c r="Y41" s="7" t="n"/>
+      <c r="Z41" s="7" t="n"/>
+      <c r="AB41" s="7" t="n"/>
+      <c r="AC41" s="7" t="n"/>
+      <c r="AD41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="T42" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U42" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V42" s="4" t="n">
+        <v>17424</v>
+      </c>
+      <c r="X42" s="4" t="n"/>
+      <c r="Y42" s="4" t="n"/>
+      <c r="Z42" s="4" t="n"/>
+      <c r="AB42" s="4" t="n"/>
+      <c r="AC42" s="4" t="n"/>
+      <c r="AD42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="T43" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U43" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V43" s="7" t="n">
+        <v>17603</v>
+      </c>
+      <c r="X43" s="7" t="n"/>
+      <c r="Y43" s="7" t="n"/>
+      <c r="Z43" s="7" t="n"/>
+      <c r="AB43" s="7" t="n"/>
+      <c r="AC43" s="7" t="n"/>
+      <c r="AD43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="T44" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="n">
+        <v>17696</v>
+      </c>
+      <c r="X44" s="4" t="n"/>
+      <c r="Y44" s="4" t="n"/>
+      <c r="Z44" s="4" t="n"/>
+      <c r="AB44" s="4" t="n"/>
+      <c r="AC44" s="4" t="n"/>
+      <c r="AD44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="T45" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U45" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V45" s="7" t="n">
+        <v>721</v>
+      </c>
+      <c r="X45" s="7" t="n"/>
+      <c r="Y45" s="7" t="n"/>
+      <c r="Z45" s="7" t="n"/>
+      <c r="AB45" s="7" t="n"/>
+      <c r="AC45" s="7" t="n"/>
+      <c r="AD45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="T46" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U46" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V46" s="4" t="n">
+        <v>705</v>
+      </c>
+      <c r="X46" s="4" t="n"/>
+      <c r="Y46" s="4" t="n"/>
+      <c r="Z46" s="4" t="n"/>
+      <c r="AB46" s="4" t="n"/>
+      <c r="AC46" s="4" t="n"/>
+      <c r="AD46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="T47" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U47" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V47" s="7" t="n">
+        <v>702</v>
+      </c>
+      <c r="X47" s="7" t="n"/>
+      <c r="Y47" s="7" t="n"/>
+      <c r="Z47" s="7" t="n"/>
+      <c r="AB47" s="7" t="n"/>
+      <c r="AC47" s="7" t="n"/>
+      <c r="AD47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="T48" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U48" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V48" s="4" t="n">
+        <v>799</v>
+      </c>
+      <c r="X48" s="4" t="n"/>
+      <c r="Y48" s="4" t="n"/>
+      <c r="Z48" s="4" t="n"/>
+      <c r="AB48" s="4" t="n"/>
+      <c r="AC48" s="4" t="n"/>
+      <c r="AD48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="T49" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U49" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V49" s="7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="X49" s="7" t="n"/>
+      <c r="Y49" s="7" t="n"/>
+      <c r="Z49" s="7" t="n"/>
+      <c r="AB49" s="7" t="n"/>
+      <c r="AC49" s="7" t="n"/>
+      <c r="AD49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="T50" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U50" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V50" s="4" t="n">
+        <v>2036</v>
+      </c>
+      <c r="X50" s="4" t="n"/>
+      <c r="Y50" s="4" t="n"/>
+      <c r="Z50" s="4" t="n"/>
+      <c r="AB50" s="4" t="n"/>
+      <c r="AC50" s="4" t="n"/>
+      <c r="AD50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="T51" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U51" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V51" s="7" t="n">
+        <v>2188</v>
+      </c>
+      <c r="X51" s="7" t="n"/>
+      <c r="Y51" s="7" t="n"/>
+      <c r="Z51" s="7" t="n"/>
+      <c r="AB51" s="7" t="n"/>
+      <c r="AC51" s="7" t="n"/>
+      <c r="AD51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="T52" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U52" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V52" s="4" t="n">
+        <v>2179</v>
+      </c>
+      <c r="X52" s="4" t="n"/>
+      <c r="Y52" s="4" t="n"/>
+      <c r="Z52" s="4" t="n"/>
+      <c r="AB52" s="4" t="n"/>
+      <c r="AC52" s="4" t="n"/>
+      <c r="AD52" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Removed July's data as its already published
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -710,10 +710,10 @@
         <v>77.40000000000001</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.88</v>
@@ -746,10 +746,10 @@
         <v>80.7</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0.88</v>
@@ -782,10 +782,10 @@
         <v>77.5</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0.88</v>
@@ -818,10 +818,10 @@
         <v>67.8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0.88</v>
@@ -854,10 +854,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0.88</v>
@@ -890,10 +890,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.88</v>
@@ -926,10 +926,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.88</v>
@@ -962,10 +962,10 @@
         <v>77.2</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.88</v>
@@ -998,10 +998,10 @@
         <v>67.7</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0.88</v>
@@ -1034,10 +1034,10 @@
         <v>67.7</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4.52</v>
+        <v>3.93</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.88</v>

</xml_diff>

<commit_message>
Added new release for the week
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -716,7 +716,7 @@
         <v>1.2</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>1.27</v>
@@ -752,7 +752,7 @@
         <v>1.2</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>1.27</v>
@@ -788,7 +788,7 @@
         <v>1.2</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>1.27</v>
@@ -824,7 +824,7 @@
         <v>1.2</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>1.27</v>
@@ -860,7 +860,7 @@
         <v>1.2</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>1.27</v>
@@ -896,7 +896,7 @@
         <v>1.2</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>1.27</v>
@@ -932,7 +932,7 @@
         <v>1.2</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>1.27</v>
@@ -968,7 +968,7 @@
         <v>1.2</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>1.27</v>
@@ -1004,7 +1004,7 @@
         <v>1.2</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>1.27</v>
@@ -1040,7 +1040,7 @@
         <v>1.2</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>1.27</v>
@@ -1170,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD78"/>
+  <dimension ref="A1:AD130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1813,29 +1813,49 @@
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
+      <c r="D8" s="4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C8)</f>
+        <v/>
+      </c>
       <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
+      <c r="G8" s="4">
+        <f>ROUND(MAX(0,MIN(100,(1-E8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>MIN(1,(G8-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4" t="n"/>
+      <c r="K8" s="4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K8/IF(D8&gt;0,D8,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>MAX(0,(L8-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>$B$2+H8+M8</f>
+        <v/>
+      </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U8" s="4" t="inlineStr"/>
       <c r="V8" s="4" t="n">
-        <v>5034</v>
+        <v>1</v>
       </c>
       <c r="X8" s="4" t="n">
         <v>5</v>
@@ -1872,29 +1892,49 @@
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
+      <c r="D9" s="7">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C9)</f>
+        <v/>
+      </c>
       <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="G9" s="7">
+        <f>ROUND(MAX(0,MIN(100,(1-E9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7">
+        <f>MIN(1,(G9-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
+      <c r="K9" s="7">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K9/IF(D9&gt;0,D9,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>MAX(0,(L9-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="7">
+        <f>$B$2+H9+M9</f>
+        <v/>
+      </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="U9" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U9" s="7" t="inlineStr"/>
       <c r="V9" s="7" t="n">
-        <v>4901</v>
+        <v>1</v>
       </c>
       <c r="X9" s="7" t="n">
         <v>3</v>
@@ -1939,29 +1979,49 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
+      <c r="D10" s="4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C10)</f>
+        <v/>
+      </c>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
+      <c r="G10" s="4">
+        <f>ROUND(MAX(0,MIN(100,(1-E10/IF(D10&gt;0,D10,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>MIN(1,(G10-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="n"/>
-      <c r="L10" s="4" t="n"/>
-      <c r="M10" s="4" t="n"/>
-      <c r="N10" s="4" t="n"/>
+      <c r="K10" s="4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K10/IF(D10&gt;0,D10,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M10" s="4">
+        <f>MAX(0,(L10-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N10" s="4">
+        <f>$B$2+H10+M10</f>
+        <v/>
+      </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U10" s="4" t="inlineStr"/>
       <c r="V10" s="4" t="n">
-        <v>5271</v>
+        <v>1</v>
       </c>
       <c r="X10" s="4" t="n">
         <v>89</v>
@@ -1998,29 +2058,49 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
+      <c r="D11" s="7">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="7">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C11)</f>
+        <v/>
+      </c>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="G11" s="7">
+        <f>ROUND(MAX(0,MIN(100,(1-E11/IF(D11&gt;0,D11,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H11" s="7">
+        <f>MIN(1,(G11-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
+      <c r="K11" s="7">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="7">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K11/IF(D11&gt;0,D11,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/31)))),2)</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>MAX(0,(L11-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N11" s="7">
+        <f>$B$2+H11+M11</f>
+        <v/>
+      </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="U11" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U11" s="7" t="inlineStr"/>
       <c r="V11" s="7" t="n">
-        <v>5154</v>
+        <v>1</v>
       </c>
       <c r="X11" s="7" t="n">
         <v>11</v>
@@ -2070,7 +2150,7 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
@@ -2079,7 +2159,7 @@
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>5294</v>
+        <v>5034</v>
       </c>
       <c r="X12" s="4" t="n">
         <v>40</v>
@@ -2129,7 +2209,7 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
@@ -2138,7 +2218,7 @@
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>5390</v>
+        <v>4901</v>
       </c>
       <c r="X13" s="7" t="n">
         <v>22</v>
@@ -2188,16 +2268,16 @@
       <c r="N14" s="4" t="n"/>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>14257</v>
+        <v>5271</v>
       </c>
       <c r="X14" s="4" t="n">
         <v>12</v>
@@ -2247,16 +2327,16 @@
       <c r="N15" s="7" t="n"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>14081</v>
+        <v>5154</v>
       </c>
       <c r="X15" s="7" t="n">
         <v>66</v>
@@ -2306,16 +2386,16 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V16" s="4" t="n">
-        <v>14699</v>
+        <v>5294</v>
       </c>
       <c r="X16" s="4" t="n">
         <v>3</v>
@@ -2365,16 +2445,16 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V17" s="7" t="n">
-        <v>14545</v>
+        <v>5390</v>
       </c>
       <c r="X17" s="7" t="n">
         <v>85</v>
@@ -2424,16 +2504,16 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>15288</v>
+        <v>5357</v>
       </c>
       <c r="X18" s="4" t="n">
         <v>11</v>
@@ -2483,16 +2563,16 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>14676</v>
+        <v>4829</v>
       </c>
       <c r="X19" s="7" t="n">
         <v>48</v>
@@ -2542,16 +2622,16 @@
       <c r="N20" s="4" t="n"/>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>81268</v>
+        <v>4770</v>
       </c>
       <c r="X20" s="4" t="n">
         <v>16</v>
@@ -2601,16 +2681,16 @@
       <c r="N21" s="7" t="n"/>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>80831</v>
+        <v>4992</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>10</v>
@@ -2660,16 +2740,16 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>84226</v>
+        <v>14257</v>
       </c>
       <c r="X22" s="4" t="n">
         <v>60</v>
@@ -2719,16 +2799,16 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>83820</v>
+        <v>14081</v>
       </c>
       <c r="X23" s="7" t="n">
         <v>7</v>
@@ -2778,16 +2858,16 @@
       <c r="N24" s="4" t="n"/>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V24" s="4" t="n">
-        <v>87306</v>
+        <v>14699</v>
       </c>
       <c r="X24" s="4" t="n">
         <v>1</v>
@@ -2837,16 +2917,16 @@
       <c r="N25" s="7" t="n"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V25" s="7" t="n">
-        <v>83042</v>
+        <v>14545</v>
       </c>
       <c r="X25" s="7" t="n">
         <v>83</v>
@@ -2896,16 +2976,16 @@
       <c r="N26" s="4" t="n"/>
       <c r="T26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V26" s="4" t="n">
-        <v>693</v>
+        <v>15288</v>
       </c>
       <c r="X26" s="4" t="n">
         <v>14</v>
@@ -2955,16 +3035,16 @@
       <c r="N27" s="7" t="n"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V27" s="7" t="n">
-        <v>688</v>
+        <v>14676</v>
       </c>
       <c r="X27" s="7" t="n">
         <v>45</v>
@@ -3014,16 +3094,16 @@
       <c r="N28" s="4" t="n"/>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V28" s="4" t="n">
-        <v>730</v>
+        <v>14651</v>
       </c>
       <c r="X28" s="4" t="n">
         <v>25</v>
@@ -3073,16 +3153,16 @@
       <c r="N29" s="7" t="n"/>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V29" s="7" t="n">
-        <v>680</v>
+        <v>14076</v>
       </c>
       <c r="X29" s="7" t="n">
         <v>7</v>
@@ -3132,16 +3212,16 @@
       <c r="N30" s="4" t="n"/>
       <c r="T30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V30" s="4" t="n">
-        <v>692</v>
+        <v>14200</v>
       </c>
       <c r="X30" s="4" t="n">
         <v>70</v>
@@ -3191,16 +3271,16 @@
       <c r="N31" s="7" t="n"/>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V31" s="7" t="n">
-        <v>682</v>
+        <v>14611</v>
       </c>
       <c r="X31" s="7" t="n">
         <v>2</v>
@@ -3255,11 +3335,11 @@
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V32" s="4" t="n">
-        <v>48099</v>
+        <v>81268</v>
       </c>
       <c r="X32" s="4" t="n">
         <v>1</v>
@@ -3323,11 +3403,11 @@
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V33" s="7" t="n">
-        <v>47253</v>
+        <v>80831</v>
       </c>
       <c r="X33" s="7" t="n">
         <v>76</v>
@@ -3358,7 +3438,7 @@
     </row>
     <row r="34">
       <c r="D34" s="26">
-        <f>AVERAGE(D2:D7)</f>
+        <f>AVERAGE(D2:D11)</f>
         <v/>
       </c>
       <c r="E34" s="27" t="n"/>
@@ -3368,7 +3448,7 @@
         <v/>
       </c>
       <c r="H34" s="29">
-        <f>AVERAGE(H2:H7)</f>
+        <f>AVERAGE(H2:H11)</f>
         <v/>
       </c>
       <c r="I34" s="29">
@@ -3396,11 +3476,11 @@
       </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V34" s="4" t="n">
-        <v>49786</v>
+        <v>84226</v>
       </c>
       <c r="X34" s="4" t="n">
         <v>15</v>
@@ -3437,11 +3517,11 @@
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V35" s="7" t="n">
-        <v>48589</v>
+        <v>83820</v>
       </c>
       <c r="X35" s="7" t="n">
         <v>50</v>
@@ -3478,11 +3558,11 @@
       </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V36" s="4" t="n">
-        <v>48093</v>
+        <v>87306</v>
       </c>
       <c r="X36" s="4" t="n">
         <v>20</v>
@@ -3519,11 +3599,11 @@
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V37" s="7" t="n">
-        <v>49210</v>
+        <v>83042</v>
       </c>
       <c r="X37" s="7" t="n">
         <v>13</v>
@@ -3555,16 +3635,16 @@
     <row r="38">
       <c r="T38" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V38" s="4" t="n">
-        <v>1</v>
+        <v>87128</v>
       </c>
       <c r="X38" s="4" t="n">
         <v>55</v>
@@ -3596,16 +3676,16 @@
     <row r="39">
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V39" s="7" t="n">
-        <v>1</v>
+        <v>81610</v>
       </c>
       <c r="X39" s="7" t="n">
         <v>7</v>
@@ -3637,16 +3717,16 @@
     <row r="40">
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V40" s="4" t="n">
-        <v>1</v>
+        <v>81125</v>
       </c>
       <c r="X40" s="4" t="n">
         <v>1</v>
@@ -3678,16 +3758,16 @@
     <row r="41">
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V41" s="7" t="n">
-        <v>1</v>
+        <v>83339</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>80</v>
@@ -3719,16 +3799,16 @@
     <row r="42">
       <c r="T42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V42" s="4" t="n">
-        <v>1</v>
+        <v>693</v>
       </c>
       <c r="X42" s="4" t="n">
         <v>12</v>
@@ -3760,16 +3840,16 @@
     <row r="43">
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V43" s="7" t="n">
-        <v>1</v>
+        <v>688</v>
       </c>
       <c r="X43" s="7" t="n">
         <v>35</v>
@@ -3801,16 +3881,16 @@
     <row r="44">
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U44" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V44" s="4" t="n">
-        <v>1</v>
+        <v>730</v>
       </c>
       <c r="X44" s="4" t="n">
         <v>18</v>
@@ -3842,16 +3922,16 @@
     <row r="45">
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V45" s="7" t="n">
-        <v>1</v>
+        <v>680</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>11</v>
@@ -3883,16 +3963,16 @@
     <row r="46">
       <c r="T46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="U46" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V46" s="4" t="n">
-        <v>1</v>
+        <v>692</v>
       </c>
       <c r="X46" s="4" t="n">
         <v>70</v>
@@ -3924,16 +4004,16 @@
     <row r="47">
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V47" s="7" t="n">
-        <v>1</v>
+        <v>682</v>
       </c>
       <c r="X47" s="7" t="n">
         <v>1</v>
@@ -3965,16 +4045,16 @@
     <row r="48">
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U48" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V48" s="4" t="n">
-        <v>1</v>
+        <v>692</v>
       </c>
       <c r="X48" s="4" t="n">
         <v>3</v>
@@ -4006,16 +4086,16 @@
     <row r="49">
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V49" s="7" t="n">
-        <v>10611</v>
+        <v>682</v>
       </c>
       <c r="X49" s="7" t="n">
         <v>2</v>
@@ -4047,20 +4127,30 @@
     <row r="50">
       <c r="T50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U50" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V50" s="4" t="n">
-        <v>10454</v>
-      </c>
-      <c r="X50" s="4" t="n"/>
-      <c r="Y50" s="4" t="n"/>
-      <c r="Z50" s="4" t="n"/>
+        <v>680</v>
+      </c>
+      <c r="X50" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="Y50" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z50" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB50" s="4" t="n">
         <v>48</v>
       </c>
@@ -4078,20 +4168,30 @@
     <row r="51">
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V51" s="7" t="n">
-        <v>10645</v>
-      </c>
-      <c r="X51" s="7" t="n"/>
-      <c r="Y51" s="7" t="n"/>
-      <c r="Z51" s="7" t="n"/>
+        <v>729</v>
+      </c>
+      <c r="X51" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y51" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z51" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB51" s="7" t="n">
         <v>231</v>
       </c>
@@ -4109,20 +4209,30 @@
     <row r="52">
       <c r="T52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U52" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V52" s="4" t="n">
-        <v>10506</v>
-      </c>
-      <c r="X52" s="4" t="n"/>
-      <c r="Y52" s="4" t="n"/>
-      <c r="Z52" s="4" t="n"/>
+        <v>48099</v>
+      </c>
+      <c r="X52" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y52" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z52" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB52" s="4" t="n">
         <v>2</v>
       </c>
@@ -4140,20 +4250,30 @@
     <row r="53">
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V53" s="7" t="n">
-        <v>10555</v>
-      </c>
-      <c r="X53" s="7" t="n"/>
-      <c r="Y53" s="7" t="n"/>
-      <c r="Z53" s="7" t="n"/>
+        <v>47253</v>
+      </c>
+      <c r="X53" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y53" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z53" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB53" s="7" t="n">
         <v>13</v>
       </c>
@@ -4171,20 +4291,30 @@
     <row r="54">
       <c r="T54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U54" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="V54" s="4" t="n">
+        <v>49786</v>
+      </c>
+      <c r="X54" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y54" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z54" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
-      <c r="V54" s="4" t="n">
-        <v>10586</v>
-      </c>
-      <c r="X54" s="4" t="n"/>
-      <c r="Y54" s="4" t="n"/>
-      <c r="Z54" s="4" t="n"/>
       <c r="AB54" s="4" t="n">
         <v>3</v>
       </c>
@@ -4202,149 +4332,289 @@
     <row r="55">
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V55" s="7" t="n">
-        <v>23698</v>
-      </c>
-      <c r="X55" s="7" t="n"/>
-      <c r="Y55" s="7" t="n"/>
-      <c r="Z55" s="7" t="n"/>
-      <c r="AB55" s="7" t="n"/>
-      <c r="AC55" s="7" t="n"/>
-      <c r="AD55" s="7" t="n"/>
+        <v>48589</v>
+      </c>
+      <c r="X55" s="7" t="n">
+        <v>81</v>
+      </c>
+      <c r="Y55" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z55" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB55" s="7" t="n">
+        <v>473</v>
+      </c>
+      <c r="AC55" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD55" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="U56" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V56" s="4" t="n">
-        <v>22677</v>
-      </c>
-      <c r="X56" s="4" t="n"/>
-      <c r="Y56" s="4" t="n"/>
-      <c r="Z56" s="4" t="n"/>
-      <c r="AB56" s="4" t="n"/>
-      <c r="AC56" s="4" t="n"/>
-      <c r="AD56" s="4" t="n"/>
+        <v>48093</v>
+      </c>
+      <c r="X56" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB56" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="U57" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V57" s="7" t="n">
-        <v>24762</v>
-      </c>
-      <c r="X57" s="7" t="n"/>
-      <c r="Y57" s="7" t="n"/>
-      <c r="Z57" s="7" t="n"/>
-      <c r="AB57" s="7" t="n"/>
-      <c r="AC57" s="7" t="n"/>
-      <c r="AD57" s="7" t="n"/>
+        <v>49210</v>
+      </c>
+      <c r="X57" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y57" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z57" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+      <c r="AB57" s="7" t="n">
+        <v>178</v>
+      </c>
+      <c r="AC57" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD57" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="T58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U58" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="V58" s="4" t="n">
+        <v>48289</v>
+      </c>
+      <c r="X58" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y58" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z58" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+      <c r="AB58" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="AC58" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD58" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V58" s="4" t="n">
-        <v>24562</v>
-      </c>
-      <c r="X58" s="4" t="n"/>
-      <c r="Y58" s="4" t="n"/>
-      <c r="Z58" s="4" t="n"/>
-      <c r="AB58" s="4" t="n"/>
-      <c r="AC58" s="4" t="n"/>
-      <c r="AD58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V59" s="7" t="n">
-        <v>25273</v>
-      </c>
-      <c r="X59" s="7" t="n"/>
-      <c r="Y59" s="7" t="n"/>
-      <c r="Z59" s="7" t="n"/>
-      <c r="AB59" s="7" t="n"/>
-      <c r="AC59" s="7" t="n"/>
-      <c r="AD59" s="7" t="n"/>
+        <v>47345</v>
+      </c>
+      <c r="X59" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y59" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z59" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="AB59" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="AC59" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD59" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U60" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="V60" s="4" t="n">
+        <v>46830</v>
+      </c>
+      <c r="X60" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y60" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z60" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V60" s="4" t="n">
-        <v>25463</v>
-      </c>
-      <c r="X60" s="4" t="n"/>
-      <c r="Y60" s="4" t="n"/>
-      <c r="Z60" s="4" t="n"/>
-      <c r="AB60" s="4" t="n"/>
-      <c r="AC60" s="4" t="n"/>
-      <c r="AD60" s="4" t="n"/>
+      <c r="AB60" s="4" t="n">
+        <v>201</v>
+      </c>
+      <c r="AC60" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD60" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V61" s="7" t="n">
-        <v>17282</v>
-      </c>
-      <c r="X61" s="7" t="n"/>
-      <c r="Y61" s="7" t="n"/>
-      <c r="Z61" s="7" t="n"/>
-      <c r="AB61" s="7" t="n"/>
-      <c r="AC61" s="7" t="n"/>
-      <c r="AD61" s="7" t="n"/>
+        <v>49033</v>
+      </c>
+      <c r="X61" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y61" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z61" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB61" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC61" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD61" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="T62" s="4" t="inlineStr">
@@ -4354,18 +4624,38 @@
       </c>
       <c r="U62" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V62" s="4" t="n">
-        <v>17424</v>
-      </c>
-      <c r="X62" s="4" t="n"/>
-      <c r="Y62" s="4" t="n"/>
-      <c r="Z62" s="4" t="n"/>
-      <c r="AB62" s="4" t="n"/>
-      <c r="AC62" s="4" t="n"/>
-      <c r="AD62" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X62" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="Y62" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z62" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB62" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC62" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD62" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="T63" s="7" t="inlineStr">
@@ -4375,18 +4665,38 @@
       </c>
       <c r="U63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V63" s="7" t="n">
-        <v>17603</v>
-      </c>
-      <c r="X63" s="7" t="n"/>
-      <c r="Y63" s="7" t="n"/>
-      <c r="Z63" s="7" t="n"/>
-      <c r="AB63" s="7" t="n"/>
-      <c r="AC63" s="7" t="n"/>
-      <c r="AD63" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X63" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y63" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z63" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB63" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC63" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="AD63" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="T64" s="4" t="inlineStr">
@@ -4396,18 +4706,38 @@
       </c>
       <c r="U64" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V64" s="4" t="n">
-        <v>17696</v>
-      </c>
-      <c r="X64" s="4" t="n"/>
-      <c r="Y64" s="4" t="n"/>
-      <c r="Z64" s="4" t="n"/>
-      <c r="AB64" s="4" t="n"/>
-      <c r="AC64" s="4" t="n"/>
-      <c r="AD64" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X64" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y64" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="Z64" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="AB64" s="4" t="n">
+        <v>445</v>
+      </c>
+      <c r="AC64" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD64" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="T65" s="7" t="inlineStr">
@@ -4417,18 +4747,38 @@
       </c>
       <c r="U65" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V65" s="7" t="n">
-        <v>17579</v>
-      </c>
-      <c r="X65" s="7" t="n"/>
-      <c r="Y65" s="7" t="n"/>
-      <c r="Z65" s="7" t="n"/>
-      <c r="AB65" s="7" t="n"/>
-      <c r="AC65" s="7" t="n"/>
-      <c r="AD65" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X65" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="Y65" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z65" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+      <c r="AB65" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="AC65" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD65" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="T66" s="4" t="inlineStr">
@@ -4438,270 +4788,1732 @@
       </c>
       <c r="U66" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+        </is>
+      </c>
+      <c r="V66" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X66" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y66" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z66" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+      <c r="AB66" s="4" t="n">
+        <v>176</v>
+      </c>
+      <c r="AC66" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD66" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.talabat</t>
         </is>
       </c>
-      <c r="V66" s="4" t="n">
-        <v>17878</v>
-      </c>
-      <c r="X66" s="4" t="n"/>
-      <c r="Y66" s="4" t="n"/>
-      <c r="Z66" s="4" t="n"/>
-      <c r="AB66" s="4" t="n"/>
-      <c r="AC66" s="4" t="n"/>
-      <c r="AD66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="T67" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U67" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V67" s="7" t="n">
-        <v>721</v>
-      </c>
-      <c r="X67" s="7" t="n"/>
-      <c r="Y67" s="7" t="n"/>
-      <c r="Z67" s="7" t="n"/>
-      <c r="AB67" s="7" t="n"/>
-      <c r="AC67" s="7" t="n"/>
-      <c r="AD67" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X67" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y67" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z67" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="AB67" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="AC67" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD67" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="T68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="U68" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V68" s="4" t="n">
-        <v>705</v>
-      </c>
-      <c r="X68" s="4" t="n"/>
-      <c r="Y68" s="4" t="n"/>
-      <c r="Z68" s="4" t="n"/>
-      <c r="AB68" s="4" t="n"/>
-      <c r="AC68" s="4" t="n"/>
-      <c r="AD68" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X68" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y68" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z68" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="AB68" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="AC68" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD68" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="T69" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="U69" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
         </is>
       </c>
       <c r="V69" s="7" t="n">
-        <v>702</v>
-      </c>
-      <c r="X69" s="7" t="n"/>
-      <c r="Y69" s="7" t="n"/>
-      <c r="Z69" s="7" t="n"/>
-      <c r="AB69" s="7" t="n"/>
-      <c r="AC69" s="7" t="n"/>
-      <c r="AD69" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X69" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y69" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z69" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB69" s="7" t="n">
+        <v>194</v>
+      </c>
+      <c r="AC69" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD69" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="U70" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo.8PDW8D52VJ</t>
+        </is>
+      </c>
+      <c r="V70" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X70" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y70" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z70" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB70" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC70" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD70" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.woowabros</t>
         </is>
       </c>
-      <c r="V70" s="4" t="n">
-        <v>799</v>
-      </c>
-      <c r="X70" s="4" t="n"/>
-      <c r="Y70" s="4" t="n"/>
-      <c r="Z70" s="4" t="n"/>
-      <c r="AB70" s="4" t="n"/>
-      <c r="AC70" s="4" t="n"/>
-      <c r="AD70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="T71" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="U71" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V71" s="7" t="n">
-        <v>746</v>
-      </c>
-      <c r="X71" s="7" t="n"/>
-      <c r="Y71" s="7" t="n"/>
-      <c r="Z71" s="7" t="n"/>
-      <c r="AB71" s="7" t="n"/>
-      <c r="AC71" s="7" t="n"/>
-      <c r="AD71" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X71" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y71" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="Z71" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB71" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="AC71" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD71" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="U72" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V72" s="4" t="n">
-        <v>752</v>
-      </c>
-      <c r="X72" s="4" t="n"/>
-      <c r="Y72" s="4" t="n"/>
-      <c r="Z72" s="4" t="n"/>
-      <c r="AB72" s="4" t="n"/>
-      <c r="AC72" s="4" t="n"/>
-      <c r="AD72" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X72" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y72" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z72" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+      <c r="AB72" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC72" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AD72" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="T73" s="7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="U73" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V73" s="7" t="n">
-        <v>2009</v>
-      </c>
-      <c r="X73" s="7" t="n"/>
-      <c r="Y73" s="7" t="n"/>
-      <c r="Z73" s="7" t="n"/>
-      <c r="AB73" s="7" t="n"/>
-      <c r="AC73" s="7" t="n"/>
-      <c r="AD73" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X73" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y73" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z73" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+      <c r="AB73" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="AC73" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD73" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="T74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U74" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V74" s="4" t="n">
-        <v>2036</v>
-      </c>
-      <c r="X74" s="4" t="n"/>
-      <c r="Y74" s="4" t="n"/>
-      <c r="Z74" s="4" t="n"/>
-      <c r="AB74" s="4" t="n"/>
-      <c r="AC74" s="4" t="n"/>
-      <c r="AD74" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X74" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="Y74" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z74" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="AB74" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="AC74" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD74" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="T75" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="U75" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V75" s="7" t="n">
-        <v>2188</v>
-      </c>
-      <c r="X75" s="7" t="n"/>
-      <c r="Y75" s="7" t="n"/>
-      <c r="Z75" s="7" t="n"/>
-      <c r="AB75" s="7" t="n"/>
-      <c r="AC75" s="7" t="n"/>
-      <c r="AD75" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X75" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="Y75" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z75" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="AB75" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="AC75" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD75" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="T76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="U76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V76" s="4" t="n">
-        <v>2179</v>
-      </c>
-      <c r="X76" s="4" t="n"/>
-      <c r="Y76" s="4" t="n"/>
-      <c r="Z76" s="4" t="n"/>
-      <c r="AB76" s="4" t="n"/>
-      <c r="AC76" s="4" t="n"/>
-      <c r="AD76" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X76" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y76" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z76" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB76" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="AC76" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD76" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="T77" s="7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="U77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
         </is>
       </c>
       <c r="V77" s="7" t="n">
-        <v>2371</v>
-      </c>
-      <c r="X77" s="7" t="n"/>
-      <c r="Y77" s="7" t="n"/>
-      <c r="Z77" s="7" t="n"/>
-      <c r="AB77" s="7" t="n"/>
-      <c r="AC77" s="7" t="n"/>
-      <c r="AD77" s="7" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X77" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="Y77" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z77" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB77" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="AC77" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD77" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="T78" s="4" t="inlineStr">
         <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U78" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V78" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X78" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y78" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="Z78" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="AB78" s="4" t="n">
+        <v>199</v>
+      </c>
+      <c r="AC78" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD78" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="T79" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U79" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V79" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="X79" s="7" t="n"/>
+      <c r="Y79" s="7" t="n"/>
+      <c r="Z79" s="7" t="n"/>
+      <c r="AB79" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="AC79" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD79" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="T80" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U80" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo.GAB3RR77LN</t>
+        </is>
+      </c>
+      <c r="V80" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X80" s="4" t="n"/>
+      <c r="Y80" s="4" t="n"/>
+      <c r="Z80" s="4" t="n"/>
+      <c r="AB80" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC80" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="AD80" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="T81" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U81" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V81" s="7" t="n">
+        <v>10611</v>
+      </c>
+      <c r="X81" s="7" t="n"/>
+      <c r="Y81" s="7" t="n"/>
+      <c r="Z81" s="7" t="n"/>
+      <c r="AB81" s="7" t="n">
+        <v>463</v>
+      </c>
+      <c r="AC81" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD81" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="T82" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U82" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V82" s="4" t="n">
+        <v>10454</v>
+      </c>
+      <c r="X82" s="4" t="n"/>
+      <c r="Y82" s="4" t="n"/>
+      <c r="Z82" s="4" t="n"/>
+      <c r="AB82" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="AC82" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD82" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="T83" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U83" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V83" s="7" t="n">
+        <v>10645</v>
+      </c>
+      <c r="X83" s="7" t="n"/>
+      <c r="Y83" s="7" t="n"/>
+      <c r="Z83" s="7" t="n"/>
+      <c r="AB83" s="7" t="n">
+        <v>158</v>
+      </c>
+      <c r="AC83" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD83" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="T84" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U84" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V84" s="4" t="n">
+        <v>10506</v>
+      </c>
+      <c r="X84" s="4" t="n"/>
+      <c r="Y84" s="4" t="n"/>
+      <c r="Z84" s="4" t="n"/>
+      <c r="AB84" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="AC84" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD84" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="T85" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="U85" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V85" s="7" t="n">
+        <v>10555</v>
+      </c>
+      <c r="X85" s="7" t="n"/>
+      <c r="Y85" s="7" t="n"/>
+      <c r="Z85" s="7" t="n"/>
+      <c r="AB85" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="AC85" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD85" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="T86" s="4" t="inlineStr">
+        <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="U78" s="4" t="inlineStr">
+      <c r="U86" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V86" s="4" t="n">
+        <v>10586</v>
+      </c>
+      <c r="X86" s="4" t="n"/>
+      <c r="Y86" s="4" t="n"/>
+      <c r="Z86" s="4" t="n"/>
+      <c r="AB86" s="4" t="n">
+        <v>195</v>
+      </c>
+      <c r="AC86" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD86" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="T87" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U87" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V87" s="7" t="n">
+        <v>10346</v>
+      </c>
+      <c r="X87" s="7" t="n"/>
+      <c r="Y87" s="7" t="n"/>
+      <c r="Z87" s="7" t="n"/>
+      <c r="AB87" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC87" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD87" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="T88" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U88" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V88" s="4" t="n">
+        <v>10451</v>
+      </c>
+      <c r="X88" s="4" t="n"/>
+      <c r="Y88" s="4" t="n"/>
+      <c r="Z88" s="4" t="n"/>
+      <c r="AB88" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC88" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD88" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="T89" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U89" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V89" s="7" t="n">
+        <v>10531</v>
+      </c>
+      <c r="X89" s="7" t="n"/>
+      <c r="Y89" s="7" t="n"/>
+      <c r="Z89" s="7" t="n"/>
+      <c r="AB89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC89" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="AD89" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="T90" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U90" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="V90" s="4" t="n">
+        <v>10562</v>
+      </c>
+      <c r="X90" s="4" t="n"/>
+      <c r="Y90" s="4" t="n"/>
+      <c r="Z90" s="4" t="n"/>
+      <c r="AB90" s="4" t="n"/>
+      <c r="AC90" s="4" t="n"/>
+      <c r="AD90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="T91" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U91" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V91" s="7" t="n">
+        <v>23698</v>
+      </c>
+      <c r="X91" s="7" t="n"/>
+      <c r="Y91" s="7" t="n"/>
+      <c r="Z91" s="7" t="n"/>
+      <c r="AB91" s="7" t="n"/>
+      <c r="AC91" s="7" t="n"/>
+      <c r="AD91" s="7" t="n"/>
+    </row>
+    <row r="92">
+      <c r="T92" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U92" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V92" s="4" t="n">
+        <v>22677</v>
+      </c>
+      <c r="X92" s="4" t="n"/>
+      <c r="Y92" s="4" t="n"/>
+      <c r="Z92" s="4" t="n"/>
+      <c r="AB92" s="4" t="n"/>
+      <c r="AC92" s="4" t="n"/>
+      <c r="AD92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="T93" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U93" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V93" s="7" t="n">
+        <v>24762</v>
+      </c>
+      <c r="X93" s="7" t="n"/>
+      <c r="Y93" s="7" t="n"/>
+      <c r="Z93" s="7" t="n"/>
+      <c r="AB93" s="7" t="n"/>
+      <c r="AC93" s="7" t="n"/>
+      <c r="AD93" s="7" t="n"/>
+    </row>
+    <row r="94">
+      <c r="T94" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U94" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V94" s="4" t="n">
+        <v>24562</v>
+      </c>
+      <c r="X94" s="4" t="n"/>
+      <c r="Y94" s="4" t="n"/>
+      <c r="Z94" s="4" t="n"/>
+      <c r="AB94" s="4" t="n"/>
+      <c r="AC94" s="4" t="n"/>
+      <c r="AD94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="T95" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="U95" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V95" s="7" t="n">
+        <v>25273</v>
+      </c>
+      <c r="X95" s="7" t="n"/>
+      <c r="Y95" s="7" t="n"/>
+      <c r="Z95" s="7" t="n"/>
+      <c r="AB95" s="7" t="n"/>
+      <c r="AC95" s="7" t="n"/>
+      <c r="AD95" s="7" t="n"/>
+    </row>
+    <row r="96">
+      <c r="T96" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="U96" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V96" s="4" t="n">
+        <v>25463</v>
+      </c>
+      <c r="X96" s="4" t="n"/>
+      <c r="Y96" s="4" t="n"/>
+      <c r="Z96" s="4" t="n"/>
+      <c r="AB96" s="4" t="n"/>
+      <c r="AC96" s="4" t="n"/>
+      <c r="AD96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="T97" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U97" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V97" s="7" t="n">
+        <v>24938</v>
+      </c>
+      <c r="X97" s="7" t="n"/>
+      <c r="Y97" s="7" t="n"/>
+      <c r="Z97" s="7" t="n"/>
+      <c r="AB97" s="7" t="n"/>
+      <c r="AC97" s="7" t="n"/>
+      <c r="AD97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="T98" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U98" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V98" s="4" t="n">
+        <v>23708</v>
+      </c>
+      <c r="X98" s="4" t="n"/>
+      <c r="Y98" s="4" t="n"/>
+      <c r="Z98" s="4" t="n"/>
+      <c r="AB98" s="4" t="n"/>
+      <c r="AC98" s="4" t="n"/>
+      <c r="AD98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="T99" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U99" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V99" s="7" t="n">
+        <v>23206</v>
+      </c>
+      <c r="X99" s="7" t="n"/>
+      <c r="Y99" s="7" t="n"/>
+      <c r="Z99" s="7" t="n"/>
+      <c r="AB99" s="7" t="n"/>
+      <c r="AC99" s="7" t="n"/>
+      <c r="AD99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="T100" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U100" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V100" s="4" t="n">
+        <v>25336</v>
+      </c>
+      <c r="X100" s="4" t="n"/>
+      <c r="Y100" s="4" t="n"/>
+      <c r="Z100" s="4" t="n"/>
+      <c r="AB100" s="4" t="n"/>
+      <c r="AC100" s="4" t="n"/>
+      <c r="AD100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="T101" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U101" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V101" s="7" t="n">
+        <v>17282</v>
+      </c>
+      <c r="X101" s="7" t="n"/>
+      <c r="Y101" s="7" t="n"/>
+      <c r="Z101" s="7" t="n"/>
+      <c r="AB101" s="7" t="n"/>
+      <c r="AC101" s="7" t="n"/>
+      <c r="AD101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="T102" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U102" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V102" s="4" t="n">
+        <v>17424</v>
+      </c>
+      <c r="X102" s="4" t="n"/>
+      <c r="Y102" s="4" t="n"/>
+      <c r="Z102" s="4" t="n"/>
+      <c r="AB102" s="4" t="n"/>
+      <c r="AC102" s="4" t="n"/>
+      <c r="AD102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="T103" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U103" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V103" s="7" t="n">
+        <v>17603</v>
+      </c>
+      <c r="X103" s="7" t="n"/>
+      <c r="Y103" s="7" t="n"/>
+      <c r="Z103" s="7" t="n"/>
+      <c r="AB103" s="7" t="n"/>
+      <c r="AC103" s="7" t="n"/>
+      <c r="AD103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="T104" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U104" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V104" s="4" t="n">
+        <v>17696</v>
+      </c>
+      <c r="X104" s="4" t="n"/>
+      <c r="Y104" s="4" t="n"/>
+      <c r="Z104" s="4" t="n"/>
+      <c r="AB104" s="4" t="n"/>
+      <c r="AC104" s="4" t="n"/>
+      <c r="AD104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="T105" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="U105" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V105" s="7" t="n">
+        <v>17579</v>
+      </c>
+      <c r="X105" s="7" t="n"/>
+      <c r="Y105" s="7" t="n"/>
+      <c r="Z105" s="7" t="n"/>
+      <c r="AB105" s="7" t="n"/>
+      <c r="AC105" s="7" t="n"/>
+      <c r="AD105" s="7" t="n"/>
+    </row>
+    <row r="106">
+      <c r="T106" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="U106" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V106" s="4" t="n">
+        <v>17878</v>
+      </c>
+      <c r="X106" s="4" t="n"/>
+      <c r="Y106" s="4" t="n"/>
+      <c r="Z106" s="4" t="n"/>
+      <c r="AB106" s="4" t="n"/>
+      <c r="AC106" s="4" t="n"/>
+      <c r="AD106" s="4" t="n"/>
+    </row>
+    <row r="107">
+      <c r="T107" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U107" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V107" s="7" t="n">
+        <v>17180</v>
+      </c>
+      <c r="X107" s="7" t="n"/>
+      <c r="Y107" s="7" t="n"/>
+      <c r="Z107" s="7" t="n"/>
+      <c r="AB107" s="7" t="n"/>
+      <c r="AC107" s="7" t="n"/>
+      <c r="AD107" s="7" t="n"/>
+    </row>
+    <row r="108">
+      <c r="T108" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U108" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V108" s="4" t="n">
+        <v>17331</v>
+      </c>
+      <c r="X108" s="4" t="n"/>
+      <c r="Y108" s="4" t="n"/>
+      <c r="Z108" s="4" t="n"/>
+      <c r="AB108" s="4" t="n"/>
+      <c r="AC108" s="4" t="n"/>
+      <c r="AD108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="T109" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U109" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V109" s="7" t="n">
+        <v>17450</v>
+      </c>
+      <c r="X109" s="7" t="n"/>
+      <c r="Y109" s="7" t="n"/>
+      <c r="Z109" s="7" t="n"/>
+      <c r="AB109" s="7" t="n"/>
+      <c r="AC109" s="7" t="n"/>
+      <c r="AD109" s="7" t="n"/>
+    </row>
+    <row r="110">
+      <c r="T110" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U110" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V110" s="4" t="n">
+        <v>17783</v>
+      </c>
+      <c r="X110" s="4" t="n"/>
+      <c r="Y110" s="4" t="n"/>
+      <c r="Z110" s="4" t="n"/>
+      <c r="AB110" s="4" t="n"/>
+      <c r="AC110" s="4" t="n"/>
+      <c r="AD110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="T111" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U111" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V111" s="7" t="n">
+        <v>721</v>
+      </c>
+      <c r="X111" s="7" t="n"/>
+      <c r="Y111" s="7" t="n"/>
+      <c r="Z111" s="7" t="n"/>
+      <c r="AB111" s="7" t="n"/>
+      <c r="AC111" s="7" t="n"/>
+      <c r="AD111" s="7" t="n"/>
+    </row>
+    <row r="112">
+      <c r="T112" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U112" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V112" s="4" t="n">
+        <v>705</v>
+      </c>
+      <c r="X112" s="4" t="n"/>
+      <c r="Y112" s="4" t="n"/>
+      <c r="Z112" s="4" t="n"/>
+      <c r="AB112" s="4" t="n"/>
+      <c r="AC112" s="4" t="n"/>
+      <c r="AD112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="T113" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U113" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V113" s="7" t="n">
+        <v>702</v>
+      </c>
+      <c r="X113" s="7" t="n"/>
+      <c r="Y113" s="7" t="n"/>
+      <c r="Z113" s="7" t="n"/>
+      <c r="AB113" s="7" t="n"/>
+      <c r="AC113" s="7" t="n"/>
+      <c r="AD113" s="7" t="n"/>
+    </row>
+    <row r="114">
+      <c r="T114" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U114" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V114" s="4" t="n">
+        <v>799</v>
+      </c>
+      <c r="X114" s="4" t="n"/>
+      <c r="Y114" s="4" t="n"/>
+      <c r="Z114" s="4" t="n"/>
+      <c r="AB114" s="4" t="n"/>
+      <c r="AC114" s="4" t="n"/>
+      <c r="AD114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="T115" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="U115" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V115" s="7" t="n">
+        <v>746</v>
+      </c>
+      <c r="X115" s="7" t="n"/>
+      <c r="Y115" s="7" t="n"/>
+      <c r="Z115" s="7" t="n"/>
+      <c r="AB115" s="7" t="n"/>
+      <c r="AC115" s="7" t="n"/>
+      <c r="AD115" s="7" t="n"/>
+    </row>
+    <row r="116">
+      <c r="T116" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="U116" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V116" s="4" t="n">
+        <v>752</v>
+      </c>
+      <c r="X116" s="4" t="n"/>
+      <c r="Y116" s="4" t="n"/>
+      <c r="Z116" s="4" t="n"/>
+      <c r="AB116" s="4" t="n"/>
+      <c r="AC116" s="4" t="n"/>
+      <c r="AD116" s="4" t="n"/>
+    </row>
+    <row r="117">
+      <c r="T117" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U117" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V117" s="7" t="n">
+        <v>739</v>
+      </c>
+      <c r="X117" s="7" t="n"/>
+      <c r="Y117" s="7" t="n"/>
+      <c r="Z117" s="7" t="n"/>
+      <c r="AB117" s="7" t="n"/>
+      <c r="AC117" s="7" t="n"/>
+      <c r="AD117" s="7" t="n"/>
+    </row>
+    <row r="118">
+      <c r="T118" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U118" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V118" s="4" t="n">
+        <v>691</v>
+      </c>
+      <c r="X118" s="4" t="n"/>
+      <c r="Y118" s="4" t="n"/>
+      <c r="Z118" s="4" t="n"/>
+      <c r="AB118" s="4" t="n"/>
+      <c r="AC118" s="4" t="n"/>
+      <c r="AD118" s="4" t="n"/>
+    </row>
+    <row r="119">
+      <c r="T119" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U119" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V119" s="7" t="n">
+        <v>715</v>
+      </c>
+      <c r="X119" s="7" t="n"/>
+      <c r="Y119" s="7" t="n"/>
+      <c r="Z119" s="7" t="n"/>
+      <c r="AB119" s="7" t="n"/>
+      <c r="AC119" s="7" t="n"/>
+      <c r="AD119" s="7" t="n"/>
+    </row>
+    <row r="120">
+      <c r="T120" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U120" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V120" s="4" t="n">
+        <v>741</v>
+      </c>
+      <c r="X120" s="4" t="n"/>
+      <c r="Y120" s="4" t="n"/>
+      <c r="Z120" s="4" t="n"/>
+      <c r="AB120" s="4" t="n"/>
+      <c r="AC120" s="4" t="n"/>
+      <c r="AD120" s="4" t="n"/>
+    </row>
+    <row r="121">
+      <c r="T121" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="U121" s="7" t="inlineStr">
         <is>
           <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
-      <c r="V78" s="4" t="n">
+      <c r="V121" s="7" t="n">
+        <v>2009</v>
+      </c>
+      <c r="X121" s="7" t="n"/>
+      <c r="Y121" s="7" t="n"/>
+      <c r="Z121" s="7" t="n"/>
+      <c r="AB121" s="7" t="n"/>
+      <c r="AC121" s="7" t="n"/>
+      <c r="AD121" s="7" t="n"/>
+    </row>
+    <row r="122">
+      <c r="T122" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="U122" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V122" s="4" t="n">
+        <v>2036</v>
+      </c>
+      <c r="X122" s="4" t="n"/>
+      <c r="Y122" s="4" t="n"/>
+      <c r="Z122" s="4" t="n"/>
+      <c r="AB122" s="4" t="n"/>
+      <c r="AC122" s="4" t="n"/>
+      <c r="AD122" s="4" t="n"/>
+    </row>
+    <row r="123">
+      <c r="T123" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="U123" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V123" s="7" t="n">
+        <v>2188</v>
+      </c>
+      <c r="X123" s="7" t="n"/>
+      <c r="Y123" s="7" t="n"/>
+      <c r="Z123" s="7" t="n"/>
+      <c r="AB123" s="7" t="n"/>
+      <c r="AC123" s="7" t="n"/>
+      <c r="AD123" s="7" t="n"/>
+    </row>
+    <row r="124">
+      <c r="T124" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="U124" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V124" s="4" t="n">
+        <v>2179</v>
+      </c>
+      <c r="X124" s="4" t="n"/>
+      <c r="Y124" s="4" t="n"/>
+      <c r="Z124" s="4" t="n"/>
+      <c r="AB124" s="4" t="n"/>
+      <c r="AC124" s="4" t="n"/>
+      <c r="AD124" s="4" t="n"/>
+    </row>
+    <row r="125">
+      <c r="T125" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="U125" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V125" s="7" t="n">
+        <v>2371</v>
+      </c>
+      <c r="X125" s="7" t="n"/>
+      <c r="Y125" s="7" t="n"/>
+      <c r="Z125" s="7" t="n"/>
+      <c r="AB125" s="7" t="n"/>
+      <c r="AC125" s="7" t="n"/>
+      <c r="AD125" s="7" t="n"/>
+    </row>
+    <row r="126">
+      <c r="T126" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="U126" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V126" s="4" t="n">
         <v>2273</v>
       </c>
-      <c r="X78" s="4" t="n"/>
-      <c r="Y78" s="4" t="n"/>
-      <c r="Z78" s="4" t="n"/>
-      <c r="AB78" s="4" t="n"/>
-      <c r="AC78" s="4" t="n"/>
-      <c r="AD78" s="4" t="n"/>
+      <c r="X126" s="4" t="n"/>
+      <c r="Y126" s="4" t="n"/>
+      <c r="Z126" s="4" t="n"/>
+      <c r="AB126" s="4" t="n"/>
+      <c r="AC126" s="4" t="n"/>
+      <c r="AD126" s="4" t="n"/>
+    </row>
+    <row r="127">
+      <c r="T127" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="U127" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V127" s="7" t="n">
+        <v>2096</v>
+      </c>
+      <c r="X127" s="7" t="n"/>
+      <c r="Y127" s="7" t="n"/>
+      <c r="Z127" s="7" t="n"/>
+      <c r="AB127" s="7" t="n"/>
+      <c r="AC127" s="7" t="n"/>
+      <c r="AD127" s="7" t="n"/>
+    </row>
+    <row r="128">
+      <c r="T128" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="U128" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V128" s="4" t="n">
+        <v>1974</v>
+      </c>
+      <c r="X128" s="4" t="n"/>
+      <c r="Y128" s="4" t="n"/>
+      <c r="Z128" s="4" t="n"/>
+      <c r="AB128" s="4" t="n"/>
+      <c r="AC128" s="4" t="n"/>
+      <c r="AD128" s="4" t="n"/>
+    </row>
+    <row r="129">
+      <c r="T129" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="U129" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V129" s="7" t="n">
+        <v>2036</v>
+      </c>
+      <c r="X129" s="7" t="n"/>
+      <c r="Y129" s="7" t="n"/>
+      <c r="Z129" s="7" t="n"/>
+      <c r="AB129" s="7" t="n"/>
+      <c r="AC129" s="7" t="n"/>
+      <c r="AD129" s="7" t="n"/>
+    </row>
+    <row r="130">
+      <c r="T130" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="U130" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V130" s="4" t="n">
+        <v>2140</v>
+      </c>
+      <c r="X130" s="4" t="n"/>
+      <c r="Y130" s="4" t="n"/>
+      <c r="Z130" s="4" t="n"/>
+      <c r="AB130" s="4" t="n"/>
+      <c r="AC130" s="4" t="n"/>
+      <c r="AD130" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Updated report for 4.2633.1
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -3265,7 +3265,7 @@
         <v>4992</v>
       </c>
       <c r="X28" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y28" s="4" t="inlineStr">
         <is>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="Z28" s="4" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>talabat rider</t>
         </is>
       </c>
       <c r="AB28" s="4" t="n">
@@ -3324,7 +3324,7 @@
         <v>4898</v>
       </c>
       <c r="X29" s="7" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="Y29" s="7" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="Z29" s="7" t="inlineStr">
         <is>
-          <t>talabat rider</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB29" s="7" t="n">
@@ -3383,7 +3383,7 @@
         <v>4829</v>
       </c>
       <c r="X30" s="4" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="Y30" s="4" t="inlineStr">
         <is>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="Z30" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB30" s="4" t="n">
@@ -3455,7 +3455,7 @@
         </is>
       </c>
       <c r="AB31" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AC31" s="7" t="inlineStr">
         <is>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="AB32" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AC32" s="4" t="inlineStr">
         <is>
@@ -3806,7 +3806,7 @@
         <v>14699</v>
       </c>
       <c r="X38" s="4" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="Y38" s="4" t="inlineStr">
         <is>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="Z38" s="4" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB38" s="4" t="n">
@@ -3847,7 +3847,7 @@
         <v>14545</v>
       </c>
       <c r="X39" s="7" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="Y39" s="7" t="inlineStr">
         <is>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="Z39" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB39" s="7" t="n">
@@ -3983,7 +3983,7 @@
         </is>
       </c>
       <c r="AB42" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC42" s="4" t="inlineStr">
         <is>
@@ -4065,7 +4065,7 @@
         </is>
       </c>
       <c r="AB44" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC44" s="4" t="inlineStr">
         <is>
@@ -4257,7 +4257,7 @@
         <v>14959</v>
       </c>
       <c r="X49" s="7" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="Y49" s="7" t="inlineStr">
         <is>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="Z49" s="7" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB49" s="7" t="n">
@@ -4298,7 +4298,7 @@
         <v>14157</v>
       </c>
       <c r="X50" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Y50" s="4" t="inlineStr">
         <is>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="Z50" s="4" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB50" s="4" t="n">
@@ -4339,7 +4339,7 @@
         <v>14314</v>
       </c>
       <c r="X51" s="7" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="Y51" s="7" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="Z51" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB51" s="7" t="n">
@@ -4421,7 +4421,7 @@
         <v>81268</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Y53" s="7" t="inlineStr">
         <is>
@@ -4430,11 +4430,11 @@
       </c>
       <c r="Z53" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB53" s="7" t="n">
-        <v>1</v>
+        <v>422</v>
       </c>
       <c r="AC53" s="7" t="inlineStr">
         <is>
@@ -4462,7 +4462,7 @@
         <v>80831</v>
       </c>
       <c r="X54" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Y54" s="4" t="inlineStr">
         <is>
@@ -4471,11 +4471,11 @@
       </c>
       <c r="Z54" s="4" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB54" s="4" t="n">
-        <v>422</v>
+        <v>1</v>
       </c>
       <c r="AC54" s="4" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
         </is>
       </c>
       <c r="AB57" s="7" t="n">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="AC57" s="7" t="inlineStr">
         <is>
@@ -4721,7 +4721,7 @@
         </is>
       </c>
       <c r="AB60" s="4" t="n">
-        <v>55</v>
+        <v>121</v>
       </c>
       <c r="AC60" s="4" t="inlineStr">
         <is>
@@ -4749,7 +4749,7 @@
         <v>81125</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Y61" s="7" t="inlineStr">
         <is>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="Z61" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB61" s="7" t="n">
@@ -4790,7 +4790,7 @@
         <v>83339</v>
       </c>
       <c r="X62" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Y62" s="4" t="inlineStr">
         <is>
@@ -4799,11 +4799,11 @@
       </c>
       <c r="Z62" s="4" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB62" s="4" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="AC62" s="4" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v>83940</v>
       </c>
       <c r="X63" s="7" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="Y63" s="7" t="inlineStr">
         <is>
@@ -4840,11 +4840,11 @@
       </c>
       <c r="Z63" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB63" s="7" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="AC63" s="7" t="inlineStr">
         <is>
@@ -4881,11 +4881,11 @@
       </c>
       <c r="Z64" s="4" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat rider</t>
         </is>
       </c>
       <c r="AB64" s="4" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="AC64" s="4" t="inlineStr">
         <is>
@@ -4913,7 +4913,7 @@
         <v>84011</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="Y65" s="7" t="inlineStr">
         <is>
@@ -4922,11 +4922,11 @@
       </c>
       <c r="Z65" s="7" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB65" s="7" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="AC65" s="7" t="inlineStr">
         <is>
@@ -4954,7 +4954,7 @@
         <v>84598</v>
       </c>
       <c r="X66" s="4" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="Y66" s="4" t="inlineStr">
         <is>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="Z66" s="4" t="inlineStr">
         <is>
-          <t>talabat rider</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB66" s="4" t="n">
@@ -5077,7 +5077,7 @@
         <v>83392</v>
       </c>
       <c r="X69" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="Y69" s="7" t="inlineStr">
         <is>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="Z69" s="7" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB69" s="7" t="n">
@@ -5118,7 +5118,7 @@
         <v>693</v>
       </c>
       <c r="X70" s="4" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Y70" s="4" t="inlineStr">
         <is>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="Z70" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB70" s="4" t="n">
@@ -5172,7 +5172,7 @@
         </is>
       </c>
       <c r="AB71" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC71" s="7" t="inlineStr">
         <is>
@@ -5213,7 +5213,7 @@
         </is>
       </c>
       <c r="AB72" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC72" s="4" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
         <v>682</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Y75" s="7" t="inlineStr">
         <is>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="Z75" s="7" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB75" s="7" t="n">
@@ -5364,7 +5364,7 @@
         <v>692</v>
       </c>
       <c r="X76" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="Y76" s="4" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="Z76" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB76" s="4" t="n">
@@ -5405,7 +5405,7 @@
         <v>682</v>
       </c>
       <c r="X77" s="7" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Y77" s="7" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
       </c>
       <c r="Z77" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB77" s="7" t="n">
@@ -5487,7 +5487,7 @@
         <v>729</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Y79" s="7" t="inlineStr">
         <is>
@@ -5496,11 +5496,11 @@
       </c>
       <c r="Z79" s="7" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB79" s="7" t="n">
-        <v>113</v>
+        <v>3</v>
       </c>
       <c r="AC79" s="7" t="inlineStr">
         <is>
@@ -5541,7 +5541,7 @@
         </is>
       </c>
       <c r="AB80" s="4" t="n">
-        <v>1</v>
+        <v>113</v>
       </c>
       <c r="AC80" s="4" t="inlineStr">
         <is>
@@ -5582,7 +5582,7 @@
         </is>
       </c>
       <c r="AB81" s="7" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="AC81" s="7" t="inlineStr">
         <is>
@@ -5610,7 +5610,7 @@
         <v>698</v>
       </c>
       <c r="X82" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="Y82" s="4" t="inlineStr">
         <is>
@@ -5619,11 +5619,11 @@
       </c>
       <c r="Z82" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerstation rider</t>
         </is>
       </c>
       <c r="AB82" s="4" t="n">
-        <v>61</v>
+        <v>1</v>
       </c>
       <c r="AC82" s="4" t="inlineStr">
         <is>
@@ -5651,7 +5651,7 @@
         <v>682</v>
       </c>
       <c r="X83" s="7" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Y83" s="7" t="inlineStr">
         <is>
@@ -5660,11 +5660,11 @@
       </c>
       <c r="Z83" s="7" t="inlineStr">
         <is>
-          <t>hungerstation rider</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB83" s="7" t="n">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="AC83" s="7" t="inlineStr">
         <is>
@@ -5705,7 +5705,7 @@
         </is>
       </c>
       <c r="AB84" s="4" t="n">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="AC84" s="4" t="inlineStr">
         <is>
@@ -5774,7 +5774,7 @@
         <v>718</v>
       </c>
       <c r="X86" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y86" s="4" t="inlineStr">
         <is>
@@ -5783,11 +5783,11 @@
       </c>
       <c r="Z86" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>efood</t>
         </is>
       </c>
       <c r="AB86" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC86" s="4" t="inlineStr">
         <is>
@@ -5815,7 +5815,7 @@
         <v>48099</v>
       </c>
       <c r="X87" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y87" s="7" t="inlineStr">
         <is>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="Z87" s="7" t="inlineStr">
         <is>
-          <t>efood</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="AB87" s="7" t="n">
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="AB88" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC88" s="4" t="inlineStr">
         <is>
@@ -5897,7 +5897,7 @@
         <v>49786</v>
       </c>
       <c r="X89" s="7" t="n">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="Y89" s="7" t="inlineStr">
         <is>
@@ -5906,7 +5906,7 @@
       </c>
       <c r="Z89" s="7" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB89" s="7" t="n">
@@ -5938,7 +5938,7 @@
         <v>48589</v>
       </c>
       <c r="X90" s="4" t="n">
-        <v>67</v>
+        <v>11</v>
       </c>
       <c r="Y90" s="4" t="inlineStr">
         <is>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="Z90" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB90" s="4" t="n">
@@ -5979,7 +5979,7 @@
         <v>48093</v>
       </c>
       <c r="X91" s="7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="Y91" s="7" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="Z91" s="7" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB91" s="7" t="n">
@@ -6020,7 +6020,7 @@
         <v>49210</v>
       </c>
       <c r="X92" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="Y92" s="4" t="inlineStr">
         <is>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="Z92" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB92" s="4" t="n">
@@ -6061,7 +6061,7 @@
         <v>48289</v>
       </c>
       <c r="X93" s="7" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="Y93" s="7" t="inlineStr">
         <is>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="Z93" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB93" s="7" t="n">
@@ -6102,7 +6102,7 @@
         <v>47345</v>
       </c>
       <c r="X94" s="4" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="Y94" s="4" t="inlineStr">
         <is>
@@ -6111,11 +6111,11 @@
       </c>
       <c r="Z94" s="4" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB94" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC94" s="4" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         </is>
       </c>
       <c r="AB95" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC95" s="7" t="inlineStr">
         <is>
@@ -6197,7 +6197,7 @@
         </is>
       </c>
       <c r="AB96" s="4" t="n">
-        <v>45</v>
+        <v>390</v>
       </c>
       <c r="AC96" s="4" t="inlineStr">
         <is>
@@ -6225,7 +6225,7 @@
         <v>49629</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Y97" s="7" t="inlineStr">
         <is>
@@ -6234,7 +6234,7 @@
       </c>
       <c r="Z97" s="7" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB97" s="7" t="n">
@@ -6266,7 +6266,7 @@
         <v>48603</v>
       </c>
       <c r="X98" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Y98" s="4" t="inlineStr">
         <is>
@@ -6275,11 +6275,11 @@
       </c>
       <c r="Z98" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB98" s="4" t="n">
-        <v>390</v>
+        <v>45</v>
       </c>
       <c r="AC98" s="4" t="inlineStr">
         <is>
@@ -6320,7 +6320,7 @@
         </is>
       </c>
       <c r="AB99" s="7" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="AC99" s="7" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="AB100" s="4" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="AC100" s="4" t="inlineStr">
         <is>
@@ -6443,7 +6443,7 @@
         </is>
       </c>
       <c r="AB102" s="4" t="n">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="AC102" s="4" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         <v>49341</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="Y103" s="7" t="inlineStr">
         <is>
@@ -6480,11 +6480,11 @@
       </c>
       <c r="Z103" s="7" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB103" s="7" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="AC103" s="7" t="inlineStr">
         <is>
@@ -6512,7 +6512,7 @@
         <v>1</v>
       </c>
       <c r="X104" s="4" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="Y104" s="4" t="inlineStr">
         <is>
@@ -6521,11 +6521,11 @@
       </c>
       <c r="Z104" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB104" s="4" t="n">
-        <v>104</v>
+        <v>1</v>
       </c>
       <c r="AC104" s="4" t="inlineStr">
         <is>
@@ -6562,11 +6562,11 @@
       </c>
       <c r="Z105" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB105" s="7" t="n">
-        <v>4</v>
+        <v>104</v>
       </c>
       <c r="AC105" s="7" t="inlineStr">
         <is>
@@ -6603,11 +6603,11 @@
       </c>
       <c r="Z106" s="4" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB106" s="4" t="n">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="AC106" s="4" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="AB107" s="7" t="n">
-        <v>61</v>
+        <v>9</v>
       </c>
       <c r="AC107" s="7" t="inlineStr">
         <is>
@@ -6689,7 +6689,7 @@
         </is>
       </c>
       <c r="AB108" s="4" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AC108" s="4" t="inlineStr">
         <is>
@@ -6730,7 +6730,7 @@
         </is>
       </c>
       <c r="AB109" s="7" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AC109" s="7" t="inlineStr">
         <is>
@@ -6771,7 +6771,7 @@
         </is>
       </c>
       <c r="AB110" s="4" t="n">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="AC110" s="4" t="inlineStr">
         <is>
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="AB111" s="7" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="AC111" s="7" t="inlineStr">
         <is>
@@ -6840,7 +6840,7 @@
         <v>1</v>
       </c>
       <c r="X112" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y112" s="4" t="inlineStr">
         <is>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="Z112" s="4" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB112" s="4" t="n">
@@ -6881,7 +6881,7 @@
         <v>1</v>
       </c>
       <c r="X113" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y113" s="7" t="inlineStr">
         <is>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="Z113" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB113" s="7" t="n">
@@ -7017,7 +7017,7 @@
         </is>
       </c>
       <c r="AB116" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC116" s="4" t="inlineStr">
         <is>
@@ -7058,7 +7058,7 @@
         </is>
       </c>
       <c r="AB117" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC117" s="7" t="inlineStr">
         <is>
@@ -7086,7 +7086,7 @@
         <v>1</v>
       </c>
       <c r="X118" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Y118" s="4" t="inlineStr">
         <is>
@@ -7095,11 +7095,11 @@
       </c>
       <c r="Z118" s="4" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>foodora rider</t>
         </is>
       </c>
       <c r="AB118" s="4" t="n">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="AC118" s="4" t="inlineStr">
         <is>
@@ -7140,7 +7140,7 @@
         </is>
       </c>
       <c r="AB119" s="7" t="n">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="AC119" s="7" t="inlineStr">
         <is>
@@ -7168,7 +7168,7 @@
         <v>1</v>
       </c>
       <c r="X120" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y120" s="4" t="inlineStr">
         <is>
@@ -7177,7 +7177,7 @@
       </c>
       <c r="Z120" s="4" t="inlineStr">
         <is>
-          <t>foodora rider</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB120" s="4" t="n">
@@ -7332,7 +7332,7 @@
         <v>1</v>
       </c>
       <c r="X124" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y124" s="4" t="inlineStr">
         <is>
@@ -7341,7 +7341,7 @@
       </c>
       <c r="Z124" s="4" t="inlineStr">
         <is>
-          <t>PedidosYa</t>
+          <t>pedidosYa</t>
         </is>
       </c>
       <c r="AB124" s="4" t="n">
@@ -7373,7 +7373,7 @@
         <v>1</v>
       </c>
       <c r="X125" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y125" s="7" t="inlineStr">
         <is>
@@ -7382,11 +7382,11 @@
       </c>
       <c r="Z125" s="7" t="inlineStr">
         <is>
-          <t>pedidosYa</t>
+          <t>PedidosYa</t>
         </is>
       </c>
       <c r="AB125" s="7" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="AC125" s="7" t="inlineStr">
         <is>
@@ -7427,7 +7427,7 @@
         </is>
       </c>
       <c r="AB126" s="4" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="AC126" s="4" t="inlineStr">
         <is>
@@ -7468,7 +7468,7 @@
         </is>
       </c>
       <c r="AB127" s="7" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="AC127" s="7" t="inlineStr">
         <is>
@@ -7632,7 +7632,7 @@
         </is>
       </c>
       <c r="AB131" s="7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AC131" s="7" t="inlineStr">
         <is>
@@ -7714,7 +7714,7 @@
         </is>
       </c>
       <c r="AB133" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AC133" s="7" t="inlineStr">
         <is>
@@ -7742,7 +7742,7 @@
         <v>1</v>
       </c>
       <c r="X134" s="4" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="Y134" s="4" t="inlineStr">
         <is>
@@ -7751,7 +7751,7 @@
       </c>
       <c r="Z134" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB134" s="4" t="n">
@@ -7783,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="X135" s="7" t="n">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="Y135" s="7" t="inlineStr">
         <is>
@@ -7792,7 +7792,7 @@
       </c>
       <c r="Z135" s="7" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB135" s="7" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="Z136" s="4" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB136" s="4" t="n">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="Z137" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB137" s="7" t="n">
@@ -8124,7 +8124,7 @@
         </is>
       </c>
       <c r="AB143" s="7" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="AC143" s="7" t="inlineStr">
         <is>
@@ -8152,7 +8152,7 @@
         <v>10451</v>
       </c>
       <c r="X144" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="Y144" s="4" t="inlineStr">
         <is>
@@ -8161,11 +8161,11 @@
       </c>
       <c r="Z144" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB144" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="AC144" s="4" t="inlineStr">
         <is>
@@ -8193,7 +8193,7 @@
         <v>10531</v>
       </c>
       <c r="X145" s="7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="Y145" s="7" t="inlineStr">
         <is>
@@ -8202,11 +8202,11 @@
       </c>
       <c r="Z145" s="7" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB145" s="7" t="n">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="AC145" s="7" t="inlineStr">
         <is>
@@ -8288,7 +8288,7 @@
         </is>
       </c>
       <c r="AB147" s="7" t="n">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="AC147" s="7" t="inlineStr">
         <is>
@@ -8357,7 +8357,7 @@
         <v>10745</v>
       </c>
       <c r="X149" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y149" s="7" t="inlineStr">
         <is>
@@ -8366,11 +8366,11 @@
       </c>
       <c r="Z149" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>efood</t>
         </is>
       </c>
       <c r="AB149" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC149" s="7" t="inlineStr">
         <is>
@@ -8398,7 +8398,7 @@
         <v>10405</v>
       </c>
       <c r="X150" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y150" s="4" t="inlineStr">
         <is>
@@ -8407,7 +8407,7 @@
       </c>
       <c r="Z150" s="4" t="inlineStr">
         <is>
-          <t>efood</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="AB150" s="4" t="n">
@@ -8448,7 +8448,7 @@
       </c>
       <c r="Z151" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>foody</t>
         </is>
       </c>
       <c r="AB151" s="7" t="n">
@@ -8489,11 +8489,11 @@
       </c>
       <c r="Z152" s="4" t="inlineStr">
         <is>
-          <t>foody</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="AB152" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC152" s="4" t="inlineStr">
         <is>
@@ -8521,7 +8521,7 @@
         <v>10760</v>
       </c>
       <c r="X153" s="7" t="n">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="Y153" s="7" t="inlineStr">
         <is>
@@ -8530,11 +8530,11 @@
       </c>
       <c r="Z153" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB153" s="7" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="AC153" s="7" t="inlineStr">
         <is>
@@ -8562,7 +8562,7 @@
         <v>23698</v>
       </c>
       <c r="X154" s="4" t="n">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="Y154" s="4" t="inlineStr">
         <is>
@@ -8571,11 +8571,11 @@
       </c>
       <c r="Z154" s="4" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB154" s="4" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="AC154" s="4" t="inlineStr">
         <is>
@@ -8603,7 +8603,7 @@
         <v>22677</v>
       </c>
       <c r="X155" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Y155" s="7" t="inlineStr">
         <is>
@@ -8612,11 +8612,11 @@
       </c>
       <c r="Z155" s="7" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB155" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC155" s="7" t="inlineStr">
         <is>
@@ -8644,7 +8644,7 @@
         <v>24762</v>
       </c>
       <c r="X156" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Y156" s="4" t="inlineStr">
         <is>
@@ -8653,7 +8653,7 @@
       </c>
       <c r="Z156" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB156" s="4" t="n">
@@ -8739,7 +8739,7 @@
         </is>
       </c>
       <c r="AB158" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AC158" s="4" t="inlineStr">
         <is>
@@ -8780,7 +8780,7 @@
         </is>
       </c>
       <c r="AB159" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AC159" s="7" t="inlineStr">
         <is>
@@ -8821,7 +8821,7 @@
         </is>
       </c>
       <c r="AB160" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC160" s="4" t="inlineStr">
         <is>
@@ -8931,7 +8931,7 @@
         <v>25336</v>
       </c>
       <c r="X163" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y163" s="7" t="inlineStr">
         <is>
@@ -8940,11 +8940,11 @@
       </c>
       <c r="Z163" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB163" s="7" t="n">
-        <v>316</v>
+        <v>8</v>
       </c>
       <c r="AC163" s="7" t="inlineStr">
         <is>
@@ -8972,7 +8972,7 @@
         <v>24628</v>
       </c>
       <c r="X164" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Y164" s="4" t="inlineStr">
         <is>
@@ -8981,11 +8981,11 @@
       </c>
       <c r="Z164" s="4" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB164" s="4" t="n">
-        <v>94</v>
+        <v>316</v>
       </c>
       <c r="AC164" s="4" t="inlineStr">
         <is>
@@ -9026,7 +9026,7 @@
         </is>
       </c>
       <c r="AB165" s="7" t="n">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="AC165" s="7" t="inlineStr">
         <is>
@@ -9067,7 +9067,7 @@
         </is>
       </c>
       <c r="AB166" s="4" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="AC166" s="4" t="inlineStr">
         <is>
@@ -9095,7 +9095,7 @@
         <v>25445</v>
       </c>
       <c r="X167" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y167" s="7" t="inlineStr">
         <is>
@@ -9104,11 +9104,11 @@
       </c>
       <c r="Z167" s="7" t="inlineStr">
         <is>
-          <t>Glovo</t>
+          <t>glovo</t>
         </is>
       </c>
       <c r="AB167" s="7" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="AC167" s="7" t="inlineStr">
         <is>
@@ -9136,7 +9136,7 @@
         <v>24666</v>
       </c>
       <c r="X168" s="4" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Y168" s="4" t="inlineStr">
         <is>
@@ -9145,11 +9145,11 @@
       </c>
       <c r="Z168" s="4" t="inlineStr">
         <is>
-          <t>glovo</t>
+          <t>Glovo</t>
         </is>
       </c>
       <c r="AB168" s="4" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="AC168" s="4" t="inlineStr">
         <is>
@@ -9177,7 +9177,7 @@
         <v>23873</v>
       </c>
       <c r="X169" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y169" s="7" t="inlineStr">
         <is>
@@ -9186,11 +9186,11 @@
       </c>
       <c r="Z169" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>efood</t>
         </is>
       </c>
       <c r="AB169" s="7" t="n">
-        <v>118</v>
+        <v>1</v>
       </c>
       <c r="AC169" s="7" t="inlineStr">
         <is>
@@ -9218,7 +9218,7 @@
         <v>25277</v>
       </c>
       <c r="X170" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y170" s="4" t="inlineStr">
         <is>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="Z170" s="4" t="inlineStr">
         <is>
-          <t>efood</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="AB170" s="4" t="n">
@@ -9272,7 +9272,7 @@
         </is>
       </c>
       <c r="AB171" s="7" t="n">
-        <v>39</v>
+        <v>118</v>
       </c>
       <c r="AC171" s="7" t="inlineStr">
         <is>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
       <c r="AB172" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AC172" s="4" t="inlineStr">
         <is>
@@ -9341,7 +9341,7 @@
         <v>17603</v>
       </c>
       <c r="X173" s="7" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="Y173" s="7" t="inlineStr">
         <is>
@@ -9350,11 +9350,11 @@
       </c>
       <c r="Z173" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB173" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC173" s="7" t="inlineStr">
         <is>
@@ -9382,7 +9382,7 @@
         <v>17696</v>
       </c>
       <c r="X174" s="4" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="Y174" s="4" t="inlineStr">
         <is>
@@ -9391,11 +9391,11 @@
       </c>
       <c r="Z174" s="4" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB174" s="4" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="AC174" s="4" t="inlineStr">
         <is>
@@ -9423,7 +9423,7 @@
         <v>17579</v>
       </c>
       <c r="X175" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Y175" s="7" t="inlineStr">
         <is>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="Z175" s="7" t="inlineStr">
         <is>
-          <t>foodora</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="AB175" s="7" t="n">
@@ -9464,7 +9464,7 @@
         <v>17878</v>
       </c>
       <c r="X176" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Y176" s="4" t="inlineStr">
         <is>
@@ -9473,11 +9473,11 @@
       </c>
       <c r="Z176" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>foodora</t>
         </is>
       </c>
       <c r="AB176" s="4" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="AC176" s="4" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>17180</v>
       </c>
       <c r="X177" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Y177" s="7" t="inlineStr">
         <is>
@@ -9514,11 +9514,11 @@
       </c>
       <c r="Z177" s="7" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB177" s="7" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="AC177" s="7" t="inlineStr">
         <is>
@@ -9559,7 +9559,7 @@
         </is>
       </c>
       <c r="AB178" s="4" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="AC178" s="4" t="inlineStr">
         <is>
@@ -9587,7 +9587,7 @@
         <v>17450</v>
       </c>
       <c r="X179" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Y179" s="7" t="inlineStr">
         <is>
@@ -9596,11 +9596,11 @@
       </c>
       <c r="Z179" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB179" s="7" t="n">
-        <v>9</v>
+        <v>152</v>
       </c>
       <c r="AC179" s="7" t="inlineStr">
         <is>
@@ -9669,7 +9669,7 @@
         <v>17861</v>
       </c>
       <c r="X181" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y181" s="7" t="inlineStr">
         <is>
@@ -9678,11 +9678,11 @@
       </c>
       <c r="Z181" s="7" t="inlineStr">
         <is>
-          <t>PedidosYa</t>
+          <t>pedidosYa</t>
         </is>
       </c>
       <c r="AB181" s="7" t="n">
-        <v>152</v>
+        <v>9</v>
       </c>
       <c r="AC181" s="7" t="inlineStr">
         <is>
@@ -9710,7 +9710,7 @@
         <v>17640</v>
       </c>
       <c r="X182" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Y182" s="4" t="inlineStr">
         <is>
@@ -9719,7 +9719,7 @@
       </c>
       <c r="Z182" s="4" t="inlineStr">
         <is>
-          <t>pedidosYa</t>
+          <t>PedidosYa</t>
         </is>
       </c>
       <c r="AB182" s="4" t="n">
@@ -9751,7 +9751,7 @@
         <v>17604</v>
       </c>
       <c r="X183" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="Y183" s="7" t="inlineStr">
         <is>
@@ -9760,11 +9760,11 @@
       </c>
       <c r="Z183" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerstation rider</t>
         </is>
       </c>
       <c r="AB183" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AC183" s="7" t="inlineStr">
         <is>
@@ -9792,7 +9792,7 @@
         <v>17082</v>
       </c>
       <c r="X184" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y184" s="4" t="inlineStr">
         <is>
@@ -9801,11 +9801,11 @@
       </c>
       <c r="Z184" s="4" t="inlineStr">
         <is>
-          <t>hungerstation rider</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB184" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AC184" s="4" t="inlineStr">
         <is>
@@ -9833,7 +9833,7 @@
         <v>17142</v>
       </c>
       <c r="X185" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y185" s="7" t="inlineStr">
         <is>
@@ -9842,7 +9842,7 @@
       </c>
       <c r="Z185" s="7" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB185" s="7" t="n">
@@ -9928,7 +9928,7 @@
         </is>
       </c>
       <c r="AB187" s="7" t="n">
-        <v>290</v>
+        <v>9</v>
       </c>
       <c r="AC187" s="7" t="inlineStr">
         <is>
@@ -9969,7 +9969,7 @@
         </is>
       </c>
       <c r="AB188" s="4" t="n">
-        <v>9</v>
+        <v>138</v>
       </c>
       <c r="AC188" s="4" t="inlineStr">
         <is>
@@ -9997,7 +9997,7 @@
         <v>705</v>
       </c>
       <c r="X189" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="Y189" s="7" t="inlineStr">
         <is>
@@ -10006,11 +10006,11 @@
       </c>
       <c r="Z189" s="7" t="inlineStr">
         <is>
-          <t>efood</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="AB189" s="7" t="n">
-        <v>138</v>
+        <v>290</v>
       </c>
       <c r="AC189" s="7" t="inlineStr">
         <is>
@@ -10038,7 +10038,7 @@
         <v>702</v>
       </c>
       <c r="X190" s="4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Y190" s="4" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
       </c>
       <c r="Z190" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>efood</t>
         </is>
       </c>
       <c r="AB190" s="4" t="n">
@@ -10174,7 +10174,7 @@
         </is>
       </c>
       <c r="AB193" s="7" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="AC193" s="7" t="inlineStr">
         <is>
@@ -10215,7 +10215,7 @@
         </is>
       </c>
       <c r="AB194" s="4" t="n">
-        <v>3</v>
+        <v>116</v>
       </c>
       <c r="AC194" s="4" t="inlineStr">
         <is>
@@ -10256,7 +10256,7 @@
         </is>
       </c>
       <c r="AB195" s="7" t="n">
-        <v>116</v>
+        <v>3</v>
       </c>
       <c r="AC195" s="7" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         <v>715</v>
       </c>
       <c r="X196" s="4" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="Y196" s="4" t="inlineStr">
         <is>
@@ -10293,11 +10293,11 @@
       </c>
       <c r="Z196" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB196" s="4" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="AC196" s="4" t="inlineStr">
         <is>
@@ -10325,7 +10325,7 @@
         <v>741</v>
       </c>
       <c r="X197" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y197" s="7" t="inlineStr">
         <is>
@@ -10334,11 +10334,11 @@
       </c>
       <c r="Z197" s="7" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB197" s="7" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="AC197" s="7" t="inlineStr">
         <is>
@@ -10366,7 +10366,7 @@
         <v>740</v>
       </c>
       <c r="X198" s="4" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="Y198" s="4" t="inlineStr">
         <is>
@@ -10375,11 +10375,11 @@
       </c>
       <c r="Z198" s="4" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB198" s="4" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="AC198" s="4" t="inlineStr">
         <is>
@@ -10407,7 +10407,7 @@
         <v>731</v>
       </c>
       <c r="X199" s="7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Y199" s="7" t="inlineStr">
         <is>
@@ -10416,7 +10416,7 @@
       </c>
       <c r="Z199" s="7" t="inlineStr">
         <is>
-          <t>pedidosYa</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="AB199" s="7" t="n">
@@ -10448,7 +10448,7 @@
         <v>757</v>
       </c>
       <c r="X200" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="Y200" s="4" t="inlineStr">
         <is>
@@ -10457,11 +10457,11 @@
       </c>
       <c r="Z200" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>pedidosYa</t>
         </is>
       </c>
       <c r="AB200" s="4" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="AC200" s="4" t="inlineStr">
         <is>
@@ -10489,7 +10489,7 @@
         <v>783</v>
       </c>
       <c r="X201" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y201" s="7" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
       </c>
       <c r="Z201" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB201" s="7" t="n">
@@ -10530,7 +10530,7 @@
         <v>757</v>
       </c>
       <c r="X202" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y202" s="4" t="inlineStr">
         <is>
@@ -10539,11 +10539,11 @@
       </c>
       <c r="Z202" s="4" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB202" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="AC202" s="4" t="inlineStr">
         <is>
@@ -10571,7 +10571,7 @@
         <v>725</v>
       </c>
       <c r="X203" s="7" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="Y203" s="7" t="inlineStr">
         <is>
@@ -10580,11 +10580,11 @@
       </c>
       <c r="Z203" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>glovo</t>
         </is>
       </c>
       <c r="AB203" s="7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AC203" s="7" t="inlineStr">
         <is>
@@ -10612,7 +10612,7 @@
         <v>746</v>
       </c>
       <c r="X204" s="4" t="n">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="Y204" s="4" t="inlineStr">
         <is>
@@ -10621,7 +10621,7 @@
       </c>
       <c r="Z204" s="4" t="inlineStr">
         <is>
-          <t>glovo</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="AB204" s="4" t="n">
@@ -10981,7 +10981,7 @@
         <v>2036</v>
       </c>
       <c r="X213" s="7" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="Y213" s="7" t="inlineStr">
         <is>
@@ -10990,7 +10990,7 @@
       </c>
       <c r="Z213" s="7" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB213" s="7" t="n">
@@ -11063,7 +11063,7 @@
         <v>2134</v>
       </c>
       <c r="X215" s="7" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="Y215" s="7" t="inlineStr">
         <is>
@@ -11072,11 +11072,11 @@
       </c>
       <c r="Z215" s="7" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB215" s="7" t="n">
-        <v>280</v>
+        <v>11</v>
       </c>
       <c r="AC215" s="7" t="inlineStr">
         <is>
@@ -11117,7 +11117,7 @@
         </is>
       </c>
       <c r="AB216" s="4" t="n">
-        <v>11</v>
+        <v>280</v>
       </c>
       <c r="AC216" s="4" t="inlineStr">
         <is>
@@ -11158,7 +11158,7 @@
         </is>
       </c>
       <c r="AB217" s="7" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="AC217" s="7" t="inlineStr">
         <is>
@@ -11199,7 +11199,7 @@
         </is>
       </c>
       <c r="AB218" s="4" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="AC218" s="4" t="inlineStr">
         <is>
@@ -11227,7 +11227,7 @@
         <v>2029</v>
       </c>
       <c r="X219" s="7" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Y219" s="7" t="inlineStr">
         <is>
@@ -11236,7 +11236,7 @@
       </c>
       <c r="Z219" s="7" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB219" s="7" t="n">
@@ -11268,7 +11268,7 @@
         <v>2037</v>
       </c>
       <c r="X220" s="4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Y220" s="4" t="inlineStr">
         <is>
@@ -11277,11 +11277,11 @@
       </c>
       <c r="Z220" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB220" s="4" t="n">
-        <v>39</v>
+        <v>136</v>
       </c>
       <c r="AC220" s="4" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         </is>
       </c>
       <c r="AB221" s="7" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="AC221" s="7" t="inlineStr">
         <is>
@@ -11384,7 +11384,7 @@
         </is>
       </c>
       <c r="AB223" s="7" t="n">
-        <v>136</v>
+        <v>6</v>
       </c>
       <c r="AC223" s="7" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         </is>
       </c>
       <c r="AB224" s="4" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="AC224" s="4" t="inlineStr">
         <is>
@@ -11446,7 +11446,7 @@
         </is>
       </c>
       <c r="AB225" s="7" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="AC225" s="7" t="inlineStr">
         <is>
@@ -11464,7 +11464,7 @@
       <c r="U226" s="4" t="n"/>
       <c r="V226" s="4" t="n"/>
       <c r="X226" s="4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="Y226" s="4" t="inlineStr">
         <is>
@@ -11473,7 +11473,7 @@
       </c>
       <c r="Z226" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>foodpanda</t>
         </is>
       </c>
       <c r="AB226" s="4" t="n">
@@ -11495,7 +11495,7 @@
       <c r="U227" s="7" t="n"/>
       <c r="V227" s="7" t="n"/>
       <c r="X227" s="7" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="Y227" s="7" t="inlineStr">
         <is>
@@ -11504,7 +11504,7 @@
       </c>
       <c r="Z227" s="7" t="inlineStr">
         <is>
-          <t>foodpanda</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="AB227" s="7" t="n">
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="AB228" s="4" t="n">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="AC228" s="4" t="inlineStr">
         <is>
@@ -11570,7 +11570,7 @@
         </is>
       </c>
       <c r="AB229" s="7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="AC229" s="7" t="inlineStr">
         <is>
@@ -11588,7 +11588,7 @@
       <c r="U230" s="4" t="n"/>
       <c r="V230" s="4" t="n"/>
       <c r="X230" s="4" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="Y230" s="4" t="inlineStr">
         <is>
@@ -11597,11 +11597,11 @@
       </c>
       <c r="Z230" s="4" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB230" s="4" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="AC230" s="4" t="inlineStr">
         <is>
@@ -11619,7 +11619,7 @@
       <c r="U231" s="7" t="n"/>
       <c r="V231" s="7" t="n"/>
       <c r="X231" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y231" s="7" t="inlineStr">
         <is>
@@ -11628,7 +11628,7 @@
       </c>
       <c r="Z231" s="7" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="AB231" s="7" t="n">
@@ -11650,7 +11650,7 @@
       <c r="U232" s="4" t="n"/>
       <c r="V232" s="4" t="n"/>
       <c r="X232" s="4" t="n">
-        <v>5</v>
+        <v>41</v>
       </c>
       <c r="Y232" s="4" t="inlineStr">
         <is>
@@ -11659,11 +11659,11 @@
       </c>
       <c r="Z232" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB232" s="4" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="AC232" s="4" t="inlineStr">
         <is>
@@ -11694,7 +11694,7 @@
         </is>
       </c>
       <c r="AB233" s="7" t="n">
-        <v>2</v>
+        <v>170</v>
       </c>
       <c r="AC233" s="7" t="inlineStr">
         <is>
@@ -11725,7 +11725,7 @@
         </is>
       </c>
       <c r="AB234" s="4" t="n">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="AC234" s="4" t="inlineStr">
         <is>
@@ -11743,7 +11743,7 @@
       <c r="U235" s="7" t="n"/>
       <c r="V235" s="7" t="n"/>
       <c r="X235" s="7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Y235" s="7" t="inlineStr">
         <is>
@@ -11752,7 +11752,7 @@
       </c>
       <c r="Z235" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>hungerStation</t>
         </is>
       </c>
       <c r="AB235" s="7" t="n">
@@ -11774,7 +11774,7 @@
       <c r="U236" s="4" t="n"/>
       <c r="V236" s="4" t="n"/>
       <c r="X236" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Y236" s="4" t="inlineStr">
         <is>
@@ -11783,7 +11783,7 @@
       </c>
       <c r="Z236" s="4" t="inlineStr">
         <is>
-          <t>hungerStation</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="AB236" s="4" t="n">
@@ -11867,7 +11867,7 @@
       <c r="U239" s="7" t="n"/>
       <c r="V239" s="7" t="n"/>
       <c r="X239" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y239" s="7" t="inlineStr">
         <is>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="Z239" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>efood</t>
         </is>
       </c>
       <c r="AB239" s="7" t="n">
@@ -11898,7 +11898,7 @@
       <c r="U240" s="4" t="n"/>
       <c r="V240" s="4" t="n"/>
       <c r="X240" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y240" s="4" t="inlineStr">
         <is>
@@ -11907,11 +11907,11 @@
       </c>
       <c r="Z240" s="4" t="inlineStr">
         <is>
-          <t>efood</t>
+          <t>com.logistics.rider.efood</t>
         </is>
       </c>
       <c r="AB240" s="4" t="n">
-        <v>151</v>
+        <v>274</v>
       </c>
       <c r="AC240" s="4" t="inlineStr">
         <is>
@@ -11932,7 +11932,7 @@
       <c r="Y241" s="7" t="n"/>
       <c r="Z241" s="7" t="n"/>
       <c r="AB241" s="7" t="n">
-        <v>274</v>
+        <v>14</v>
       </c>
       <c r="AC241" s="7" t="inlineStr">
         <is>
@@ -11953,7 +11953,7 @@
       <c r="Y242" s="4" t="n"/>
       <c r="Z242" s="4" t="n"/>
       <c r="AB242" s="4" t="n">
-        <v>14</v>
+        <v>151</v>
       </c>
       <c r="AC242" s="4" t="inlineStr">
         <is>
@@ -12037,7 +12037,7 @@
       <c r="Y246" s="4" t="n"/>
       <c r="Z246" s="4" t="n"/>
       <c r="AB246" s="4" t="n">
-        <v>25</v>
+        <v>138</v>
       </c>
       <c r="AC246" s="4" t="inlineStr">
         <is>
@@ -12100,7 +12100,7 @@
       <c r="Y249" s="7" t="n"/>
       <c r="Z249" s="7" t="n"/>
       <c r="AB249" s="7" t="n">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="AC249" s="7" t="inlineStr">
         <is>
@@ -12121,7 +12121,7 @@
       <c r="Y250" s="4" t="n"/>
       <c r="Z250" s="4" t="n"/>
       <c r="AB250" s="4" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="AC250" s="4" t="inlineStr">
         <is>
@@ -12163,7 +12163,7 @@
       <c r="Y252" s="4" t="n"/>
       <c r="Z252" s="4" t="n"/>
       <c r="AB252" s="4" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="AC252" s="4" t="inlineStr">
         <is>
@@ -12499,7 +12499,7 @@
       <c r="Y268" s="4" t="n"/>
       <c r="Z268" s="4" t="n"/>
       <c r="AB268" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="AC268" s="4" t="inlineStr">
         <is>
@@ -12520,7 +12520,7 @@
       <c r="Y269" s="7" t="n"/>
       <c r="Z269" s="7" t="n"/>
       <c r="AB269" s="7" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AC269" s="7" t="inlineStr">
         <is>
@@ -12541,7 +12541,7 @@
       <c r="Y270" s="4" t="n"/>
       <c r="Z270" s="4" t="n"/>
       <c r="AB270" s="4" t="n">
-        <v>137</v>
+        <v>2</v>
       </c>
       <c r="AC270" s="4" t="inlineStr">
         <is>
@@ -12583,7 +12583,7 @@
       <c r="Y272" s="4" t="n"/>
       <c r="Z272" s="4" t="n"/>
       <c r="AB272" s="4" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="AC272" s="4" t="inlineStr">
         <is>
@@ -12604,7 +12604,7 @@
       <c r="Y273" s="7" t="n"/>
       <c r="Z273" s="7" t="n"/>
       <c r="AB273" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC273" s="7" t="inlineStr">
         <is>
@@ -12646,7 +12646,7 @@
       <c r="Y275" s="7" t="n"/>
       <c r="Z275" s="7" t="n"/>
       <c r="AB275" s="7" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="AC275" s="7" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
       <c r="Y276" s="4" t="n"/>
       <c r="Z276" s="4" t="n"/>
       <c r="AB276" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="AC276" s="4" t="inlineStr">
         <is>
@@ -12688,7 +12688,7 @@
       <c r="Y277" s="7" t="n"/>
       <c r="Z277" s="7" t="n"/>
       <c r="AB277" s="7" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="AC277" s="7" t="inlineStr">
         <is>
@@ -12709,7 +12709,7 @@
       <c r="Y278" s="4" t="n"/>
       <c r="Z278" s="4" t="n"/>
       <c r="AB278" s="4" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="AC278" s="4" t="inlineStr">
         <is>
@@ -12730,7 +12730,7 @@
       <c r="Y279" s="7" t="n"/>
       <c r="Z279" s="7" t="n"/>
       <c r="AB279" s="7" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AC279" s="7" t="inlineStr">
         <is>
@@ -12751,7 +12751,7 @@
       <c r="Y280" s="4" t="n"/>
       <c r="Z280" s="4" t="n"/>
       <c r="AB280" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AC280" s="4" t="inlineStr">
         <is>
@@ -12814,7 +12814,7 @@
       <c r="Y283" s="7" t="n"/>
       <c r="Z283" s="7" t="n"/>
       <c r="AB283" s="7" t="n">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="AC283" s="7" t="inlineStr">
         <is>
@@ -12835,7 +12835,7 @@
       <c r="Y284" s="4" t="n"/>
       <c r="Z284" s="4" t="n"/>
       <c r="AB284" s="4" t="n">
-        <v>38</v>
+        <v>143</v>
       </c>
       <c r="AC284" s="4" t="inlineStr">
         <is>
@@ -12856,7 +12856,7 @@
       <c r="Y285" s="7" t="n"/>
       <c r="Z285" s="7" t="n"/>
       <c r="AB285" s="7" t="n">
-        <v>143</v>
+        <v>3</v>
       </c>
       <c r="AC285" s="7" t="inlineStr">
         <is>
@@ -12961,7 +12961,7 @@
       <c r="Y290" s="4" t="n"/>
       <c r="Z290" s="4" t="n"/>
       <c r="AB290" s="4" t="n">
-        <v>170</v>
+        <v>205</v>
       </c>
       <c r="AC290" s="4" t="inlineStr">
         <is>
@@ -13003,7 +13003,7 @@
       <c r="Y292" s="4" t="n"/>
       <c r="Z292" s="4" t="n"/>
       <c r="AB292" s="4" t="n">
-        <v>205</v>
+        <v>170</v>
       </c>
       <c r="AC292" s="4" t="inlineStr">
         <is>
@@ -13024,7 +13024,7 @@
       <c r="Y293" s="7" t="n"/>
       <c r="Z293" s="7" t="n"/>
       <c r="AB293" s="7" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="AC293" s="7" t="inlineStr">
         <is>
@@ -13045,7 +13045,7 @@
       <c r="Y294" s="4" t="n"/>
       <c r="Z294" s="4" t="n"/>
       <c r="AB294" s="4" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="AC294" s="4" t="inlineStr">
         <is>
@@ -13066,7 +13066,7 @@
       <c r="Y295" s="7" t="n"/>
       <c r="Z295" s="7" t="n"/>
       <c r="AB295" s="7" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="AC295" s="7" t="inlineStr">
         <is>
@@ -13108,7 +13108,7 @@
       <c r="Y297" s="7" t="n"/>
       <c r="Z297" s="7" t="n"/>
       <c r="AB297" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC297" s="7" t="inlineStr">
         <is>
@@ -13129,7 +13129,7 @@
       <c r="Y298" s="4" t="n"/>
       <c r="Z298" s="4" t="n"/>
       <c r="AB298" s="4" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="AC298" s="4" t="inlineStr">
         <is>
@@ -13150,7 +13150,7 @@
       <c r="Y299" s="7" t="n"/>
       <c r="Z299" s="7" t="n"/>
       <c r="AB299" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AC299" s="7" t="inlineStr">
         <is>
@@ -13192,7 +13192,7 @@
       <c r="Y301" s="7" t="n"/>
       <c r="Z301" s="7" t="n"/>
       <c r="AB301" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AC301" s="7" t="inlineStr">
         <is>
@@ -13276,7 +13276,7 @@
       <c r="Y305" s="7" t="n"/>
       <c r="Z305" s="7" t="n"/>
       <c r="AB305" s="7" t="n">
-        <v>6</v>
+        <v>129</v>
       </c>
       <c r="AC305" s="7" t="inlineStr">
         <is>
@@ -13297,7 +13297,7 @@
       <c r="Y306" s="4" t="n"/>
       <c r="Z306" s="4" t="n"/>
       <c r="AB306" s="4" t="n">
-        <v>129</v>
+        <v>4</v>
       </c>
       <c r="AC306" s="4" t="inlineStr">
         <is>
@@ -13318,7 +13318,7 @@
       <c r="Y307" s="7" t="n"/>
       <c r="Z307" s="7" t="n"/>
       <c r="AB307" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC307" s="7" t="inlineStr">
         <is>
@@ -13612,7 +13612,7 @@
       <c r="Y321" s="7" t="n"/>
       <c r="Z321" s="7" t="n"/>
       <c r="AB321" s="7" t="n">
-        <v>126</v>
+        <v>2</v>
       </c>
       <c r="AC321" s="7" t="inlineStr">
         <is>
@@ -13633,7 +13633,7 @@
       <c r="Y322" s="4" t="n"/>
       <c r="Z322" s="4" t="n"/>
       <c r="AB322" s="4" t="n">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="AC322" s="4" t="inlineStr">
         <is>
@@ -13675,7 +13675,7 @@
       <c r="Y324" s="4" t="n"/>
       <c r="Z324" s="4" t="n"/>
       <c r="AB324" s="4" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="AC324" s="4" t="inlineStr">
         <is>
@@ -13696,7 +13696,7 @@
       <c r="Y325" s="7" t="n"/>
       <c r="Z325" s="7" t="n"/>
       <c r="AB325" s="7" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="AC325" s="7" t="inlineStr">
         <is>
@@ -13717,7 +13717,7 @@
       <c r="Y326" s="4" t="n"/>
       <c r="Z326" s="4" t="n"/>
       <c r="AB326" s="4" t="n">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="AC326" s="4" t="inlineStr">
         <is>
@@ -13738,7 +13738,7 @@
       <c r="Y327" s="7" t="n"/>
       <c r="Z327" s="7" t="n"/>
       <c r="AB327" s="7" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="AC327" s="7" t="inlineStr">
         <is>
@@ -13759,7 +13759,7 @@
       <c r="Y328" s="4" t="n"/>
       <c r="Z328" s="4" t="n"/>
       <c r="AB328" s="4" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="AC328" s="4" t="inlineStr">
         <is>
@@ -13780,7 +13780,7 @@
       <c r="Y329" s="7" t="n"/>
       <c r="Z329" s="7" t="n"/>
       <c r="AB329" s="7" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="AC329" s="7" t="inlineStr">
         <is>
@@ -13801,7 +13801,7 @@
       <c r="Y330" s="4" t="n"/>
       <c r="Z330" s="4" t="n"/>
       <c r="AB330" s="4" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="AC330" s="4" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
       <c r="Y332" s="4" t="n"/>
       <c r="Z332" s="4" t="n"/>
       <c r="AB332" s="4" t="n">
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="AC332" s="4" t="inlineStr">
         <is>
@@ -13864,7 +13864,7 @@
       <c r="Y333" s="7" t="n"/>
       <c r="Z333" s="7" t="n"/>
       <c r="AB333" s="7" t="n">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="AC333" s="7" t="inlineStr">
         <is>
@@ -13885,7 +13885,7 @@
       <c r="Y334" s="4" t="n"/>
       <c r="Z334" s="4" t="n"/>
       <c r="AB334" s="4" t="n">
-        <v>3</v>
+        <v>64</v>
       </c>
       <c r="AC334" s="4" t="inlineStr">
         <is>
@@ -13906,7 +13906,7 @@
       <c r="Y335" s="7" t="n"/>
       <c r="Z335" s="7" t="n"/>
       <c r="AB335" s="7" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="AC335" s="7" t="inlineStr">
         <is>
@@ -14499,7 +14499,7 @@
         </is>
       </c>
       <c r="AB5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
@@ -14585,7 +14585,7 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
@@ -14671,7 +14671,7 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
@@ -14757,7 +14757,7 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
@@ -15001,7 +15001,7 @@
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
@@ -15079,7 +15079,7 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -15547,7 +15547,7 @@
         </is>
       </c>
       <c r="AB18" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
@@ -15580,7 +15580,7 @@
         <v>2347</v>
       </c>
       <c r="X19" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -15589,11 +15589,11 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>glovo</t>
+          <t>Glovo</t>
         </is>
       </c>
       <c r="AB19" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
@@ -15635,11 +15635,11 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Glovo</t>
+          <t>glovo rider</t>
         </is>
       </c>
       <c r="AB20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
@@ -15672,7 +15672,7 @@
         <v>4098</v>
       </c>
       <c r="X21" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
@@ -15681,11 +15681,11 @@
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>glovo rider</t>
+          <t>glovo</t>
         </is>
       </c>
       <c r="AB21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
@@ -15731,7 +15731,7 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
@@ -15777,7 +15777,7 @@
         </is>
       </c>
       <c r="AB23" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC23" t="inlineStr">
         <is>
@@ -15810,7 +15810,7 @@
         <v>8276</v>
       </c>
       <c r="X24" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
@@ -15819,11 +15819,11 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB24" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
@@ -15856,7 +15856,7 @@
         <v>1</v>
       </c>
       <c r="X25" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
@@ -15865,11 +15865,11 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB25" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
@@ -15915,7 +15915,7 @@
         </is>
       </c>
       <c r="AB26" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="AC26" t="inlineStr">
         <is>
@@ -16191,7 +16191,7 @@
         </is>
       </c>
       <c r="AB32" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="AC32" t="inlineStr">
         <is>
@@ -16252,7 +16252,7 @@
         </is>
       </c>
       <c r="AB33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC33" t="inlineStr">
         <is>
@@ -16321,7 +16321,7 @@
         </is>
       </c>
       <c r="AB34" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="AC34" t="inlineStr">
         <is>
@@ -16362,7 +16362,7 @@
         </is>
       </c>
       <c r="AB35" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC35" t="inlineStr">
         <is>
@@ -16390,7 +16390,7 @@
         <v>1928</v>
       </c>
       <c r="X36" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -16399,11 +16399,11 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>glovo</t>
+          <t>Glovo</t>
         </is>
       </c>
       <c r="AB36" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AC36" t="inlineStr">
         <is>
@@ -16431,7 +16431,7 @@
         <v>2243</v>
       </c>
       <c r="X37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
@@ -16440,11 +16440,11 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>Glovo</t>
+          <t>glovo</t>
         </is>
       </c>
       <c r="AB37" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
@@ -16485,7 +16485,7 @@
         </is>
       </c>
       <c r="AB38" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
@@ -16526,7 +16526,7 @@
         </is>
       </c>
       <c r="AB39" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
@@ -16567,7 +16567,7 @@
         </is>
       </c>
       <c r="AB40" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="AC40" t="inlineStr">
         <is>
@@ -16595,7 +16595,7 @@
         <v>1</v>
       </c>
       <c r="X41" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
@@ -16604,7 +16604,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB41" t="n">
@@ -16636,7 +16636,7 @@
         <v>126</v>
       </c>
       <c r="X42" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
@@ -16645,11 +16645,11 @@
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB42" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="AC42" t="inlineStr">
         <is>
@@ -16882,7 +16882,7 @@
         <v>916</v>
       </c>
       <c r="X48" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -16891,11 +16891,11 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>Talabat</t>
+          <t>talabat</t>
         </is>
       </c>
       <c r="AB48" t="n">
-        <v>5</v>
+        <v>58</v>
       </c>
       <c r="AC48" t="inlineStr">
         <is>
@@ -16923,7 +16923,7 @@
         <v>1</v>
       </c>
       <c r="X49" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -16932,7 +16932,7 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Talabat</t>
         </is>
       </c>
       <c r="AB49" t="n">
@@ -16977,7 +16977,7 @@
         </is>
       </c>
       <c r="AB50" t="n">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="AC50" t="inlineStr">
         <is>
@@ -17018,7 +17018,7 @@
         </is>
       </c>
       <c r="AB51" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="AC51" t="inlineStr">
         <is>
@@ -17059,7 +17059,7 @@
         </is>
       </c>
       <c r="AB52" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="AC52" t="inlineStr">
         <is>
@@ -17128,7 +17128,7 @@
         <v>6904</v>
       </c>
       <c r="AB54" t="n">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="AC54" t="inlineStr">
         <is>
@@ -17156,7 +17156,7 @@
         <v>8440</v>
       </c>
       <c r="AB55" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="AC55" t="inlineStr">
         <is>
@@ -17184,7 +17184,7 @@
         <v>9811</v>
       </c>
       <c r="AB56" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AC56" t="inlineStr">
         <is>
@@ -17268,7 +17268,7 @@
         <v>2</v>
       </c>
       <c r="AB59" t="n">
-        <v>90</v>
+        <v>6</v>
       </c>
       <c r="AC59" t="inlineStr">
         <is>
@@ -17296,7 +17296,7 @@
         <v>349</v>
       </c>
       <c r="AB60" t="n">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="AC60" t="inlineStr">
         <is>
@@ -17380,7 +17380,7 @@
         <v>925</v>
       </c>
       <c r="AB63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AC63" t="inlineStr">
         <is>
@@ -17408,7 +17408,7 @@
         <v>1000</v>
       </c>
       <c r="AB64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC64" t="inlineStr">
         <is>
@@ -17436,7 +17436,7 @@
         <v>1284</v>
       </c>
       <c r="AB65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC65" t="inlineStr">
         <is>
@@ -17464,7 +17464,7 @@
         <v>2067</v>
       </c>
       <c r="AB66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC66" t="inlineStr">
         <is>
@@ -17492,7 +17492,7 @@
         <v>1</v>
       </c>
       <c r="AB67" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AC67" t="inlineStr">
         <is>
@@ -17520,7 +17520,7 @@
         <v>47</v>
       </c>
       <c r="AB68" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="AC68" t="inlineStr">
         <is>
@@ -17548,7 +17548,7 @@
         <v>98</v>
       </c>
       <c r="AB69" t="n">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="AC69" t="inlineStr">
         <is>
@@ -17604,7 +17604,7 @@
         <v>150</v>
       </c>
       <c r="AB71" t="n">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="AC71" t="inlineStr">
         <is>
@@ -17733,7 +17733,7 @@
     </row>
     <row r="77">
       <c r="AB77" t="n">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="AC77" t="inlineStr">
         <is>
@@ -17748,7 +17748,7 @@
     </row>
     <row r="78">
       <c r="AB78" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="AC78" t="inlineStr">
         <is>
@@ -17763,7 +17763,7 @@
     </row>
     <row r="79">
       <c r="AB79" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="AC79" t="inlineStr">
         <is>
@@ -17778,7 +17778,7 @@
     </row>
     <row r="80">
       <c r="AB80" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AC80" t="inlineStr">
         <is>
@@ -17793,7 +17793,7 @@
     </row>
     <row r="81">
       <c r="AB81" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC81" t="inlineStr">
         <is>
@@ -17823,7 +17823,7 @@
     </row>
     <row r="83">
       <c r="AB83" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="AC83" t="inlineStr">
         <is>
@@ -17838,7 +17838,7 @@
     </row>
     <row r="84">
       <c r="AB84" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="AC84" t="inlineStr">
         <is>
@@ -17883,7 +17883,7 @@
     </row>
     <row r="87">
       <c r="AB87" t="n">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="AC87" t="inlineStr">
         <is>
@@ -17898,7 +17898,7 @@
     </row>
     <row r="88">
       <c r="AB88" t="n">
-        <v>130</v>
+        <v>9</v>
       </c>
       <c r="AC88" t="inlineStr">
         <is>
@@ -17943,7 +17943,7 @@
     </row>
     <row r="91">
       <c r="AB91" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="AC91" t="inlineStr">
         <is>
@@ -17958,7 +17958,7 @@
     </row>
     <row r="92">
       <c r="AB92" t="n">
-        <v>3</v>
+        <v>73</v>
       </c>
       <c r="AC92" t="inlineStr">
         <is>
@@ -17973,7 +17973,7 @@
     </row>
     <row r="93">
       <c r="AB93" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC93" t="inlineStr">
         <is>
@@ -17988,7 +17988,7 @@
     </row>
     <row r="94">
       <c r="AB94" t="n">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="AC94" t="inlineStr">
         <is>
@@ -18003,7 +18003,7 @@
     </row>
     <row r="95">
       <c r="AB95" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="AC95" t="inlineStr">
         <is>
@@ -18033,7 +18033,7 @@
     </row>
     <row r="97">
       <c r="AB97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC97" t="inlineStr">
         <is>
@@ -18048,7 +18048,7 @@
     </row>
     <row r="98">
       <c r="AB98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC98" t="inlineStr">
         <is>
@@ -18078,7 +18078,7 @@
     </row>
     <row r="100">
       <c r="AB100" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="AC100" t="inlineStr">
         <is>
@@ -18093,7 +18093,7 @@
     </row>
     <row r="101">
       <c r="AB101" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AC101" t="inlineStr">
         <is>
@@ -18108,7 +18108,7 @@
     </row>
     <row r="102">
       <c r="AB102" t="n">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="AC102" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Updated device class report
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -1372,19 +1372,9 @@
       <c r="V2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="X2" s="4" t="n">
-        <v>68</v>
-      </c>
-      <c r="Y2" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z2" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foodpanda</t>
-        </is>
-      </c>
+      <c r="X2" s="4" t="n"/>
+      <c r="Y2" s="4" t="n"/>
+      <c r="Z2" s="4" t="n"/>
       <c r="AB2" s="4" t="n">
         <v>295</v>
       </c>
@@ -1457,19 +1447,9 @@
       <c r="V3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="X3" s="7" t="n">
-        <v>68</v>
-      </c>
-      <c r="Y3" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z3" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foodpanda</t>
-        </is>
-      </c>
+      <c r="X3" s="7" t="n"/>
+      <c r="Y3" s="7" t="n"/>
+      <c r="Z3" s="7" t="n"/>
       <c r="AB3" s="7" t="n">
         <v>6</v>
       </c>
@@ -1522,21 +1502,11 @@
       <c r="V4" s="4" t="n">
         <v>5519</v>
       </c>
-      <c r="X4" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="Y4" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z4" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foodora</t>
-        </is>
-      </c>
+      <c r="X4" s="4" t="n"/>
+      <c r="Y4" s="4" t="n"/>
+      <c r="Z4" s="4" t="n"/>
       <c r="AB4" s="4" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="AC4" s="4" t="inlineStr">
         <is>
@@ -1581,21 +1551,11 @@
       <c r="V5" s="7" t="n">
         <v>5569</v>
       </c>
-      <c r="X5" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y5" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z5" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foodora</t>
-        </is>
-      </c>
+      <c r="X5" s="7" t="n"/>
+      <c r="Y5" s="7" t="n"/>
+      <c r="Z5" s="7" t="n"/>
       <c r="AB5" s="7" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AC5" s="7" t="inlineStr">
         <is>
@@ -1646,21 +1606,11 @@
       <c r="V6" s="4" t="n">
         <v>15184</v>
       </c>
-      <c r="X6" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="Y6" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z6" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.talabat</t>
-        </is>
-      </c>
+      <c r="X6" s="4" t="n"/>
+      <c r="Y6" s="4" t="n"/>
+      <c r="Z6" s="4" t="n"/>
       <c r="AB6" s="4" t="n">
-        <v>162</v>
+        <v>5</v>
       </c>
       <c r="AC6" s="4" t="inlineStr">
         <is>
@@ -1711,19 +1661,9 @@
       <c r="V7" s="7" t="n">
         <v>15708</v>
       </c>
-      <c r="X7" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y7" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z7" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.talabat</t>
-        </is>
-      </c>
+      <c r="X7" s="7" t="n"/>
+      <c r="Y7" s="7" t="n"/>
+      <c r="Z7" s="7" t="n"/>
       <c r="AB7" s="7" t="n">
         <v>8</v>
       </c>
@@ -1776,21 +1716,11 @@
       <c r="V8" s="4" t="n">
         <v>87207</v>
       </c>
-      <c r="X8" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="Y8" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z8" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.talabat</t>
-        </is>
-      </c>
+      <c r="X8" s="4" t="n"/>
+      <c r="Y8" s="4" t="n"/>
+      <c r="Z8" s="4" t="n"/>
       <c r="AB8" s="4" t="n">
-        <v>5</v>
+        <v>162</v>
       </c>
       <c r="AC8" s="4" t="inlineStr">
         <is>
@@ -1835,21 +1765,11 @@
       <c r="V9" s="7" t="n">
         <v>86030</v>
       </c>
-      <c r="X9" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y9" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z9" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.pedidosya</t>
-        </is>
-      </c>
+      <c r="X9" s="7" t="n"/>
+      <c r="Y9" s="7" t="n"/>
+      <c r="Z9" s="7" t="n"/>
       <c r="AB9" s="7" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="AC9" s="7" t="inlineStr">
         <is>
@@ -1902,19 +1822,9 @@
       <c r="V10" s="4" t="n">
         <v>721</v>
       </c>
-      <c r="X10" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Y10" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z10" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.pedidosya</t>
-        </is>
-      </c>
+      <c r="X10" s="4" t="n"/>
+      <c r="Y10" s="4" t="n"/>
+      <c r="Z10" s="4" t="n"/>
       <c r="AB10" s="4" t="n">
         <v>5</v>
       </c>
@@ -1961,21 +1871,11 @@
       <c r="V11" s="7" t="n">
         <v>729</v>
       </c>
-      <c r="X11" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="Y11" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z11" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.pedidosya</t>
-        </is>
-      </c>
+      <c r="X11" s="7" t="n"/>
+      <c r="Y11" s="7" t="n"/>
+      <c r="Z11" s="7" t="n"/>
       <c r="AB11" s="7" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="AC11" s="7" t="inlineStr">
         <is>
@@ -2020,19 +1920,9 @@
       <c r="V12" s="4" t="n">
         <v>50559</v>
       </c>
-      <c r="X12" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="Y12" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z12" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.hungerstation</t>
-        </is>
-      </c>
+      <c r="X12" s="4" t="n"/>
+      <c r="Y12" s="4" t="n"/>
+      <c r="Z12" s="4" t="n"/>
       <c r="AB12" s="4" t="n">
         <v>57</v>
       </c>
@@ -2079,19 +1969,9 @@
       <c r="V13" s="7" t="n">
         <v>51501</v>
       </c>
-      <c r="X13" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="Y13" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z13" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.hungerstation</t>
-        </is>
-      </c>
+      <c r="X13" s="7" t="n"/>
+      <c r="Y13" s="7" t="n"/>
+      <c r="Z13" s="7" t="n"/>
       <c r="AB13" s="7" t="n">
         <v>2</v>
       </c>
@@ -2138,19 +2018,9 @@
       <c r="V14" s="4" t="n">
         <v>11599</v>
       </c>
-      <c r="X14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y14" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z14" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.hungerstation</t>
-        </is>
-      </c>
+      <c r="X14" s="4" t="n"/>
+      <c r="Y14" s="4" t="n"/>
+      <c r="Z14" s="4" t="n"/>
       <c r="AB14" s="4" t="n">
         <v>3</v>
       </c>
@@ -2197,19 +2067,9 @@
       <c r="V15" s="7" t="n">
         <v>11522</v>
       </c>
-      <c r="X15" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="Y15" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z15" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
+      <c r="X15" s="7" t="n"/>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="n"/>
       <c r="AB15" s="7" t="n">
         <v>13</v>
       </c>
@@ -2256,19 +2116,9 @@
       <c r="V16" s="4" t="n">
         <v>26509</v>
       </c>
-      <c r="X16" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y16" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z16" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
+      <c r="X16" s="4" t="n"/>
+      <c r="Y16" s="4" t="n"/>
+      <c r="Z16" s="4" t="n"/>
       <c r="AB16" s="4" t="n">
         <v>188</v>
       </c>
@@ -2315,19 +2165,9 @@
       <c r="V17" s="7" t="n">
         <v>26876</v>
       </c>
-      <c r="X17" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y17" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z17" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
+      <c r="X17" s="7" t="n"/>
+      <c r="Y17" s="7" t="n"/>
+      <c r="Z17" s="7" t="n"/>
       <c r="AB17" s="7" t="n">
         <v>2</v>
       </c>
@@ -2374,19 +2214,9 @@
       <c r="V18" s="4" t="n">
         <v>17949</v>
       </c>
-      <c r="X18" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y18" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z18" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
+      <c r="X18" s="4" t="n"/>
+      <c r="Y18" s="4" t="n"/>
+      <c r="Z18" s="4" t="n"/>
       <c r="AB18" s="4" t="n">
         <v>19</v>
       </c>
@@ -2433,19 +2263,9 @@
       <c r="V19" s="7" t="n">
         <v>17549</v>
       </c>
-      <c r="X19" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="Y19" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z19" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
+      <c r="X19" s="7" t="n"/>
+      <c r="Y19" s="7" t="n"/>
+      <c r="Z19" s="7" t="n"/>
       <c r="AB19" s="7" t="n">
         <v>2</v>
       </c>
@@ -2492,19 +2312,9 @@
       <c r="V20" s="4" t="n">
         <v>745</v>
       </c>
-      <c r="X20" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="Y20" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="Z20" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+      <c r="X20" s="4" t="n"/>
+      <c r="Y20" s="4" t="n"/>
+      <c r="Z20" s="4" t="n"/>
       <c r="AB20" s="4" t="n">
         <v>1</v>
       </c>
@@ -2551,19 +2361,9 @@
       <c r="V21" s="7" t="n">
         <v>763</v>
       </c>
-      <c r="X21" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="Y21" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z21" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+      <c r="X21" s="7" t="n"/>
+      <c r="Y21" s="7" t="n"/>
+      <c r="Z21" s="7" t="n"/>
       <c r="AB21" s="7" t="n">
         <v>4</v>
       </c>
@@ -2610,19 +2410,9 @@
       <c r="V22" s="4" t="n">
         <v>2142</v>
       </c>
-      <c r="X22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y22" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z22" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+      <c r="X22" s="4" t="n"/>
+      <c r="Y22" s="4" t="n"/>
+      <c r="Z22" s="4" t="n"/>
       <c r="AB22" s="4" t="n">
         <v>327</v>
       </c>
@@ -2669,19 +2459,9 @@
       <c r="V23" s="7" t="n">
         <v>2408</v>
       </c>
-      <c r="X23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y23" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="Z23" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foody</t>
-        </is>
-      </c>
+      <c r="X23" s="7" t="n"/>
+      <c r="Y23" s="7" t="n"/>
+      <c r="Z23" s="7" t="n"/>
       <c r="AB23" s="7" t="n">
         <v>2</v>
       </c>
@@ -2800,7 +2580,7 @@
       <c r="Y26" s="4" t="n"/>
       <c r="Z26" s="4" t="n"/>
       <c r="AB26" s="4" t="n">
-        <v>2</v>
+        <v>155</v>
       </c>
       <c r="AC26" s="4" t="inlineStr">
         <is>
@@ -2839,7 +2619,7 @@
       <c r="Y27" s="7" t="n"/>
       <c r="Z27" s="7" t="n"/>
       <c r="AB27" s="7" t="n">
-        <v>155</v>
+        <v>2</v>
       </c>
       <c r="AC27" s="7" t="inlineStr">
         <is>
@@ -2878,7 +2658,7 @@
       <c r="Y28" s="4" t="n"/>
       <c r="Z28" s="4" t="n"/>
       <c r="AB28" s="4" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="AC28" s="4" t="inlineStr">
         <is>
@@ -2917,7 +2697,7 @@
       <c r="Y29" s="7" t="n"/>
       <c r="Z29" s="7" t="n"/>
       <c r="AB29" s="7" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="AC29" s="7" t="inlineStr">
         <is>
@@ -2995,7 +2775,7 @@
       <c r="Y31" s="7" t="n"/>
       <c r="Z31" s="7" t="n"/>
       <c r="AB31" s="7" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="AC31" s="7" t="inlineStr">
         <is>
@@ -3043,7 +2823,7 @@
       <c r="Y32" s="4" t="n"/>
       <c r="Z32" s="4" t="n"/>
       <c r="AB32" s="4" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AC32" s="4" t="inlineStr">
         <is>
@@ -3738,7 +3518,7 @@
         <v>2322</v>
       </c>
       <c r="AB8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
@@ -3771,7 +3551,7 @@
         <v>3533</v>
       </c>
       <c r="AB9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
@@ -4111,7 +3891,7 @@
         <v>820</v>
       </c>
       <c r="AB19" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
@@ -4144,7 +3924,7 @@
         <v>90</v>
       </c>
       <c r="AB20" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
@@ -4177,7 +3957,7 @@
         <v>119</v>
       </c>
       <c r="AB21" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
@@ -4197,7 +3977,7 @@
         </is>
       </c>
       <c r="AB22" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
@@ -4217,7 +3997,7 @@
         </is>
       </c>
       <c r="AB23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AC23" t="inlineStr">
         <is>
@@ -4257,7 +4037,7 @@
         </is>
       </c>
       <c r="AB25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
@@ -4277,7 +4057,7 @@
         </is>
       </c>
       <c r="AB26" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AC26" t="inlineStr">
         <is>
@@ -4297,7 +4077,7 @@
         </is>
       </c>
       <c r="AB27" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AC27" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Updated report by fixing crash query
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -738,7 +738,7 @@
         <v>0.86</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>78203</v>
@@ -774,7 +774,7 @@
         <v>0.86</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14946</v>
@@ -810,7 +810,7 @@
         <v>0.86</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>16988</v>
@@ -846,7 +846,7 @@
         <v>0.86</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>20641</v>
@@ -882,7 +882,7 @@
         <v>0.86</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>10630</v>
@@ -918,7 +918,7 @@
         <v>0.86</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>2186</v>
@@ -954,7 +954,7 @@
         <v>0.86</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>46896</v>
@@ -990,7 +990,7 @@
         <v>0.86</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>731</v>
@@ -1026,7 +1026,7 @@
         <v>0.86</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>5258</v>
@@ -1062,7 +1062,7 @@
         <v>0.86</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>729</v>
@@ -1189,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD41"/>
+  <dimension ref="A1:AD62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1372,11 +1372,21 @@
       <c r="V2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="X2" s="4" t="n"/>
-      <c r="Y2" s="4" t="n"/>
-      <c r="Z2" s="4" t="n"/>
+      <c r="X2" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="Y2" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z2" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB2" s="4" t="n">
-        <v>295</v>
+        <v>6</v>
       </c>
       <c r="AC2" s="4" t="inlineStr">
         <is>
@@ -1447,11 +1457,21 @@
       <c r="V3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="X3" s="7" t="n"/>
-      <c r="Y3" s="7" t="n"/>
-      <c r="Z3" s="7" t="n"/>
+      <c r="X3" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="Y3" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB3" s="7" t="n">
-        <v>6</v>
+        <v>295</v>
       </c>
       <c r="AC3" s="7" t="inlineStr">
         <is>
@@ -1478,35 +1498,65 @@
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
+      <c r="D4" s="4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C4)</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C4)</f>
+        <v/>
+      </c>
       <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
+      <c r="G4" s="4">
+        <f>ROUND(MAX(0,MIN(100,(1-E4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>MIN(1,(G4-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
+      <c r="K4" s="4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)))),2)</f>
+        <v/>
+      </c>
+      <c r="M4" s="4">
+        <f>MAX(0,(L4-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N4" s="4">
+        <f>$B$2+H4+M4</f>
+        <v/>
+      </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
-      </c>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr"/>
       <c r="V4" s="4" t="n">
-        <v>5519</v>
-      </c>
-      <c r="X4" s="4" t="n"/>
-      <c r="Y4" s="4" t="n"/>
-      <c r="Z4" s="4" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB4" s="4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="AC4" s="4" t="inlineStr">
         <is>
@@ -1540,7 +1590,7 @@
       <c r="N5" s="7" t="n"/>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
@@ -1549,13 +1599,23 @@
         </is>
       </c>
       <c r="V5" s="7" t="n">
-        <v>5569</v>
-      </c>
-      <c r="X5" s="7" t="n"/>
-      <c r="Y5" s="7" t="n"/>
-      <c r="Z5" s="7" t="n"/>
+        <v>5519</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
       <c r="AB5" s="7" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="AC5" s="7" t="inlineStr">
         <is>
@@ -1595,20 +1655,30 @@
       <c r="N6" s="4" t="n"/>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="n">
+        <v>5569</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Y6" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z6" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.foodora</t>
         </is>
       </c>
-      <c r="V6" s="4" t="n">
-        <v>15184</v>
-      </c>
-      <c r="X6" s="4" t="n"/>
-      <c r="Y6" s="4" t="n"/>
-      <c r="Z6" s="4" t="n"/>
       <c r="AB6" s="4" t="n">
         <v>5</v>
       </c>
@@ -1650,20 +1720,30 @@
       <c r="N7" s="7" t="n"/>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="V7" s="7" t="n">
+        <v>5621</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.foodora</t>
         </is>
       </c>
-      <c r="V7" s="7" t="n">
-        <v>15708</v>
-      </c>
-      <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
       <c r="AB7" s="7" t="n">
         <v>8</v>
       </c>
@@ -1710,15 +1790,25 @@
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V8" s="4" t="n">
-        <v>87207</v>
-      </c>
-      <c r="X8" s="4" t="n"/>
-      <c r="Y8" s="4" t="n"/>
-      <c r="Z8" s="4" t="n"/>
+        <v>15184</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="Y8" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z8" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB8" s="4" t="n">
         <v>162</v>
       </c>
@@ -1759,15 +1849,25 @@
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V9" s="7" t="n">
-        <v>86030</v>
-      </c>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="7" t="n"/>
-      <c r="Z9" s="7" t="n"/>
+        <v>15708</v>
+      </c>
+      <c r="X9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y9" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z9" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB9" s="7" t="n">
         <v>50</v>
       </c>
@@ -1811,20 +1911,30 @@
       <c r="N10" s="4" t="n"/>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V10" s="4" t="n">
-        <v>721</v>
-      </c>
-      <c r="X10" s="4" t="n"/>
-      <c r="Y10" s="4" t="n"/>
-      <c r="Z10" s="4" t="n"/>
+        <v>15056</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="Y10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z10" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB10" s="4" t="n">
         <v>5</v>
       </c>
@@ -1860,20 +1970,30 @@
       <c r="N11" s="7" t="n"/>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V11" s="7" t="n">
-        <v>729</v>
-      </c>
-      <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
+        <v>87207</v>
+      </c>
+      <c r="X11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z11" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB11" s="7" t="n">
         <v>4</v>
       </c>
@@ -1909,22 +2029,32 @@
       <c r="N12" s="4" t="n"/>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V12" s="4" t="n">
-        <v>50559</v>
-      </c>
-      <c r="X12" s="4" t="n"/>
-      <c r="Y12" s="4" t="n"/>
-      <c r="Z12" s="4" t="n"/>
+        <v>86030</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="Y12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z12" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
       <c r="AB12" s="4" t="n">
-        <v>57</v>
+        <v>2</v>
       </c>
       <c r="AC12" s="4" t="inlineStr">
         <is>
@@ -1958,22 +2088,32 @@
       <c r="N13" s="7" t="n"/>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V13" s="7" t="n">
-        <v>51501</v>
-      </c>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
+        <v>82667</v>
+      </c>
+      <c r="X13" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z13" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB13" s="7" t="n">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="AC13" s="7" t="inlineStr">
         <is>
@@ -2012,15 +2152,25 @@
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V14" s="4" t="n">
-        <v>11599</v>
-      </c>
-      <c r="X14" s="4" t="n"/>
-      <c r="Y14" s="4" t="n"/>
-      <c r="Z14" s="4" t="n"/>
+        <v>721</v>
+      </c>
+      <c r="X14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z14" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB14" s="4" t="n">
         <v>3</v>
       </c>
@@ -2061,15 +2211,25 @@
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.foody</t>
         </is>
       </c>
       <c r="V15" s="7" t="n">
-        <v>11522</v>
-      </c>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
+        <v>729</v>
+      </c>
+      <c r="X15" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y15" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z15" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
       <c r="AB15" s="7" t="n">
         <v>13</v>
       </c>
@@ -2105,20 +2265,30 @@
       <c r="N16" s="4" t="n"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>717</v>
+      </c>
+      <c r="X16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="Y16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V16" s="4" t="n">
-        <v>26509</v>
-      </c>
-      <c r="X16" s="4" t="n"/>
-      <c r="Y16" s="4" t="n"/>
-      <c r="Z16" s="4" t="n"/>
       <c r="AB16" s="4" t="n">
         <v>188</v>
       </c>
@@ -2154,20 +2324,30 @@
       <c r="N17" s="7" t="n"/>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="V17" s="7" t="n">
+        <v>50559</v>
+      </c>
+      <c r="X17" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y17" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z17" s="7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
-      <c r="V17" s="7" t="n">
-        <v>26876</v>
-      </c>
-      <c r="X17" s="7" t="n"/>
-      <c r="Y17" s="7" t="n"/>
-      <c r="Z17" s="7" t="n"/>
       <c r="AB17" s="7" t="n">
         <v>2</v>
       </c>
@@ -2203,20 +2383,30 @@
       <c r="N18" s="4" t="n"/>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V18" s="4" t="n">
-        <v>17949</v>
-      </c>
-      <c r="X18" s="4" t="n"/>
-      <c r="Y18" s="4" t="n"/>
-      <c r="Z18" s="4" t="n"/>
+        <v>51501</v>
+      </c>
+      <c r="X18" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y18" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z18" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
       <c r="AB18" s="4" t="n">
         <v>19</v>
       </c>
@@ -2252,20 +2442,30 @@
       <c r="N19" s="7" t="n"/>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V19" s="7" t="n">
-        <v>17549</v>
-      </c>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
+        <v>51715</v>
+      </c>
+      <c r="X19" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="Y19" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z19" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
       <c r="AB19" s="7" t="n">
         <v>2</v>
       </c>
@@ -2306,17 +2506,27 @@
       </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V20" s="4" t="n">
-        <v>745</v>
-      </c>
-      <c r="X20" s="4" t="n"/>
-      <c r="Y20" s="4" t="n"/>
-      <c r="Z20" s="4" t="n"/>
+        <v>11599</v>
+      </c>
+      <c r="X20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z20" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
       <c r="AB20" s="4" t="n">
-        <v>1</v>
+        <v>327</v>
       </c>
       <c r="AC20" s="4" t="inlineStr">
         <is>
@@ -2355,15 +2565,25 @@
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V21" s="7" t="n">
-        <v>763</v>
-      </c>
-      <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="n"/>
-      <c r="Z21" s="7" t="n"/>
+        <v>11522</v>
+      </c>
+      <c r="X21" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="Y21" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z21" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
       <c r="AB21" s="7" t="n">
         <v>4</v>
       </c>
@@ -2399,22 +2619,32 @@
       <c r="N22" s="4" t="n"/>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V22" s="4" t="n">
-        <v>2142</v>
-      </c>
-      <c r="X22" s="4" t="n"/>
-      <c r="Y22" s="4" t="n"/>
-      <c r="Z22" s="4" t="n"/>
+        <v>11614</v>
+      </c>
+      <c r="X22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y22" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z22" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
       <c r="AB22" s="4" t="n">
-        <v>327</v>
+        <v>1</v>
       </c>
       <c r="AC22" s="4" t="inlineStr">
         <is>
@@ -2448,20 +2678,30 @@
       <c r="N23" s="7" t="n"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V23" s="7" t="n">
-        <v>2408</v>
-      </c>
-      <c r="X23" s="7" t="n"/>
-      <c r="Y23" s="7" t="n"/>
-      <c r="Z23" s="7" t="n"/>
+        <v>26509</v>
+      </c>
+      <c r="X23" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="Y23" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z23" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB23" s="7" t="n">
         <v>2</v>
       </c>
@@ -2495,12 +2735,32 @@
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="4" t="n"/>
-      <c r="T24" s="4" t="n"/>
-      <c r="U24" s="4" t="n"/>
-      <c r="V24" s="4" t="n"/>
-      <c r="X24" s="4" t="n"/>
-      <c r="Y24" s="4" t="n"/>
-      <c r="Z24" s="4" t="n"/>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V24" s="4" t="n">
+        <v>26876</v>
+      </c>
+      <c r="X24" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y24" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z24" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB24" s="4" t="n">
         <v>29</v>
       </c>
@@ -2534,12 +2794,32 @@
       <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="7" t="n"/>
-      <c r="T25" s="7" t="n"/>
-      <c r="U25" s="7" t="n"/>
-      <c r="V25" s="7" t="n"/>
-      <c r="X25" s="7" t="n"/>
-      <c r="Y25" s="7" t="n"/>
-      <c r="Z25" s="7" t="n"/>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U25" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="V25" s="7" t="n">
+        <v>27154</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y25" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z25" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB25" s="7" t="n">
         <v>3</v>
       </c>
@@ -2573,12 +2853,32 @@
       <c r="L26" s="4" t="n"/>
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="4" t="n"/>
-      <c r="T26" s="4" t="n"/>
-      <c r="U26" s="4" t="n"/>
-      <c r="V26" s="4" t="n"/>
-      <c r="X26" s="4" t="n"/>
-      <c r="Y26" s="4" t="n"/>
-      <c r="Z26" s="4" t="n"/>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V26" s="4" t="n">
+        <v>17949</v>
+      </c>
+      <c r="X26" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="Y26" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z26" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB26" s="4" t="n">
         <v>155</v>
       </c>
@@ -2612,12 +2912,32 @@
       <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="n"/>
       <c r="N27" s="7" t="n"/>
-      <c r="T27" s="7" t="n"/>
-      <c r="U27" s="7" t="n"/>
-      <c r="V27" s="7" t="n"/>
-      <c r="X27" s="7" t="n"/>
-      <c r="Y27" s="7" t="n"/>
-      <c r="Z27" s="7" t="n"/>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U27" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V27" s="7" t="n">
+        <v>17549</v>
+      </c>
+      <c r="X27" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y27" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z27" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB27" s="7" t="n">
         <v>2</v>
       </c>
@@ -2651,12 +2971,32 @@
       <c r="L28" s="4" t="n"/>
       <c r="M28" s="4" t="n"/>
       <c r="N28" s="4" t="n"/>
-      <c r="T28" s="4" t="n"/>
-      <c r="U28" s="4" t="n"/>
-      <c r="V28" s="4" t="n"/>
-      <c r="X28" s="4" t="n"/>
-      <c r="Y28" s="4" t="n"/>
-      <c r="Z28" s="4" t="n"/>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="n">
+        <v>17646</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y28" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z28" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB28" s="4" t="n">
         <v>4</v>
       </c>
@@ -2690,14 +3030,34 @@
       <c r="L29" s="7" t="n"/>
       <c r="M29" s="7" t="n"/>
       <c r="N29" s="7" t="n"/>
-      <c r="T29" s="7" t="n"/>
-      <c r="U29" s="7" t="n"/>
-      <c r="V29" s="7" t="n"/>
-      <c r="X29" s="7" t="n"/>
-      <c r="Y29" s="7" t="n"/>
-      <c r="Z29" s="7" t="n"/>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U29" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V29" s="7" t="n">
+        <v>745</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y29" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z29" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB29" s="7" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="AC29" s="7" t="inlineStr">
         <is>
@@ -2729,14 +3089,34 @@
       <c r="L30" s="4" t="n"/>
       <c r="M30" s="4" t="n"/>
       <c r="N30" s="4" t="n"/>
-      <c r="T30" s="4" t="n"/>
-      <c r="U30" s="4" t="n"/>
-      <c r="V30" s="4" t="n"/>
-      <c r="X30" s="4" t="n"/>
-      <c r="Y30" s="4" t="n"/>
-      <c r="Z30" s="4" t="n"/>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="n">
+        <v>763</v>
+      </c>
+      <c r="X30" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="Y30" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z30" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
       <c r="AB30" s="4" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="AC30" s="4" t="inlineStr">
         <is>
@@ -2768,14 +3148,34 @@
       <c r="L31" s="7" t="n"/>
       <c r="M31" s="7" t="n"/>
       <c r="N31" s="7" t="n"/>
-      <c r="T31" s="7" t="n"/>
-      <c r="U31" s="7" t="n"/>
-      <c r="V31" s="7" t="n"/>
-      <c r="X31" s="7" t="n"/>
-      <c r="Y31" s="7" t="n"/>
-      <c r="Z31" s="7" t="n"/>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U31" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V31" s="7" t="n">
+        <v>740</v>
+      </c>
+      <c r="X31" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y31" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z31" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB31" s="7" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="AC31" s="7" t="inlineStr">
         <is>
@@ -2816,14 +3216,34 @@
           <t>Projected AQS including hangs</t>
         </is>
       </c>
-      <c r="T32" s="4" t="n"/>
-      <c r="U32" s="4" t="n"/>
-      <c r="V32" s="4" t="n"/>
-      <c r="X32" s="4" t="n"/>
-      <c r="Y32" s="4" t="n"/>
-      <c r="Z32" s="4" t="n"/>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="n">
+        <v>2142</v>
+      </c>
+      <c r="X32" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y32" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z32" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB32" s="4" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="AC32" s="4" t="inlineStr">
         <is>
@@ -2838,7 +3258,7 @@
     </row>
     <row r="33">
       <c r="D33" s="26">
-        <f>AVERAGE(D2:D3)</f>
+        <f>AVERAGE(D2:D4)</f>
         <v/>
       </c>
       <c r="E33" s="27" t="n"/>
@@ -2848,7 +3268,7 @@
         <v/>
       </c>
       <c r="H33" s="29">
-        <f>AVERAGE(H2:H3)</f>
+        <f>AVERAGE(H2:H4)</f>
         <v/>
       </c>
       <c r="I33" s="29">
@@ -2869,12 +3289,32 @@
         <f>$B$2+MAX(0,(G33-$B$3)/($B$4-$B$3)*($B$1-$B$8))+M33</f>
         <v/>
       </c>
-      <c r="T33" s="7" t="n"/>
-      <c r="U33" s="7" t="n"/>
-      <c r="V33" s="7" t="n"/>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="7" t="n"/>
-      <c r="Z33" s="7" t="n"/>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U33" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V33" s="7" t="n">
+        <v>2408</v>
+      </c>
+      <c r="X33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y33" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z33" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB33" s="7" t="n">
         <v>1</v>
       </c>
@@ -2890,12 +3330,32 @@
       </c>
     </row>
     <row r="34">
-      <c r="T34" s="4" t="n"/>
-      <c r="U34" s="4" t="n"/>
-      <c r="V34" s="4" t="n"/>
-      <c r="X34" s="4" t="n"/>
-      <c r="Y34" s="4" t="n"/>
-      <c r="Z34" s="4" t="n"/>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.yemeksepeti</t>
+        </is>
+      </c>
+      <c r="V34" s="4" t="n">
+        <v>2141</v>
+      </c>
+      <c r="X34" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y34" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z34" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB34" s="4" t="n">
         <v>5</v>
       </c>
@@ -2914,11 +3374,21 @@
       <c r="T35" s="7" t="n"/>
       <c r="U35" s="7" t="n"/>
       <c r="V35" s="7" t="n"/>
-      <c r="X35" s="7" t="n"/>
-      <c r="Y35" s="7" t="n"/>
-      <c r="Z35" s="7" t="n"/>
+      <c r="X35" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y35" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z35" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
       <c r="AB35" s="7" t="n">
-        <v>10</v>
+        <v>180</v>
       </c>
       <c r="AC35" s="7" t="inlineStr">
         <is>
@@ -2935,11 +3405,21 @@
       <c r="T36" s="4" t="n"/>
       <c r="U36" s="4" t="n"/>
       <c r="V36" s="4" t="n"/>
-      <c r="X36" s="4" t="n"/>
-      <c r="Y36" s="4" t="n"/>
-      <c r="Z36" s="4" t="n"/>
+      <c r="X36" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y36" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z36" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
       <c r="AB36" s="4" t="n">
-        <v>180</v>
+        <v>2</v>
       </c>
       <c r="AC36" s="4" t="inlineStr">
         <is>
@@ -2960,7 +3440,7 @@
       <c r="Y37" s="7" t="n"/>
       <c r="Z37" s="7" t="n"/>
       <c r="AB37" s="7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AC37" s="7" t="inlineStr">
         <is>
@@ -3052,6 +3532,447 @@
         </is>
       </c>
       <c r="AD41" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="T42" s="4" t="n"/>
+      <c r="U42" s="4" t="n"/>
+      <c r="V42" s="4" t="n"/>
+      <c r="X42" s="4" t="n"/>
+      <c r="Y42" s="4" t="n"/>
+      <c r="Z42" s="4" t="n"/>
+      <c r="AB42" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD42" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="T43" s="7" t="n"/>
+      <c r="U43" s="7" t="n"/>
+      <c r="V43" s="7" t="n"/>
+      <c r="X43" s="7" t="n"/>
+      <c r="Y43" s="7" t="n"/>
+      <c r="Z43" s="7" t="n"/>
+      <c r="AB43" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC43" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD43" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="T44" s="4" t="n"/>
+      <c r="U44" s="4" t="n"/>
+      <c r="V44" s="4" t="n"/>
+      <c r="X44" s="4" t="n"/>
+      <c r="Y44" s="4" t="n"/>
+      <c r="Z44" s="4" t="n"/>
+      <c r="AB44" s="4" t="n">
+        <v>276</v>
+      </c>
+      <c r="AC44" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD44" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="T45" s="7" t="n"/>
+      <c r="U45" s="7" t="n"/>
+      <c r="V45" s="7" t="n"/>
+      <c r="X45" s="7" t="n"/>
+      <c r="Y45" s="7" t="n"/>
+      <c r="Z45" s="7" t="n"/>
+      <c r="AB45" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="AC45" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD45" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="T46" s="4" t="n"/>
+      <c r="U46" s="4" t="n"/>
+      <c r="V46" s="4" t="n"/>
+      <c r="X46" s="4" t="n"/>
+      <c r="Y46" s="4" t="n"/>
+      <c r="Z46" s="4" t="n"/>
+      <c r="AB46" s="4" t="n">
+        <v>175</v>
+      </c>
+      <c r="AC46" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD46" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="T47" s="7" t="n"/>
+      <c r="U47" s="7" t="n"/>
+      <c r="V47" s="7" t="n"/>
+      <c r="X47" s="7" t="n"/>
+      <c r="Y47" s="7" t="n"/>
+      <c r="Z47" s="7" t="n"/>
+      <c r="AB47" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC47" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD47" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="T48" s="4" t="n"/>
+      <c r="U48" s="4" t="n"/>
+      <c r="V48" s="4" t="n"/>
+      <c r="X48" s="4" t="n"/>
+      <c r="Y48" s="4" t="n"/>
+      <c r="Z48" s="4" t="n"/>
+      <c r="AB48" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC48" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD48" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="T49" s="7" t="n"/>
+      <c r="U49" s="7" t="n"/>
+      <c r="V49" s="7" t="n"/>
+      <c r="X49" s="7" t="n"/>
+      <c r="Y49" s="7" t="n"/>
+      <c r="Z49" s="7" t="n"/>
+      <c r="AB49" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="AC49" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD49" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="T50" s="4" t="n"/>
+      <c r="U50" s="4" t="n"/>
+      <c r="V50" s="4" t="n"/>
+      <c r="X50" s="4" t="n"/>
+      <c r="Y50" s="4" t="n"/>
+      <c r="Z50" s="4" t="n"/>
+      <c r="AB50" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD50" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="T51" s="7" t="n"/>
+      <c r="U51" s="7" t="n"/>
+      <c r="V51" s="7" t="n"/>
+      <c r="X51" s="7" t="n"/>
+      <c r="Y51" s="7" t="n"/>
+      <c r="Z51" s="7" t="n"/>
+      <c r="AB51" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC51" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD51" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="T52" s="4" t="n"/>
+      <c r="U52" s="4" t="n"/>
+      <c r="V52" s="4" t="n"/>
+      <c r="X52" s="4" t="n"/>
+      <c r="Y52" s="4" t="n"/>
+      <c r="Z52" s="4" t="n"/>
+      <c r="AB52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC52" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD52" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="T53" s="7" t="n"/>
+      <c r="U53" s="7" t="n"/>
+      <c r="V53" s="7" t="n"/>
+      <c r="X53" s="7" t="n"/>
+      <c r="Y53" s="7" t="n"/>
+      <c r="Z53" s="7" t="n"/>
+      <c r="AB53" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC53" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD53" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="T54" s="4" t="n"/>
+      <c r="U54" s="4" t="n"/>
+      <c r="V54" s="4" t="n"/>
+      <c r="X54" s="4" t="n"/>
+      <c r="Y54" s="4" t="n"/>
+      <c r="Z54" s="4" t="n"/>
+      <c r="AB54" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD54" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="T55" s="7" t="n"/>
+      <c r="U55" s="7" t="n"/>
+      <c r="V55" s="7" t="n"/>
+      <c r="X55" s="7" t="n"/>
+      <c r="Y55" s="7" t="n"/>
+      <c r="Z55" s="7" t="n"/>
+      <c r="AB55" s="7" t="n">
+        <v>197</v>
+      </c>
+      <c r="AC55" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD55" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="T56" s="4" t="n"/>
+      <c r="U56" s="4" t="n"/>
+      <c r="V56" s="4" t="n"/>
+      <c r="X56" s="4" t="n"/>
+      <c r="Y56" s="4" t="n"/>
+      <c r="Z56" s="4" t="n"/>
+      <c r="AB56" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="T57" s="7" t="n"/>
+      <c r="U57" s="7" t="n"/>
+      <c r="V57" s="7" t="n"/>
+      <c r="X57" s="7" t="n"/>
+      <c r="Y57" s="7" t="n"/>
+      <c r="Z57" s="7" t="n"/>
+      <c r="AB57" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC57" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD57" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="T58" s="4" t="n"/>
+      <c r="U58" s="4" t="n"/>
+      <c r="V58" s="4" t="n"/>
+      <c r="X58" s="4" t="n"/>
+      <c r="Y58" s="4" t="n"/>
+      <c r="Z58" s="4" t="n"/>
+      <c r="AB58" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC58" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD58" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="T59" s="7" t="n"/>
+      <c r="U59" s="7" t="n"/>
+      <c r="V59" s="7" t="n"/>
+      <c r="X59" s="7" t="n"/>
+      <c r="Y59" s="7" t="n"/>
+      <c r="Z59" s="7" t="n"/>
+      <c r="AB59" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC59" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD59" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="T60" s="4" t="n"/>
+      <c r="U60" s="4" t="n"/>
+      <c r="V60" s="4" t="n"/>
+      <c r="X60" s="4" t="n"/>
+      <c r="Y60" s="4" t="n"/>
+      <c r="Z60" s="4" t="n"/>
+      <c r="AB60" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC60" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD60" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="T61" s="7" t="n"/>
+      <c r="U61" s="7" t="n"/>
+      <c r="V61" s="7" t="n"/>
+      <c r="X61" s="7" t="n"/>
+      <c r="Y61" s="7" t="n"/>
+      <c r="Z61" s="7" t="n"/>
+      <c r="AB61" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC61" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD61" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="T62" s="4" t="n"/>
+      <c r="U62" s="4" t="n"/>
+      <c r="V62" s="4" t="n"/>
+      <c r="X62" s="4" t="n"/>
+      <c r="Y62" s="4" t="n"/>
+      <c r="Z62" s="4" t="n"/>
+      <c r="AB62" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AC62" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD62" s="4" t="inlineStr">
         <is>
           <t>com.logistics.rider.foody</t>
         </is>
@@ -3073,7 +3994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD33"/>
+  <dimension ref="A1:AD49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3247,8 +4168,21 @@
       <c r="V2" t="n">
         <v>7773</v>
       </c>
+      <c r="X2" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB2" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
@@ -3320,8 +4254,21 @@
       <c r="V3" t="n">
         <v>10781</v>
       </c>
+      <c r="X3" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
       <c r="AB3" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
@@ -3348,21 +4295,66 @@
           <t>2026-09-03</t>
         </is>
       </c>
+      <c r="D4">
+        <f>SUMIFS(V:V,U:U,"*"&amp;$B$10&amp;"*",T:T,C4)</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>SUMIFS(X:X,Z:Z,"*"&amp;$B$10&amp;"*",Y:Y,C4)</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>ROUND(MAX(0,MIN(100,(1-E4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30))*100)),2)</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>MIN(1,(G4-$B$3)/($B$4-$B$3))*$B$1</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>SUMIFS(AB:AB,AD:AD,"*"&amp;$B$10&amp;"*",AC:AC,C4)</f>
+        <v/>
+      </c>
+      <c r="L4">
+        <f>ROUND(MAX(0,MIN(100,100*(1-K4/IF(D4&gt;0,D4,SUMIFS(Consolidation!$M:$M,Consolidation!$A:$A,"*"&amp;$B$10&amp;"*")/30)))),2)</f>
+        <v/>
+      </c>
+      <c r="M4">
+        <f>MAX(0,(L4-$B$6)/($B$7-$B$6)*$B$8)</f>
+        <v/>
+      </c>
+      <c r="N4">
+        <f>$B$2+H4+M4</f>
+        <v/>
+      </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>1530</v>
+        <v>14077</v>
+      </c>
+      <c r="X4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
       </c>
       <c r="AB4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
@@ -3383,7 +4375,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -3392,10 +4384,23 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>2311</v>
+        <v>1530</v>
+      </c>
+      <c r="X5" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
       </c>
       <c r="AB5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
@@ -3424,16 +4429,29 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1815</v>
+        <v>2311</v>
+      </c>
+      <c r="X6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
       </c>
       <c r="AB6" t="n">
         <v>4</v>
@@ -3465,16 +4483,29 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>2868</v>
+      </c>
+      <c r="X7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
           <t>com.logistics.rider.talabat</t>
         </is>
-      </c>
-      <c r="V7" t="n">
-        <v>2333</v>
       </c>
       <c r="AB7" t="n">
         <v>14</v>
@@ -3511,11 +4542,24 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>2322</v>
+        <v>1815</v>
+      </c>
+      <c r="X8" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
       </c>
       <c r="AB8" t="n">
         <v>6</v>
@@ -3544,11 +4588,24 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>3533</v>
+        <v>2333</v>
+      </c>
+      <c r="X9" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
       </c>
       <c r="AB9" t="n">
         <v>5</v>
@@ -3582,16 +4639,29 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>1827</v>
+        <v>3182</v>
+      </c>
+      <c r="X10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
       </c>
       <c r="AB10" t="n">
         <v>2</v>
@@ -3615,16 +4685,29 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>2275</v>
+        <v>2322</v>
+      </c>
+      <c r="X11" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
       </c>
       <c r="AB11" t="n">
         <v>8</v>
@@ -3648,19 +4731,32 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>250</v>
+        <v>3533</v>
+      </c>
+      <c r="X12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
       </c>
       <c r="AB12" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -3681,16 +4777,29 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>com.logistics.rider.yemeksepeti</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>428</v>
+        <v>4891</v>
+      </c>
+      <c r="X13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
       </c>
       <c r="AB13" t="n">
         <v>3</v>
@@ -3719,14 +4828,27 @@
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>6249</v>
+        <v>1827</v>
+      </c>
+      <c r="X14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
       </c>
       <c r="AB14" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
@@ -3752,11 +4874,24 @@
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>8329</v>
+        <v>2275</v>
+      </c>
+      <c r="X15" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
       </c>
       <c r="AB15" t="n">
         <v>1</v>
@@ -3780,16 +4915,29 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>30</v>
+        <v>2882</v>
+      </c>
+      <c r="X16" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
       </c>
       <c r="AB16" t="n">
         <v>1</v>
@@ -3813,16 +4961,29 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>com.logistics.rider.woowabros</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>81</v>
+        <v>250</v>
+      </c>
+      <c r="X17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
       </c>
       <c r="AB17" t="n">
         <v>4</v>
@@ -3846,16 +5007,29 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>603</v>
+        <v>428</v>
+      </c>
+      <c r="X18" t="n">
+        <v>13</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
       </c>
       <c r="AB18" t="n">
         <v>57</v>
@@ -3879,16 +5053,29 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.yemeksepeti</t>
         </is>
       </c>
       <c r="V19" t="n">
-        <v>820</v>
+        <v>365</v>
+      </c>
+      <c r="X19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
       </c>
       <c r="AB19" t="n">
         <v>8</v>
@@ -3917,11 +5104,24 @@
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>90</v>
+        <v>6249</v>
+      </c>
+      <c r="X20" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
       </c>
       <c r="AB20" t="n">
         <v>2</v>
@@ -3950,11 +5150,24 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foody</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
       <c r="V21" t="n">
-        <v>119</v>
+        <v>8329</v>
+      </c>
+      <c r="X21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
       </c>
       <c r="AB21" t="n">
         <v>28</v>
@@ -3976,6 +5189,32 @@
           <t>2026-09-21</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>10619</v>
+      </c>
+      <c r="X22" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB22" t="n">
         <v>2</v>
       </c>
@@ -3996,6 +5235,32 @@
           <t>2026-09-22</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>30</v>
+      </c>
+      <c r="X23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB23" t="n">
         <v>4</v>
       </c>
@@ -4016,8 +5281,34 @@
           <t>2026-09-23</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>81</v>
+      </c>
+      <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
@@ -4036,8 +5327,34 @@
           <t>2026-09-24</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.woowabros</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>103</v>
+      </c>
+      <c r="X25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
       <c r="AB25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
@@ -4056,8 +5373,34 @@
           <t>2026-09-25</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>603</v>
+      </c>
+      <c r="X26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
       <c r="AB26" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AC26" t="inlineStr">
         <is>
@@ -4076,8 +5419,34 @@
           <t>2026-09-26</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>820</v>
+      </c>
+      <c r="X27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
       <c r="AB27" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
@@ -4096,8 +5465,21 @@
           <t>2026-09-27</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>1204</v>
+      </c>
       <c r="AB28" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AC28" t="inlineStr">
         <is>
@@ -4116,8 +5498,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>90</v>
+      </c>
       <c r="AB29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AC29" t="inlineStr">
         <is>
@@ -4136,6 +5531,19 @@
           <t>2026-09-29</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>119</v>
+      </c>
       <c r="AB30" t="n">
         <v>21</v>
       </c>
@@ -4156,6 +5564,19 @@
           <t>2026-09-30</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>157</v>
+      </c>
       <c r="AB31" t="n">
         <v>1</v>
       </c>
@@ -4207,7 +5628,7 @@
     </row>
     <row r="33">
       <c r="D33">
-        <f>AVERAGE(D2:D3)</f>
+        <f>AVERAGE(D2:D4)</f>
         <v/>
       </c>
       <c r="G33" s="37">
@@ -4215,7 +5636,7 @@
         <v/>
       </c>
       <c r="H33">
-        <f>AVERAGE(H2:H3)</f>
+        <f>AVERAGE(H2:H4)</f>
         <v/>
       </c>
       <c r="I33" s="38">
@@ -4233,6 +5654,259 @@
       <c r="N33" s="38">
         <f>$B$2+MAX(0,(G33-$B$3)/($B$4-$B$3)*($B$1-$B$8))+M33</f>
         <v/>
+      </c>
+      <c r="AB33" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="AB34" t="n">
+        <v>63</v>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodpanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="AB35" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="AB36" t="n">
+        <v>43</v>
+      </c>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="AB37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="AB38" t="n">
+        <v>3</v>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="AB39" t="n">
+        <v>5</v>
+      </c>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="AB40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="AB41" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="AB42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="AB43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="AB44" t="n">
+        <v>10</v>
+      </c>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="AB45" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="AB46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="AB47" t="n">
+        <v>47</v>
+      </c>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="AB48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.efood</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="AB49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foody</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>